<commit_message>
4807, 4908, 4909 - Update Excel Exports with new sheets
</commit_message>
<xml_diff>
--- a/GenBOE/GenBOE.Web/Templates/Export/WorkspaceDataMST.xlsx
+++ b/GenBOE/GenBOE.Web/Templates/Export/WorkspaceDataMST.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="20228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="22527"/>
   <workbookPr showPivotChartFilter="1" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ranzalon\Source\genBOE\dev\GenBOE\GenBOE.Web\Templates\Export\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ranzalon\Source\repos\IES\GenBOE\GenBOE.Web\Templates\Export\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8E97CBD-2C41-47CD-96FA-467136265FA5}" xr6:coauthVersionLast="34" xr6:coauthVersionMax="34" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58097765-AAC1-4376-A4D2-B691E2FF6DBD}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="12" windowWidth="19032" windowHeight="10752" firstSheet="5" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="25080" yWindow="-120" windowWidth="25440" windowHeight="15990" firstSheet="5" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="BOE3 Pivot" sheetId="19" state="hidden" r:id="rId1"/>
@@ -22,22 +22,27 @@
     <sheet name="BOEs" sheetId="16" r:id="rId7"/>
     <sheet name="BOE Status" sheetId="23" r:id="rId8"/>
     <sheet name="Resource Spreads" sheetId="41" r:id="rId9"/>
-    <sheet name="WBS" sheetId="24" r:id="rId10"/>
-    <sheet name="CLINs" sheetId="25" r:id="rId11"/>
-    <sheet name="User Permissions" sheetId="39" r:id="rId12"/>
-    <sheet name="Workspace Identification" sheetId="40" r:id="rId13"/>
-    <sheet name="Travel Unit Cost" sheetId="43" r:id="rId14"/>
-    <sheet name="Travel Extended Cost" sheetId="44" r:id="rId15"/>
+    <sheet name="MOQ by BOE by Task" sheetId="45" r:id="rId10"/>
+    <sheet name="MOQ Table Data" sheetId="46" r:id="rId11"/>
+    <sheet name="MOQ Summary" sheetId="47" r:id="rId12"/>
+    <sheet name="WBS" sheetId="24" r:id="rId13"/>
+    <sheet name="CLINs" sheetId="25" r:id="rId14"/>
+    <sheet name="User Permissions" sheetId="39" r:id="rId15"/>
+    <sheet name="Workspace Identification" sheetId="40" r:id="rId16"/>
+    <sheet name="Travel Unit Cost" sheetId="43" r:id="rId17"/>
+    <sheet name="Travel Extended Cost" sheetId="44" r:id="rId18"/>
   </sheets>
   <externalReferences>
-    <externalReference r:id="rId16"/>
-    <externalReference r:id="rId17"/>
+    <externalReference r:id="rId19"/>
+    <externalReference r:id="rId20"/>
   </externalReferences>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'BOE &amp; Resource Combo'!$A$1:$AP$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">BOEs!$A$1:$AQ$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'BOEs (2)'!$B$1:$T$16</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'BOEs (3)'!$A$1:$N$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'MOQ by BOE by Task'!$A$1:$G$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'MOQ Table Data'!$A$1:$Q$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Resource Spreads'!$A$1:$N$2</definedName>
     <definedName name="Approvers">'[1]Options Lists'!$D$2:$D$4</definedName>
     <definedName name="Authors">'[1]Options Lists'!$C$2:$C$4</definedName>
@@ -47,12 +52,22 @@
     <definedName name="SpreadCurve">[2]Lists!$C$2:$C$52</definedName>
     <definedName name="WBS">'[1]Options Lists'!$A$2:$A$8</definedName>
   </definedNames>
-  <calcPr calcId="125725"/>
+  <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="0" r:id="rId18"/>
-    <pivotCache cacheId="1" r:id="rId19"/>
-    <pivotCache cacheId="2" r:id="rId20"/>
+    <pivotCache cacheId="3" r:id="rId21"/>
+    <pivotCache cacheId="4" r:id="rId22"/>
+    <pivotCache cacheId="5" r:id="rId23"/>
   </pivotCaches>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -306,7 +321,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="852" uniqueCount="127">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="879" uniqueCount="142">
   <si>
     <t>Start Date</t>
   </si>
@@ -687,6 +702,51 @@
   </si>
   <si>
     <t xml:space="preserve"> </t>
+  </si>
+  <si>
+    <t>Total MOQ Hours</t>
+  </si>
+  <si>
+    <t>Table Name</t>
+  </si>
+  <si>
+    <t>Repository Name</t>
+  </si>
+  <si>
+    <t>Query Type (Weekly/Monthly)</t>
+  </si>
+  <si>
+    <t>Date of Report</t>
+  </si>
+  <si>
+    <t>Historical Program Name</t>
+  </si>
+  <si>
+    <t>Contract Number</t>
+  </si>
+  <si>
+    <t>WBS/WBS Element</t>
+  </si>
+  <si>
+    <t>Period of Performance (PoP): Start Date</t>
+  </si>
+  <si>
+    <t>Period of Performance (PoP): End Date</t>
+  </si>
+  <si>
+    <t>Total WBS/WBS Element Hours</t>
+  </si>
+  <si>
+    <t>Additional Query Filters (i.e. cost number, employee id)</t>
+  </si>
+  <si>
+    <t>Total Relevant Hours After Additional Query Filters Applied</t>
+  </si>
+  <si>
+    <t>MOQ Hours Bid/Spread</t>
+  </si>
+  <si>
+    <t>% of total</t>
   </si>
 </sst>
 </file>
@@ -699,7 +759,7 @@
     <numFmt numFmtId="166" formatCode="0.000"/>
     <numFmt numFmtId="167" formatCode="&quot;$&quot;#,##0.00"/>
   </numFmts>
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="14" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -772,8 +832,36 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFECF0F1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color rgb="FFECF0F1"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color rgb="FF452DB2"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -789,6 +877,36 @@
           <color theme="0" tint="-0.25098422193060094"/>
         </stop>
       </gradientFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF070729"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF9F9F9F"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF452DB2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD35714"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="6">
@@ -865,11 +983,17 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyNumberFormat="0" applyProtection="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="61">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -1030,9 +1154,15 @@
       <alignment horizontal="right"/>
     </xf>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="8">
     <cellStyle name="genBOE" xfId="1" xr:uid="{00000000-0005-0000-0000-000000000000}"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="PPDuplicateRow" xfId="5" xr:uid="{4174D75E-DF3C-4FB5-818B-80FEF28D3C31}"/>
+    <cellStyle name="PPHeaderColumn" xfId="3" xr:uid="{E41BCDE1-0C2A-4B7E-A982-545BCBA2200C}"/>
+    <cellStyle name="PPHeaderRequired" xfId="4" xr:uid="{4D34DCEF-AEC0-411E-90C4-13CE8F215C3F}"/>
+    <cellStyle name="PPHeaderTop" xfId="2" xr:uid="{CA1C622E-7369-4A25-9534-19ECF05668D0}"/>
+    <cellStyle name="PPInvalidValue" xfId="6" xr:uid="{ADD299A4-3361-487A-A034-817C29687CE2}"/>
+    <cellStyle name="PPMissingValue" xfId="7" xr:uid="{0E54516F-D159-48DC-839B-1F2ED1B552F4}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -4219,7 +4349,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0000-000000000000}" name="PivotTable7" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="3" minRefreshableVersion="3" showCalcMbrs="0" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="3" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0000-000000000000}" name="PivotTable7" cacheId="3" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="3" minRefreshableVersion="3" showCalcMbrs="0" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="3" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
   <location ref="A3:N33" firstHeaderRow="1" firstDataRow="1" firstDataCol="14"/>
   <pivotFields count="14">
     <pivotField axis="axisRow" compact="0" outline="0" showAll="0" insertBlankRow="1" defaultSubtotal="0">
@@ -4568,7 +4698,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0200-000000000000}" name="PivotTable9" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="3" minRefreshableVersion="3" showCalcMbrs="0" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="3" indent="0" compact="0" compactData="0" multipleFieldFilters="0" rowHeaderCaption="Type">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0200-000000000000}" name="PivotTable9" cacheId="4" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="3" minRefreshableVersion="3" showCalcMbrs="0" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="3" indent="0" compact="0" compactData="0" multipleFieldFilters="0" rowHeaderCaption="Type">
   <location ref="A3:H11" firstHeaderRow="1" firstDataRow="1" firstDataCol="8"/>
   <pivotFields count="19">
     <pivotField axis="axisRow" compact="0" outline="0" showAll="0" defaultSubtotal="0">
@@ -4777,7 +4907,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0300-000000000000}" name="PivotTable4" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" missingCaption="_" updatedVersion="3" minRefreshableVersion="3" showCalcMbrs="0" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="3" indent="0" compact="0" compactData="0" multipleFieldFilters="0" rowHeaderCaption="BOE ID">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0300-000000000000}" name="PivotTable4" cacheId="5" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" missingCaption="_" updatedVersion="3" minRefreshableVersion="3" showCalcMbrs="0" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="3" indent="0" compact="0" compactData="0" multipleFieldFilters="0" rowHeaderCaption="BOE ID">
   <location ref="A3:T33" firstHeaderRow="1" firstDataRow="1" firstDataCol="20"/>
   <pivotFields count="20">
     <pivotField axis="axisRow" compact="0" outline="0" showAll="0" insertBlankRow="1" defaultSubtotal="0">
@@ -5541,25 +5671,25 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A3:N32"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="22.5546875" customWidth="1"/>
-    <col min="2" max="2" width="11.44140625" customWidth="1"/>
-    <col min="3" max="3" width="10.5546875" customWidth="1"/>
+    <col min="1" max="1" width="22.5703125" customWidth="1"/>
+    <col min="2" max="2" width="11.42578125" customWidth="1"/>
+    <col min="3" max="3" width="10.5703125" customWidth="1"/>
     <col min="4" max="4" width="15" customWidth="1"/>
-    <col min="5" max="5" width="11.6640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.88671875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13.109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.44140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.42578125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="17" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="12" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="11.109375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="11.140625" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="15" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="11.44140625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="11.42578125" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="15" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
         <v>33</v>
       </c>
@@ -5603,7 +5733,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>59</v>
       </c>
@@ -5647,7 +5777,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
       <c r="G6" t="s">
         <v>57</v>
       </c>
@@ -5673,7 +5803,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
       <c r="H8" t="s">
         <v>43</v>
       </c>
@@ -5696,7 +5826,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
       <c r="D10" t="s">
         <v>62</v>
       </c>
@@ -5731,7 +5861,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
       <c r="G12" t="s">
         <v>57</v>
       </c>
@@ -5757,7 +5887,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:14" x14ac:dyDescent="0.25">
       <c r="H14" t="s">
         <v>43</v>
       </c>
@@ -5780,7 +5910,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:14" x14ac:dyDescent="0.25">
       <c r="D16" t="s">
         <v>57</v>
       </c>
@@ -5815,7 +5945,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="18" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>60</v>
       </c>
@@ -5859,7 +5989,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="20" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:14" x14ac:dyDescent="0.25">
       <c r="G20" t="s">
         <v>57</v>
       </c>
@@ -5885,7 +6015,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="22" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:14" x14ac:dyDescent="0.25">
       <c r="H22" t="s">
         <v>43</v>
       </c>
@@ -5908,7 +6038,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="24" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:14" x14ac:dyDescent="0.25">
       <c r="H24" t="s">
         <v>55</v>
       </c>
@@ -5931,7 +6061,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="26" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:14" x14ac:dyDescent="0.25">
       <c r="H26" t="s">
         <v>51</v>
       </c>
@@ -5954,7 +6084,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="28" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:14" x14ac:dyDescent="0.25">
       <c r="D28" t="s">
         <v>64</v>
       </c>
@@ -5989,7 +6119,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="30" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:14" x14ac:dyDescent="0.25">
       <c r="G30" t="s">
         <v>57</v>
       </c>
@@ -6015,7 +6145,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="32" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:14" x14ac:dyDescent="0.25">
       <c r="D32" t="s">
         <v>62</v>
       </c>
@@ -6057,17 +6187,171 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3DA6D2FB-3F32-46E9-963C-DCD2D761F967}">
+  <dimension ref="A1:G2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="11.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="24" customWidth="1"/>
+    <col min="6" max="6" width="21.140625" customWidth="1"/>
+    <col min="7" max="7" width="40.85546875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>115</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="5" t="s">
+        <v>119</v>
+      </c>
+      <c r="F1" s="5" t="s">
+        <v>127</v>
+      </c>
+      <c r="G1" s="5" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
+  </sheetData>
+  <autoFilter ref="A1:G1" xr:uid="{1E7471F8-87B8-4A9F-A5C2-80CE50F530C1}"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EDDB750B-2EAA-4C67-B526-87C6863613C3}">
+  <dimension ref="A1:Q2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="11.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="24" customWidth="1"/>
+    <col min="5" max="5" width="42.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.85546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="21.28515625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="33.7109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="18.85546875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="28.85546875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="23" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="42" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="41.140625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="35.28515625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="57.85546875" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="61.42578125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:17" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>115</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="F1" s="5" t="s">
+        <v>128</v>
+      </c>
+      <c r="G1" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="H1" s="5" t="s">
+        <v>130</v>
+      </c>
+      <c r="I1" s="5" t="s">
+        <v>131</v>
+      </c>
+      <c r="J1" s="5" t="s">
+        <v>132</v>
+      </c>
+      <c r="K1" s="5" t="s">
+        <v>133</v>
+      </c>
+      <c r="L1" s="5" t="s">
+        <v>134</v>
+      </c>
+      <c r="M1" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="N1" s="5" t="s">
+        <v>136</v>
+      </c>
+      <c r="O1" s="5" t="s">
+        <v>137</v>
+      </c>
+      <c r="P1" s="5" t="s">
+        <v>138</v>
+      </c>
+      <c r="Q1" s="5" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="2" spans="1:17" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
+  </sheetData>
+  <autoFilter ref="A1:Q1" xr:uid="{24A73A91-4C44-47FC-8450-35CF267C3337}"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C5C2B818-1ECD-43FE-AA03-6B27248B8CDB}">
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="40.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="24.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>140</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
   <dimension ref="A1:E2"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="13.8" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="30.6640625" style="6" hidden="1" customWidth="1"/>
-    <col min="2" max="4" width="30.6640625" style="8" customWidth="1"/>
-    <col min="5" max="5" width="33.109375" style="7" customWidth="1"/>
-    <col min="6" max="16384" width="9.109375" style="7"/>
+    <col min="1" max="1" width="30.7109375" style="6" hidden="1" customWidth="1"/>
+    <col min="2" max="4" width="30.7109375" style="8" customWidth="1"/>
+    <col min="5" max="5" width="33.140625" style="7" customWidth="1"/>
+    <col min="6" max="16384" width="9.140625" style="7"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="5" customFormat="1" ht="20.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" s="5" customFormat="1" ht="20.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
         <v>68</v>
       </c>
@@ -6084,7 +6368,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="14.4" thickTop="1" x14ac:dyDescent="0.3"/>
+    <row r="2" spans="1:5" ht="13.5" thickTop="1" x14ac:dyDescent="0.2"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -6092,19 +6376,19 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
   <dimension ref="A1:E2"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="13.8" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="13.109375" style="6" hidden="1" customWidth="1"/>
-    <col min="2" max="2" width="30.6640625" style="8" customWidth="1"/>
-    <col min="3" max="3" width="50.6640625" style="8" customWidth="1"/>
-    <col min="4" max="5" width="20.6640625" style="8" customWidth="1"/>
-    <col min="6" max="16384" width="9.109375" style="7"/>
+    <col min="1" max="1" width="13.140625" style="6" hidden="1" customWidth="1"/>
+    <col min="2" max="2" width="30.7109375" style="8" customWidth="1"/>
+    <col min="3" max="3" width="50.7109375" style="8" customWidth="1"/>
+    <col min="4" max="5" width="20.7109375" style="8" customWidth="1"/>
+    <col min="6" max="16384" width="9.140625" style="7"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="5" customFormat="1" ht="20.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" s="5" customFormat="1" ht="20.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
         <v>98</v>
       </c>
@@ -6121,7 +6405,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="14.4" thickTop="1" x14ac:dyDescent="0.3"/>
+    <row r="2" spans="1:5" ht="13.5" thickTop="1" x14ac:dyDescent="0.2"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -6129,23 +6413,23 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0B00-000000000000}">
   <dimension ref="A1:I2"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="18.88671875" style="15" customWidth="1"/>
-    <col min="2" max="3" width="35.6640625" style="15" customWidth="1"/>
-    <col min="4" max="4" width="26.109375" style="15" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.5546875" style="15" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="22.109375" style="15" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="10.88671875" style="15" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="13.109375" style="15" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="21.88671875" style="15" bestFit="1" customWidth="1"/>
-    <col min="10" max="16384" width="9.109375" style="15"/>
+    <col min="1" max="1" width="18.85546875" style="15" customWidth="1"/>
+    <col min="2" max="3" width="35.7109375" style="15" customWidth="1"/>
+    <col min="4" max="4" width="26.140625" style="15" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.5703125" style="15" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="22.140625" style="15" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.85546875" style="15" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.140625" style="15" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="21.85546875" style="15" bestFit="1" customWidth="1"/>
+    <col min="10" max="16384" width="9.140625" style="15"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" s="14" customFormat="1" ht="16.8" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:9" s="14" customFormat="1" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>71</v>
       </c>
@@ -6174,91 +6458,91 @@
         <v>125</v>
       </c>
     </row>
-    <row r="2" spans="1:9" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
+    <row r="2" spans="1:9" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0C00-000000000000}">
   <dimension ref="A1:A16"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="28" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="82.109375" style="1" customWidth="1"/>
-    <col min="3" max="16384" width="9.109375" style="1"/>
+    <col min="2" max="2" width="82.140625" style="1" customWidth="1"/>
+    <col min="3" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" hidden="1" x14ac:dyDescent="0.3"/>
-    <row r="2" spans="1:1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:1" hidden="1" x14ac:dyDescent="0.25"/>
+    <row r="2" spans="1:1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="10" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="3" spans="1:1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="10" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="4" spans="1:1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="10" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="5" spans="1:1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="10"/>
     </row>
-    <row r="6" spans="1:1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="7" spans="1:1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="10" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="8" spans="1:1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="11" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="9" spans="1:1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="11" t="s">
         <v>122</v>
       </c>
     </row>
-    <row r="10" spans="1:1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="11" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="11" spans="1:1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="12" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="12" spans="1:1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="12" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="13" spans="1:1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="10" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="14" spans="1:1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="19" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="15" spans="1:1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="20"/>
     </row>
-    <row r="16" spans="1:1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="20"/>
     </row>
   </sheetData>
@@ -6267,33 +6551,33 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1E9E49D2-B4A1-426D-8F6A-B85DD2E6A5AA}">
   <dimension ref="A1:AA7"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
-    <col min="2" max="2" width="7.109375" customWidth="1"/>
-    <col min="3" max="3" width="29.44140625" customWidth="1"/>
-    <col min="4" max="4" width="26.88671875" customWidth="1"/>
-    <col min="5" max="5" width="12.33203125" customWidth="1"/>
+    <col min="2" max="2" width="7.140625" customWidth="1"/>
+    <col min="3" max="3" width="29.42578125" customWidth="1"/>
+    <col min="4" max="4" width="26.85546875" customWidth="1"/>
+    <col min="5" max="5" width="12.28515625" customWidth="1"/>
     <col min="6" max="6" width="16" customWidth="1"/>
-    <col min="7" max="7" width="20.5546875" customWidth="1"/>
-    <col min="8" max="8" width="10.5546875" style="40" customWidth="1"/>
-    <col min="9" max="11" width="8.88671875" style="40"/>
-    <col min="12" max="12" width="12.88671875" style="40" customWidth="1"/>
-    <col min="13" max="13" width="8.88671875" style="40"/>
-    <col min="14" max="14" width="15.5546875" style="57" customWidth="1"/>
-    <col min="15" max="15" width="19.109375" style="57" customWidth="1"/>
-    <col min="16" max="16" width="15.6640625" style="57" customWidth="1"/>
-    <col min="17" max="17" width="19.33203125" style="57" customWidth="1"/>
-    <col min="18" max="18" width="13.6640625" style="57" customWidth="1"/>
-    <col min="19" max="19" width="17.88671875" style="57" customWidth="1"/>
-    <col min="20" max="20" width="17.6640625" customWidth="1"/>
-    <col min="21" max="21" width="15.33203125" customWidth="1"/>
+    <col min="7" max="7" width="20.5703125" customWidth="1"/>
+    <col min="8" max="8" width="10.5703125" style="40" customWidth="1"/>
+    <col min="9" max="11" width="8.85546875" style="40"/>
+    <col min="12" max="12" width="12.85546875" style="40" customWidth="1"/>
+    <col min="13" max="13" width="8.85546875" style="40"/>
+    <col min="14" max="14" width="15.5703125" style="57" customWidth="1"/>
+    <col min="15" max="15" width="19.140625" style="57" customWidth="1"/>
+    <col min="16" max="16" width="15.7109375" style="57" customWidth="1"/>
+    <col min="17" max="17" width="19.28515625" style="57" customWidth="1"/>
+    <col min="18" max="18" width="13.7109375" style="57" customWidth="1"/>
+    <col min="19" max="19" width="17.85546875" style="57" customWidth="1"/>
+    <col min="20" max="20" width="17.7109375" customWidth="1"/>
+    <col min="21" max="21" width="15.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:27" s="45" customFormat="1" ht="19.2" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:27" s="45" customFormat="1" ht="20.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="41"/>
       <c r="B1" s="42"/>
       <c r="C1" s="42"/>
@@ -6321,7 +6605,7 @@
       <c r="Z1" s="54"/>
       <c r="AA1" s="54"/>
     </row>
-    <row r="2" spans="1:27" s="45" customFormat="1" ht="18.600000000000001" thickTop="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:27" s="45" customFormat="1" ht="19.5" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A2" s="41"/>
       <c r="B2" s="42"/>
       <c r="C2" s="42"/>
@@ -6350,7 +6634,7 @@
       <c r="Z2" s="54"/>
       <c r="AA2" s="54"/>
     </row>
-    <row r="3" spans="1:27" s="45" customFormat="1" ht="18" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:27" s="45" customFormat="1" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A3" s="41"/>
       <c r="B3" s="42"/>
       <c r="C3" s="42"/>
@@ -6379,7 +6663,7 @@
       <c r="Z3" s="54"/>
       <c r="AA3" s="54"/>
     </row>
-    <row r="4" spans="1:27" s="45" customFormat="1" ht="18" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:27" s="45" customFormat="1" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A4" s="41"/>
       <c r="B4" s="42"/>
       <c r="C4" s="42"/>
@@ -6408,7 +6692,7 @@
       <c r="Z4" s="54"/>
       <c r="AA4" s="54"/>
     </row>
-    <row r="5" spans="1:27" s="45" customFormat="1" ht="18" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:27" s="45" customFormat="1" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A5" s="55"/>
       <c r="B5" s="42"/>
       <c r="C5" s="42"/>
@@ -6437,7 +6721,7 @@
       <c r="Z5" s="54"/>
       <c r="AA5" s="54"/>
     </row>
-    <row r="6" spans="1:27" s="45" customFormat="1" ht="18" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:27" s="45" customFormat="1" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A6" s="55"/>
       <c r="B6" s="56"/>
       <c r="C6" s="56"/>
@@ -6466,7 +6750,7 @@
       <c r="Z6" s="54"/>
       <c r="AA6" s="54"/>
     </row>
-    <row r="7" spans="1:27" s="55" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:27" s="55" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="H7" s="43"/>
       <c r="I7" s="43"/>
       <c r="J7" s="43"/>
@@ -6488,32 +6772,32 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00BB237A-2FF2-450F-81EE-9A098F6C7133}">
   <dimension ref="A1:AA6"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.6640625" style="58" customWidth="1"/>
-    <col min="2" max="2" width="7.109375" style="58" customWidth="1"/>
-    <col min="3" max="3" width="29.44140625" style="58" customWidth="1"/>
-    <col min="4" max="4" width="26.88671875" style="58" customWidth="1"/>
-    <col min="5" max="5" width="12.33203125" style="58" customWidth="1"/>
+    <col min="1" max="1" width="11.7109375" style="58" customWidth="1"/>
+    <col min="2" max="2" width="7.140625" style="58" customWidth="1"/>
+    <col min="3" max="3" width="29.42578125" style="58" customWidth="1"/>
+    <col min="4" max="4" width="26.85546875" style="58" customWidth="1"/>
+    <col min="5" max="5" width="12.28515625" style="58" customWidth="1"/>
     <col min="6" max="6" width="16" style="58" customWidth="1"/>
-    <col min="7" max="7" width="20.5546875" style="58" customWidth="1"/>
-    <col min="8" max="8" width="10.5546875" style="59" customWidth="1"/>
-    <col min="9" max="13" width="9.109375" style="59"/>
-    <col min="14" max="14" width="15.5546875" style="57" customWidth="1"/>
-    <col min="15" max="15" width="24.5546875" style="57" customWidth="1"/>
-    <col min="16" max="16" width="15.6640625" style="57" customWidth="1"/>
-    <col min="17" max="17" width="19.33203125" style="57" customWidth="1"/>
-    <col min="18" max="18" width="13.6640625" style="57" customWidth="1"/>
-    <col min="19" max="19" width="17.88671875" style="57" customWidth="1"/>
-    <col min="20" max="20" width="17.6640625" style="57" customWidth="1"/>
-    <col min="21" max="21" width="15.33203125" style="57" customWidth="1"/>
-    <col min="22" max="16384" width="9.109375" style="60"/>
+    <col min="7" max="7" width="20.5703125" style="58" customWidth="1"/>
+    <col min="8" max="8" width="10.5703125" style="59" customWidth="1"/>
+    <col min="9" max="13" width="9.140625" style="59"/>
+    <col min="14" max="14" width="15.5703125" style="57" customWidth="1"/>
+    <col min="15" max="15" width="24.5703125" style="57" customWidth="1"/>
+    <col min="16" max="16" width="15.7109375" style="57" customWidth="1"/>
+    <col min="17" max="17" width="19.28515625" style="57" customWidth="1"/>
+    <col min="18" max="18" width="13.7109375" style="57" customWidth="1"/>
+    <col min="19" max="19" width="17.85546875" style="57" customWidth="1"/>
+    <col min="20" max="20" width="17.7109375" style="57" customWidth="1"/>
+    <col min="21" max="21" width="15.28515625" style="57" customWidth="1"/>
+    <col min="22" max="16384" width="9.140625" style="60"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:27" s="52" customFormat="1" ht="19.2" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:27" s="52" customFormat="1" ht="20.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="42"/>
       <c r="B1" s="42"/>
       <c r="C1" s="42"/>
@@ -6542,7 +6826,7 @@
       <c r="Z1" s="51"/>
       <c r="AA1" s="51"/>
     </row>
-    <row r="2" spans="1:27" s="52" customFormat="1" ht="18.600000000000001" thickTop="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:27" s="52" customFormat="1" ht="19.5" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A2" s="42"/>
       <c r="B2" s="42"/>
       <c r="C2" s="42"/>
@@ -6571,7 +6855,7 @@
       <c r="Z2" s="51"/>
       <c r="AA2" s="51"/>
     </row>
-    <row r="3" spans="1:27" s="52" customFormat="1" ht="18" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:27" s="52" customFormat="1" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A3" s="42"/>
       <c r="B3" s="42"/>
       <c r="C3" s="42"/>
@@ -6600,7 +6884,7 @@
       <c r="Z3" s="51"/>
       <c r="AA3" s="51"/>
     </row>
-    <row r="4" spans="1:27" s="52" customFormat="1" ht="18" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:27" s="52" customFormat="1" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A4" s="42"/>
       <c r="B4" s="42"/>
       <c r="C4" s="42"/>
@@ -6629,7 +6913,7 @@
       <c r="Z4" s="51"/>
       <c r="AA4" s="51"/>
     </row>
-    <row r="5" spans="1:27" s="52" customFormat="1" ht="18" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:27" s="52" customFormat="1" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A5" s="42"/>
       <c r="B5" s="42"/>
       <c r="C5" s="42"/>
@@ -6658,7 +6942,7 @@
       <c r="Z5" s="51"/>
       <c r="AA5" s="51"/>
     </row>
-    <row r="6" spans="1:27" s="45" customFormat="1" ht="18" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:27" s="45" customFormat="1" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A6" s="56"/>
       <c r="B6" s="56"/>
       <c r="C6" s="56"/>
@@ -6695,28 +6979,28 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:N16"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="16.88671875" style="3" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.44140625" style="3" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.5546875" style="3" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.44140625" style="3" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.6640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.88671875" style="3" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="15.44140625" style="3" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="13.109375" style="3" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="18.88671875" style="3" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="13.88671875" style="3" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.85546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.42578125" style="3" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.5703125" style="3" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.42578125" style="3" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.7109375" style="3" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.85546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.42578125" style="3" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.140625" style="3" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="18.85546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="13.85546875" style="3" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="13" style="3" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="16.88671875" style="3" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="16.85546875" style="3" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="13" style="3" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="17" style="3" bestFit="1" customWidth="1"/>
-    <col min="15" max="17" width="13.5546875" style="3" customWidth="1"/>
-    <col min="18" max="18" width="15.44140625" style="3" bestFit="1" customWidth="1"/>
-    <col min="19" max="16384" width="9.109375" style="3"/>
+    <col min="15" max="17" width="13.5703125" style="3" customWidth="1"/>
+    <col min="18" max="18" width="15.42578125" style="3" bestFit="1" customWidth="1"/>
+    <col min="19" max="16384" width="9.140625" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="16.8" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:14" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>33</v>
       </c>
@@ -6760,7 +7044,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="2" spans="1:14" ht="15" thickTop="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:14" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>59</v>
       </c>
@@ -6771,7 +7055,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>59</v>
       </c>
@@ -6794,7 +7078,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>59</v>
       </c>
@@ -6835,7 +7119,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
         <v>59</v>
       </c>
@@ -6876,7 +7160,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
         <v>59</v>
       </c>
@@ -6899,7 +7183,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
         <v>59</v>
       </c>
@@ -6940,7 +7224,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
         <v>59</v>
       </c>
@@ -6981,7 +7265,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
         <v>60</v>
       </c>
@@ -7001,7 +7285,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>60</v>
       </c>
@@ -7024,7 +7308,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
         <v>60</v>
       </c>
@@ -7065,7 +7349,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>60</v>
       </c>
@@ -7106,7 +7390,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
         <v>60</v>
       </c>
@@ -7147,7 +7431,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
         <v>60</v>
       </c>
@@ -7188,7 +7472,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
         <v>60</v>
       </c>
@@ -7211,7 +7495,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
         <v>60</v>
       </c>
@@ -7262,20 +7546,20 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A3:H11"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="7.5546875" customWidth="1"/>
-    <col min="2" max="2" width="8.88671875" customWidth="1"/>
-    <col min="3" max="3" width="11.88671875" customWidth="1"/>
-    <col min="4" max="4" width="8.6640625" customWidth="1"/>
-    <col min="5" max="5" width="11.6640625" customWidth="1"/>
-    <col min="6" max="6" width="11.44140625" customWidth="1"/>
-    <col min="7" max="7" width="10.5546875" customWidth="1"/>
-    <col min="8" max="8" width="9.44140625" customWidth="1"/>
+    <col min="1" max="1" width="7.5703125" customWidth="1"/>
+    <col min="2" max="2" width="8.85546875" customWidth="1"/>
+    <col min="3" max="3" width="11.85546875" customWidth="1"/>
+    <col min="4" max="4" width="8.7109375" customWidth="1"/>
+    <col min="5" max="5" width="11.7109375" customWidth="1"/>
+    <col min="6" max="6" width="11.42578125" customWidth="1"/>
+    <col min="7" max="7" width="10.5703125" customWidth="1"/>
+    <col min="8" max="8" width="9.42578125" customWidth="1"/>
     <col min="9" max="19" width="15" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
         <v>26</v>
       </c>
@@ -7301,7 +7585,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>33</v>
       </c>
@@ -7327,7 +7611,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
         <v>45</v>
       </c>
@@ -7335,7 +7619,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>12</v>
       </c>
@@ -7361,12 +7645,12 @@
         <v>38</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="H7" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B8" t="s">
         <v>45</v>
       </c>
@@ -7374,7 +7658,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>34</v>
       </c>
@@ -7400,12 +7684,12 @@
         <v>38</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="H10" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B11" t="s">
         <v>45</v>
       </c>
@@ -7422,29 +7706,29 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A3:T32"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="22.44140625" customWidth="1"/>
-    <col min="2" max="2" width="12.44140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.88671875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.6640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.44140625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.5546875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="9.44140625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.5546875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="11.6640625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="10.88671875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.109375" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="11.44140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="22.42578125" customWidth="1"/>
+    <col min="2" max="2" width="12.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="13.140625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="11.42578125" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="17" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="12" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.109375" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.140625" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="15" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="11.44140625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="11.42578125" bestFit="1" customWidth="1"/>
     <col min="20" max="20" width="15" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
         <v>70</v>
       </c>
@@ -7506,7 +7790,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="4" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>58</v>
       </c>
@@ -7568,7 +7852,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="6" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:20" x14ac:dyDescent="0.25">
       <c r="B6" t="s">
         <v>34</v>
       </c>
@@ -7627,7 +7911,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="8" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:20" x14ac:dyDescent="0.25">
       <c r="I8" t="s">
         <v>40</v>
       </c>
@@ -7665,7 +7949,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="10" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:20" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
         <v>12</v>
       </c>
@@ -7724,7 +8008,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="12" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:20" x14ac:dyDescent="0.25">
       <c r="R12" t="s">
         <v>20</v>
       </c>
@@ -7735,7 +8019,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="14" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:20" x14ac:dyDescent="0.25">
       <c r="N14" t="s">
         <v>43</v>
       </c>
@@ -7758,7 +8042,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="16" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:20" x14ac:dyDescent="0.25">
       <c r="O16" t="s">
         <v>53</v>
       </c>
@@ -7778,7 +8062,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="18" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>45</v>
       </c>
@@ -7840,7 +8124,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="20" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:20" x14ac:dyDescent="0.25">
       <c r="B20" t="s">
         <v>34</v>
       </c>
@@ -7899,7 +8183,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="22" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:20" x14ac:dyDescent="0.25">
       <c r="I22" t="s">
         <v>49</v>
       </c>
@@ -7937,7 +8221,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="24" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:20" x14ac:dyDescent="0.25">
       <c r="B24" t="s">
         <v>12</v>
       </c>
@@ -7996,7 +8280,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="26" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:20" x14ac:dyDescent="0.25">
       <c r="O26" t="s">
         <v>52</v>
       </c>
@@ -8016,7 +8300,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="28" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:20" x14ac:dyDescent="0.25">
       <c r="N28" t="s">
         <v>43</v>
       </c>
@@ -8039,7 +8323,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="30" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:20" x14ac:dyDescent="0.25">
       <c r="N30" t="s">
         <v>55</v>
       </c>
@@ -8062,7 +8346,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="32" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:20" x14ac:dyDescent="0.25">
       <c r="N32" t="s">
         <v>51</v>
       </c>
@@ -8094,33 +8378,33 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:T16"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.109375" style="3"/>
-    <col min="2" max="3" width="10.5546875" style="3" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.5546875" style="3" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.5546875" style="3" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.5546875" style="3" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13.44140625" style="3" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="12.5546875" style="3" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="11.44140625" style="3" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="13.5546875" style="3" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="13.6640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="12.88671875" style="3" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="15.44140625" style="3" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="13.109375" style="3" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="18.88671875" style="3" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="13.88671875" style="3" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.140625" style="3"/>
+    <col min="2" max="3" width="10.5703125" style="3" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.5703125" style="3" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.5703125" style="3" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.5703125" style="3" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.42578125" style="3" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12.5703125" style="3" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="11.42578125" style="3" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="13.5703125" style="3" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="13.7109375" style="3" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="12.85546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="15.42578125" style="3" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="13.140625" style="3" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="18.85546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="13.85546875" style="3" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="13" style="3" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="16.88671875" style="3" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="16.85546875" style="3" bestFit="1" customWidth="1"/>
     <col min="19" max="19" width="13" style="3" bestFit="1" customWidth="1"/>
     <col min="20" max="20" width="17" style="3" bestFit="1" customWidth="1"/>
-    <col min="21" max="23" width="13.5546875" style="3" customWidth="1"/>
-    <col min="24" max="24" width="15.44140625" style="3" bestFit="1" customWidth="1"/>
-    <col min="25" max="16384" width="9.109375" style="3"/>
+    <col min="21" max="23" width="13.5703125" style="3" customWidth="1"/>
+    <col min="24" max="24" width="15.42578125" style="3" bestFit="1" customWidth="1"/>
+    <col min="25" max="16384" width="9.140625" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" ht="16.8" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:20" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>70</v>
       </c>
@@ -8182,7 +8466,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="2" spans="1:20" ht="15" thickTop="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:20" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>58</v>
       </c>
@@ -8208,7 +8492,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="3" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>58</v>
       </c>
@@ -8231,7 +8515,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="4" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>58</v>
       </c>
@@ -8260,7 +8544,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="5" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
         <v>58</v>
       </c>
@@ -8289,7 +8573,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="6" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
         <v>58</v>
       </c>
@@ -8312,7 +8596,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="7" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
         <v>58</v>
       </c>
@@ -8341,7 +8625,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="8" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
         <v>58</v>
       </c>
@@ -8370,7 +8654,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="9" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
         <v>45</v>
       </c>
@@ -8396,7 +8680,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="10" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>45</v>
       </c>
@@ -8419,7 +8703,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="11" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
         <v>45</v>
       </c>
@@ -8448,7 +8732,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="12" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>45</v>
       </c>
@@ -8477,7 +8761,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="13" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
         <v>45</v>
       </c>
@@ -8506,7 +8790,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="14" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
         <v>45</v>
       </c>
@@ -8535,7 +8819,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="15" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
         <v>45</v>
       </c>
@@ -8558,7 +8842,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="16" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
         <v>45</v>
       </c>
@@ -8597,54 +8881,54 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:AP2"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.88671875" style="1" customWidth="1"/>
-    <col min="3" max="3" width="11.44140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.5546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="18.44140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="14.5546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="19.109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="19.88671875" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="10.5546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="13.5546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="19.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="10.5546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.5546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="13.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="13.44140625" style="38" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="12.5546875" style="38" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="21.44140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="20.109375" style="33" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="18.6640625" style="31" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="20.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="21.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="13.6640625" style="38" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="12.88671875" style="38" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="21.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="20.44140625" style="33" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.85546875" style="1" customWidth="1"/>
+    <col min="3" max="3" width="11.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="18.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="19.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="19.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="10.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="13.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="19.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="10.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="13.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="13.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="13.42578125" style="38" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="12.5703125" style="38" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="21.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="20.140625" style="33" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="18.7109375" style="31" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="17.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="20.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="21.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="13.7109375" style="38" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="12.85546875" style="38" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="21.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="20.42578125" style="33" bestFit="1" customWidth="1"/>
     <col min="27" max="27" width="19" style="31" bestFit="1" customWidth="1"/>
     <col min="28" max="28" width="20" style="1" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="24.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="18.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="18.5546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="18.88671875" style="1" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="23.88671875" style="1" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="16.88671875" style="1" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="24.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="18.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="18.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="18.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="23.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="16.85546875" style="1" bestFit="1" customWidth="1"/>
     <col min="35" max="35" width="13" style="35" bestFit="1" customWidth="1"/>
     <col min="36" max="36" width="17" style="33" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="15.6640625" style="31" bestFit="1" customWidth="1"/>
-    <col min="38" max="38" width="26.109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="39" max="39" width="8.6640625" style="40" customWidth="1"/>
-    <col min="40" max="40" width="10.5546875" style="40" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="15.7109375" style="31" bestFit="1" customWidth="1"/>
+    <col min="38" max="38" width="26.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="39" max="39" width="8.7109375" style="40" customWidth="1"/>
+    <col min="40" max="40" width="10.5703125" style="40" bestFit="1" customWidth="1"/>
     <col min="41" max="41" width="10" style="33" bestFit="1" customWidth="1"/>
-    <col min="42" max="42" width="8.6640625" style="31" customWidth="1"/>
-    <col min="43" max="16384" width="9.109375" style="1"/>
+    <col min="42" max="42" width="8.7109375" style="31" customWidth="1"/>
+    <col min="43" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:42" s="5" customFormat="1" ht="16.8" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:42" s="5" customFormat="1" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
         <v>70</v>
       </c>
@@ -8772,7 +9056,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="2" spans="1:42" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
+    <row r="2" spans="1:42" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <autoFilter ref="A1:AP1" xr:uid="{00000000-0009-0000-0000-000005000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -8783,48 +9067,48 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:AQ2"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.44140625" style="3" customWidth="1"/>
-    <col min="2" max="3" width="10.5546875" style="3" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.5546875" style="3" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.109375" style="3" customWidth="1"/>
-    <col min="6" max="6" width="10.5546875" style="3" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13.5546875" style="3" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="13.44140625" style="3" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="12.5546875" style="3" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="21.44140625" style="3" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="20.109375" style="22" bestFit="1" customWidth="1"/>
-    <col min="12" max="13" width="20.109375" style="27" customWidth="1"/>
-    <col min="14" max="14" width="20.109375" style="3" customWidth="1"/>
-    <col min="15" max="15" width="11.44140625" style="3" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="13.5546875" style="3" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="20.109375" style="3" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="18.44140625" style="3" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="23.88671875" style="3" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.42578125" style="3" customWidth="1"/>
+    <col min="2" max="3" width="10.5703125" style="3" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.5703125" style="3" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.140625" style="3" customWidth="1"/>
+    <col min="6" max="6" width="10.5703125" style="3" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.5703125" style="3" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.42578125" style="3" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12.5703125" style="3" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="21.42578125" style="3" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="20.140625" style="22" bestFit="1" customWidth="1"/>
+    <col min="12" max="13" width="20.140625" style="27" customWidth="1"/>
+    <col min="14" max="14" width="20.140625" style="3" customWidth="1"/>
+    <col min="15" max="15" width="11.42578125" style="3" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="13.5703125" style="3" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="20.140625" style="3" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="18.42578125" style="3" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="23.85546875" style="3" bestFit="1" customWidth="1"/>
     <col min="20" max="20" width="19" style="3" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="21.109375" style="3" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="13.6640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="12.88671875" style="3" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="21.6640625" style="3" customWidth="1"/>
-    <col min="25" max="25" width="20.44140625" style="22" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="20.44140625" style="27" customWidth="1"/>
-    <col min="27" max="27" width="20.44140625" style="3" customWidth="1"/>
-    <col min="28" max="28" width="24.6640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="29" max="31" width="24.6640625" style="3" customWidth="1"/>
-    <col min="32" max="32" width="18.88671875" style="3" bestFit="1" customWidth="1"/>
-    <col min="33" max="36" width="18.88671875" style="3" customWidth="1"/>
-    <col min="37" max="37" width="13.88671875" style="3" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="21.140625" style="3" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="13.7109375" style="3" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="12.85546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="21.7109375" style="3" customWidth="1"/>
+    <col min="25" max="25" width="20.42578125" style="22" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="20.42578125" style="27" customWidth="1"/>
+    <col min="27" max="27" width="20.42578125" style="3" customWidth="1"/>
+    <col min="28" max="28" width="24.7109375" style="3" bestFit="1" customWidth="1"/>
+    <col min="29" max="31" width="24.7109375" style="3" customWidth="1"/>
+    <col min="32" max="32" width="18.85546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="33" max="36" width="18.85546875" style="3" customWidth="1"/>
+    <col min="37" max="37" width="13.85546875" style="3" bestFit="1" customWidth="1"/>
     <col min="38" max="38" width="13" style="3" bestFit="1" customWidth="1"/>
-    <col min="39" max="39" width="16.88671875" style="3" bestFit="1" customWidth="1"/>
+    <col min="39" max="39" width="16.85546875" style="3" bestFit="1" customWidth="1"/>
     <col min="40" max="40" width="13" style="18" bestFit="1" customWidth="1"/>
     <col min="41" max="41" width="13" style="22" customWidth="1"/>
     <col min="42" max="42" width="17" style="27" bestFit="1" customWidth="1"/>
-    <col min="43" max="43" width="24.88671875" style="3" bestFit="1" customWidth="1"/>
-    <col min="44" max="16384" width="9.109375" style="3"/>
+    <col min="43" max="43" width="24.85546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="44" max="16384" width="9.140625" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:43" s="5" customFormat="1" ht="16.8" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:43" s="5" customFormat="1" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
         <v>70</v>
       </c>
@@ -8955,7 +9239,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="2" spans="1:43" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
+    <row r="2" spans="1:43" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <autoFilter ref="A1:AQ1" xr:uid="{00000000-0009-0000-0000-000006000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -8967,22 +9251,22 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1:N2"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="13.8" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="20.6640625" style="7" customWidth="1"/>
-    <col min="2" max="3" width="25.6640625" style="7" customWidth="1"/>
-    <col min="4" max="4" width="20.6640625" style="7" customWidth="1"/>
-    <col min="5" max="5" width="25.6640625" style="7" customWidth="1"/>
-    <col min="6" max="7" width="15.6640625" style="7" customWidth="1"/>
-    <col min="8" max="8" width="13.109375" style="23" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.109375" style="28" bestFit="1" customWidth="1"/>
-    <col min="10" max="11" width="25.6640625" style="7" customWidth="1"/>
-    <col min="12" max="13" width="15.44140625" style="7" customWidth="1"/>
+    <col min="1" max="1" width="20.7109375" style="7" customWidth="1"/>
+    <col min="2" max="3" width="25.7109375" style="7" customWidth="1"/>
+    <col min="4" max="4" width="20.7109375" style="7" customWidth="1"/>
+    <col min="5" max="5" width="25.7109375" style="7" customWidth="1"/>
+    <col min="6" max="7" width="15.7109375" style="7" customWidth="1"/>
+    <col min="8" max="8" width="13.140625" style="23" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13.140625" style="28" bestFit="1" customWidth="1"/>
+    <col min="10" max="11" width="25.7109375" style="7" customWidth="1"/>
+    <col min="12" max="13" width="15.42578125" style="7" customWidth="1"/>
     <col min="14" max="14" width="11" style="7" customWidth="1"/>
-    <col min="15" max="16384" width="9.109375" style="7"/>
+    <col min="15" max="16384" width="9.140625" style="7"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" s="9" customFormat="1" ht="20.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:14" s="9" customFormat="1" ht="20.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="9" t="s">
         <v>27</v>
       </c>
@@ -9026,7 +9310,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="2" spans="1:14" ht="14.4" thickTop="1" x14ac:dyDescent="0.3"/>
+    <row r="2" spans="1:14" ht="13.5" thickTop="1" x14ac:dyDescent="0.2"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -9036,24 +9320,24 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
   <dimension ref="A1:N2"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12" style="16" customWidth="1"/>
     <col min="2" max="2" width="24" style="16" customWidth="1"/>
-    <col min="3" max="3" width="25.5546875" style="16" customWidth="1"/>
-    <col min="4" max="4" width="10.5546875" style="16" customWidth="1"/>
-    <col min="5" max="6" width="10.5546875" style="16" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="10.5546875" style="16" customWidth="1"/>
-    <col min="8" max="8" width="20.44140625" style="16" customWidth="1"/>
-    <col min="9" max="9" width="18.109375" style="16" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="18.88671875" style="16" bestFit="1" customWidth="1"/>
-    <col min="11" max="12" width="10.6640625" style="17" customWidth="1"/>
-    <col min="13" max="13" width="20.6640625" style="25" customWidth="1"/>
-    <col min="14" max="14" width="20.6640625" style="30" customWidth="1"/>
-    <col min="15" max="16384" width="9.109375" style="16"/>
+    <col min="3" max="3" width="25.5703125" style="16" customWidth="1"/>
+    <col min="4" max="4" width="10.5703125" style="16" customWidth="1"/>
+    <col min="5" max="6" width="10.5703125" style="16" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.5703125" style="16" customWidth="1"/>
+    <col min="8" max="8" width="20.42578125" style="16" customWidth="1"/>
+    <col min="9" max="9" width="18.140625" style="16" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="18.85546875" style="16" bestFit="1" customWidth="1"/>
+    <col min="11" max="12" width="10.7109375" style="17" customWidth="1"/>
+    <col min="13" max="13" width="20.7109375" style="25" customWidth="1"/>
+    <col min="14" max="14" width="20.7109375" style="30" customWidth="1"/>
+    <col min="15" max="16384" width="9.140625" style="16"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" s="2" customFormat="1" ht="16.8" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:14" s="2" customFormat="1" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>2</v>
       </c>
@@ -9097,7 +9381,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="2" spans="1:14" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
+    <row r="2" spans="1:14" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <autoFilter ref="A1:N2" xr:uid="{00000000-0009-0000-0000-000008000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -9106,6 +9390,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance">
   <documentManagement>
     <Unity_Description xmlns="D75E00DB-06CE-4005-B397-8C0860A4229B" xsi:nil="true"/>
@@ -9116,15 +9409,6 @@
     </SipLabel>
   </documentManagement>
 </p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -9231,6 +9515,14 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2653FDDC-5C81-4B5A-A42F-7A63208AFFF7}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{268822B0-DCAE-4D2C-8340-AB7554C48D72}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
@@ -9243,14 +9535,6 @@
     <ds:schemaRef ds:uri="372b77af-8063-48a8-888c-73c0edf01dea"/>
     <ds:schemaRef ds:uri="d75e00db-06ce-4005-b397-8c0860a4229b"/>
     <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2653FDDC-5C81-4B5A-A42F-7A63208AFFF7}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
4806 - Update existing Excel export sheets for MOQ types
</commit_message>
<xml_diff>
--- a/GenBOE/GenBOE.Web/Templates/Export/WorkspaceDataMST.xlsx
+++ b/GenBOE/GenBOE.Web/Templates/Export/WorkspaceDataMST.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ranzalon\Source\repos\IES\GenBOE\GenBOE.Web\Templates\Export\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58097765-AAC1-4376-A4D2-B691E2FF6DBD}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{979CE1BE-6AD7-450F-82CE-0EC06B50ACC2}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="25080" yWindow="-120" windowWidth="25440" windowHeight="15990" firstSheet="5" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -54,9 +54,9 @@
   </definedNames>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="3" r:id="rId21"/>
-    <pivotCache cacheId="4" r:id="rId22"/>
-    <pivotCache cacheId="5" r:id="rId23"/>
+    <pivotCache cacheId="12" r:id="rId21"/>
+    <pivotCache cacheId="13" r:id="rId22"/>
+    <pivotCache cacheId="14" r:id="rId23"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -3145,7 +3145,7 @@
 <file path=xl/pivotCache/pivotCacheDefinition2.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="Lindsay Yorks" refreshedDate="40653.729487847224" createdVersion="3" refreshedVersion="3" minRefreshableVersion="3" recordCount="15" xr:uid="{00000000-000A-0000-FFFF-FFFF01000000}">
   <cacheSource type="worksheet">
-    <worksheetSource ref="B1:AP1" sheet="BOEs"/>
+    <worksheetSource ref="C1:AP1" sheet="BOEs"/>
   </cacheSource>
   <cacheFields count="19">
     <cacheField name="Type" numFmtId="49">
@@ -4349,7 +4349,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0000-000000000000}" name="PivotTable7" cacheId="3" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="3" minRefreshableVersion="3" showCalcMbrs="0" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="3" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0000-000000000000}" name="PivotTable7" cacheId="12" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="3" minRefreshableVersion="3" showCalcMbrs="0" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="3" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
   <location ref="A3:N33" firstHeaderRow="1" firstDataRow="1" firstDataCol="14"/>
   <pivotFields count="14">
     <pivotField axis="axisRow" compact="0" outline="0" showAll="0" insertBlankRow="1" defaultSubtotal="0">
@@ -4698,7 +4698,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0200-000000000000}" name="PivotTable9" cacheId="4" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="3" minRefreshableVersion="3" showCalcMbrs="0" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="3" indent="0" compact="0" compactData="0" multipleFieldFilters="0" rowHeaderCaption="Type">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0200-000000000000}" name="PivotTable9" cacheId="13" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="3" minRefreshableVersion="3" showCalcMbrs="0" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="3" indent="0" compact="0" compactData="0" multipleFieldFilters="0" rowHeaderCaption="Type">
   <location ref="A3:H11" firstHeaderRow="1" firstDataRow="1" firstDataCol="8"/>
   <pivotFields count="19">
     <pivotField axis="axisRow" compact="0" outline="0" showAll="0" defaultSubtotal="0">
@@ -4907,7 +4907,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0300-000000000000}" name="PivotTable4" cacheId="5" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" missingCaption="_" updatedVersion="3" minRefreshableVersion="3" showCalcMbrs="0" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="3" indent="0" compact="0" compactData="0" multipleFieldFilters="0" rowHeaderCaption="BOE ID">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0300-000000000000}" name="PivotTable4" cacheId="14" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" missingCaption="_" updatedVersion="3" minRefreshableVersion="3" showCalcMbrs="0" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="3" indent="0" compact="0" compactData="0" multipleFieldFilters="0" rowHeaderCaption="BOE ID">
   <location ref="A3:T33" firstHeaderRow="1" firstDataRow="1" firstDataCol="20"/>
   <pivotFields count="20">
     <pivotField axis="axisRow" compact="0" outline="0" showAll="0" insertBlankRow="1" defaultSubtotal="0">
@@ -8884,19 +8884,19 @@
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.85546875" style="1" customWidth="1"/>
-    <col min="3" max="3" width="11.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="18.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="14.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="19.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="19.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="10.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="13.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="19.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="10.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="13.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.85546875" style="1" customWidth="1"/>
+    <col min="4" max="4" width="11.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="18.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="19.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="19.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="10.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="13.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="19.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="10.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="13.5703125" style="1" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="13.42578125" style="38" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="12.5703125" style="38" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="21.42578125" style="1" bestFit="1" customWidth="1"/>
@@ -8933,43 +8933,43 @@
         <v>70</v>
       </c>
       <c r="B1" s="5" t="s">
+        <v>115</v>
+      </c>
+      <c r="C1" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="D1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="E1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="5" t="s">
+      <c r="F1" s="5" t="s">
         <v>119</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="G1" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="G1" s="5" t="s">
+      <c r="H1" s="5" t="s">
         <v>118</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="I1" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="I1" s="5" t="s">
+      <c r="J1" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="J1" s="5" t="s">
+      <c r="K1" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="K1" s="5" t="s">
+      <c r="L1" s="5" t="s">
         <v>124</v>
       </c>
-      <c r="L1" s="5" t="s">
+      <c r="M1" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="M1" s="5" t="s">
+      <c r="N1" s="5" t="s">
         <v>30</v>
-      </c>
-      <c r="N1" s="5" t="s">
-        <v>115</v>
       </c>
       <c r="O1" s="37" t="s">
         <v>31</v>
@@ -9070,9 +9070,9 @@
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.42578125" style="3" customWidth="1"/>
-    <col min="2" max="3" width="10.5703125" style="3" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.5703125" style="3" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.140625" style="3" customWidth="1"/>
+    <col min="2" max="2" width="12.140625" style="3" customWidth="1"/>
+    <col min="3" max="4" width="10.5703125" style="3" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.5703125" style="3" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="10.5703125" style="3" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="13.5703125" style="3" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="13.42578125" style="3" bestFit="1" customWidth="1"/>
@@ -9113,16 +9113,16 @@
         <v>70</v>
       </c>
       <c r="B1" s="5" t="s">
+        <v>115</v>
+      </c>
+      <c r="C1" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="D1" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="E1" s="5" t="s">
         <v>28</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>115</v>
       </c>
       <c r="F1" s="5" t="s">
         <v>29</v>
@@ -9390,28 +9390,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance">
-  <documentManagement>
-    <Unity_Description xmlns="D75E00DB-06CE-4005-B397-8C0860A4229B" xsi:nil="true"/>
-    <Unity_Tag xmlns="D75E00DB-06CE-4005-B397-8C0860A4229B" xsi:nil="true"/>
-    <Capabilities xmlns="d75e00db-06ce-4005-b397-8c0860a4229b" xsi:nil="true"/>
-    <SipLabel xmlns="372b77af-8063-48a8-888c-73c0edf01dea">
-      <Value>2</Value>
-    </SipLabel>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Custom Document" ma:contentTypeID="0x010100E6322E8F405D4D9EA89D8C83B7E1048B001BB96E1BE0ACBB41BF00782ED0412411" ma:contentTypeVersion="3" ma:contentTypeDescription="Custom Document" ma:contentTypeScope="" ma:versionID="3c14126572fa3c0d4c677ac1f3ba4426">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="D75E00DB-06CE-4005-B397-8C0860A4229B" xmlns:ns3="372b77af-8063-48a8-888c-73c0edf01dea" xmlns:ns4="d75e00db-06ce-4005-b397-8c0860a4229b" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="9e89026a025b72b85b9543506e7af3e1" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="D75E00DB-06CE-4005-B397-8C0860A4229B"/>
@@ -9514,10 +9492,43 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance">
+  <documentManagement>
+    <Unity_Description xmlns="D75E00DB-06CE-4005-B397-8C0860A4229B" xsi:nil="true"/>
+    <Unity_Tag xmlns="D75E00DB-06CE-4005-B397-8C0860A4229B" xsi:nil="true"/>
+    <Capabilities xmlns="d75e00db-06ce-4005-b397-8c0860a4229b" xsi:nil="true"/>
+    <SipLabel xmlns="372b77af-8063-48a8-888c-73c0edf01dea">
+      <Value>2</Value>
+    </SipLabel>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2653FDDC-5C81-4B5A-A42F-7A63208AFFF7}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1DE4120D-B400-435F-B862-B3B8683830A5}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="D75E00DB-06CE-4005-B397-8C0860A4229B"/>
+    <ds:schemaRef ds:uri="372b77af-8063-48a8-888c-73c0edf01dea"/>
+    <ds:schemaRef ds:uri="d75e00db-06ce-4005-b397-8c0860a4229b"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/internal/2005/internalDocumentation"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -9540,20 +9551,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1DE4120D-B400-435F-B862-B3B8683830A5}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2653FDDC-5C81-4B5A-A42F-7A63208AFFF7}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="D75E00DB-06CE-4005-B397-8C0860A4229B"/>
-    <ds:schemaRef ds:uri="372b77af-8063-48a8-888c-73c0edf01dea"/>
-    <ds:schemaRef ds:uri="d75e00db-06ce-4005-b397-8c0860a4229b"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/internal/2005/internalDocumentation"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
4910 - MOQ Table Data sheet for excel export
</commit_message>
<xml_diff>
--- a/GenBOE/GenBOE.Web/Templates/Export/WorkspaceDataMST.xlsx
+++ b/GenBOE/GenBOE.Web/Templates/Export/WorkspaceDataMST.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ranzalon\Source\repos\IES\GenBOE\GenBOE.Web\Templates\Export\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{979CE1BE-6AD7-450F-82CE-0EC06B50ACC2}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{355601B4-D73E-4EB5-BF6C-4DDA9020847B}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="25080" yWindow="-120" windowWidth="25440" windowHeight="15990" firstSheet="5" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -42,7 +42,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'BOEs (2)'!$B$1:$T$16</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'BOEs (3)'!$A$1:$N$16</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'MOQ by BOE by Task'!$A$1:$G$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'MOQ Table Data'!$A$1:$Q$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'MOQ Table Data'!$A$1:$O$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Resource Spreads'!$A$1:$N$2</definedName>
     <definedName name="Approvers">'[1]Options Lists'!$D$2:$D$4</definedName>
     <definedName name="Authors">'[1]Options Lists'!$C$2:$C$4</definedName>
@@ -54,9 +54,9 @@
   </definedNames>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="12" r:id="rId21"/>
-    <pivotCache cacheId="13" r:id="rId22"/>
-    <pivotCache cacheId="14" r:id="rId23"/>
+    <pivotCache cacheId="9" r:id="rId21"/>
+    <pivotCache cacheId="10" r:id="rId22"/>
+    <pivotCache cacheId="11" r:id="rId23"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -321,7 +321,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="879" uniqueCount="142">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="877" uniqueCount="140">
   <si>
     <t>Start Date</t>
   </si>
@@ -708,12 +708,6 @@
   </si>
   <si>
     <t>Table Name</t>
-  </si>
-  <si>
-    <t>Repository Name</t>
-  </si>
-  <si>
-    <t>Query Type (Weekly/Monthly)</t>
   </si>
   <si>
     <t>Date of Report</t>
@@ -4349,7 +4343,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0000-000000000000}" name="PivotTable7" cacheId="12" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="3" minRefreshableVersion="3" showCalcMbrs="0" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="3" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0000-000000000000}" name="PivotTable7" cacheId="9" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="3" minRefreshableVersion="3" showCalcMbrs="0" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="3" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
   <location ref="A3:N33" firstHeaderRow="1" firstDataRow="1" firstDataCol="14"/>
   <pivotFields count="14">
     <pivotField axis="axisRow" compact="0" outline="0" showAll="0" insertBlankRow="1" defaultSubtotal="0">
@@ -4698,7 +4692,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0200-000000000000}" name="PivotTable9" cacheId="13" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="3" minRefreshableVersion="3" showCalcMbrs="0" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="3" indent="0" compact="0" compactData="0" multipleFieldFilters="0" rowHeaderCaption="Type">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0200-000000000000}" name="PivotTable9" cacheId="10" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="3" minRefreshableVersion="3" showCalcMbrs="0" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="3" indent="0" compact="0" compactData="0" multipleFieldFilters="0" rowHeaderCaption="Type">
   <location ref="A3:H11" firstHeaderRow="1" firstDataRow="1" firstDataCol="8"/>
   <pivotFields count="19">
     <pivotField axis="axisRow" compact="0" outline="0" showAll="0" defaultSubtotal="0">
@@ -4907,7 +4901,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0300-000000000000}" name="PivotTable4" cacheId="14" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" missingCaption="_" updatedVersion="3" minRefreshableVersion="3" showCalcMbrs="0" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="3" indent="0" compact="0" compactData="0" multipleFieldFilters="0" rowHeaderCaption="BOE ID">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0300-000000000000}" name="PivotTable4" cacheId="11" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" missingCaption="_" updatedVersion="3" minRefreshableVersion="3" showCalcMbrs="0" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="3" indent="0" compact="0" compactData="0" multipleFieldFilters="0" rowHeaderCaption="BOE ID">
   <location ref="A3:T33" firstHeaderRow="1" firstDataRow="1" firstDataCol="20"/>
   <pivotFields count="20">
     <pivotField axis="axisRow" compact="0" outline="0" showAll="0" insertBlankRow="1" defaultSubtotal="0">
@@ -6231,7 +6225,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EDDB750B-2EAA-4C67-B526-87C6863613C3}">
-  <dimension ref="A1:Q2"/>
+  <dimension ref="A1:O2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.140625" bestFit="1" customWidth="1"/>
@@ -6240,20 +6234,18 @@
     <col min="4" max="4" width="24" customWidth="1"/>
     <col min="5" max="5" width="42.28515625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="15.85546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="21.28515625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="33.7109375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="18.85546875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="28.85546875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="21.140625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="23" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="42" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="41.140625" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="35.28515625" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="57.85546875" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="61.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="18.85546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="28.85546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="23" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="42" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="41.140625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="35.28515625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="57.85546875" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="61.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:15" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
         <v>70</v>
       </c>
@@ -6299,16 +6291,10 @@
       <c r="O1" s="5" t="s">
         <v>137</v>
       </c>
-      <c r="P1" s="5" t="s">
-        <v>138</v>
-      </c>
-      <c r="Q1" s="5" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="2" spans="1:17" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
+    </row>
+    <row r="2" spans="1:15" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
   </sheetData>
-  <autoFilter ref="A1:Q1" xr:uid="{24A73A91-4C44-47FC-8450-35CF267C3337}"/>
+  <autoFilter ref="A1:O1" xr:uid="{24A73A91-4C44-47FC-8450-35CF267C3337}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -6328,10 +6314,10 @@
         <v>84</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
     </row>
     <row r="2" spans="1:3" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
@@ -9070,7 +9056,7 @@
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.42578125" style="3" customWidth="1"/>
-    <col min="2" max="2" width="12.140625" style="3" customWidth="1"/>
+    <col min="2" max="2" width="13.28515625" style="3" bestFit="1" customWidth="1"/>
     <col min="3" max="4" width="10.5703125" style="3" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="13.5703125" style="3" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="10.5703125" style="3" bestFit="1" customWidth="1"/>
@@ -9390,6 +9376,28 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance">
+  <documentManagement>
+    <Unity_Description xmlns="D75E00DB-06CE-4005-B397-8C0860A4229B" xsi:nil="true"/>
+    <Unity_Tag xmlns="D75E00DB-06CE-4005-B397-8C0860A4229B" xsi:nil="true"/>
+    <Capabilities xmlns="d75e00db-06ce-4005-b397-8c0860a4229b" xsi:nil="true"/>
+    <SipLabel xmlns="372b77af-8063-48a8-888c-73c0edf01dea">
+      <Value>2</Value>
+    </SipLabel>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Custom Document" ma:contentTypeID="0x010100E6322E8F405D4D9EA89D8C83B7E1048B001BB96E1BE0ACBB41BF00782ED0412411" ma:contentTypeVersion="3" ma:contentTypeDescription="Custom Document" ma:contentTypeScope="" ma:versionID="3c14126572fa3c0d4c677ac1f3ba4426">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="D75E00DB-06CE-4005-B397-8C0860A4229B" xmlns:ns3="372b77af-8063-48a8-888c-73c0edf01dea" xmlns:ns4="d75e00db-06ce-4005-b397-8c0860a4229b" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="9e89026a025b72b85b9543506e7af3e1" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="D75E00DB-06CE-4005-B397-8C0860A4229B"/>
@@ -9492,43 +9500,10 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance">
-  <documentManagement>
-    <Unity_Description xmlns="D75E00DB-06CE-4005-B397-8C0860A4229B" xsi:nil="true"/>
-    <Unity_Tag xmlns="D75E00DB-06CE-4005-B397-8C0860A4229B" xsi:nil="true"/>
-    <Capabilities xmlns="d75e00db-06ce-4005-b397-8c0860a4229b" xsi:nil="true"/>
-    <SipLabel xmlns="372b77af-8063-48a8-888c-73c0edf01dea">
-      <Value>2</Value>
-    </SipLabel>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1DE4120D-B400-435F-B862-B3B8683830A5}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2653FDDC-5C81-4B5A-A42F-7A63208AFFF7}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="D75E00DB-06CE-4005-B397-8C0860A4229B"/>
-    <ds:schemaRef ds:uri="372b77af-8063-48a8-888c-73c0edf01dea"/>
-    <ds:schemaRef ds:uri="d75e00db-06ce-4005-b397-8c0860a4229b"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/internal/2005/internalDocumentation"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -9551,9 +9526,20 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2653FDDC-5C81-4B5A-A42F-7A63208AFFF7}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1DE4120D-B400-435F-B862-B3B8683830A5}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="D75E00DB-06CE-4005-B397-8C0860A4229B"/>
+    <ds:schemaRef ds:uri="372b77af-8063-48a8-888c-73c0edf01dea"/>
+    <ds:schemaRef ds:uri="d75e00db-06ce-4005-b397-8c0860a4229b"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/internal/2005/internalDocumentation"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
4911 - MOQ Summary sheet for excel export
</commit_message>
<xml_diff>
--- a/GenBOE/GenBOE.Web/Templates/Export/WorkspaceDataMST.xlsx
+++ b/GenBOE/GenBOE.Web/Templates/Export/WorkspaceDataMST.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ranzalon\Source\repos\IES\GenBOE\GenBOE.Web\Templates\Export\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{355601B4-D73E-4EB5-BF6C-4DDA9020847B}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9C4AECB-FEE8-49D8-A00A-246A93C2370B}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="25080" yWindow="-120" windowWidth="25440" windowHeight="15990" firstSheet="5" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -54,9 +54,9 @@
   </definedNames>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="9" r:id="rId21"/>
-    <pivotCache cacheId="10" r:id="rId22"/>
-    <pivotCache cacheId="11" r:id="rId23"/>
+    <pivotCache cacheId="33" r:id="rId21"/>
+    <pivotCache cacheId="34" r:id="rId22"/>
+    <pivotCache cacheId="35" r:id="rId23"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -747,11 +747,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="4">
+  <numFmts count="5">
     <numFmt numFmtId="164" formatCode="m/yyyy"/>
     <numFmt numFmtId="165" formatCode="m/d/yyyy;@"/>
     <numFmt numFmtId="166" formatCode="0.000"/>
     <numFmt numFmtId="167" formatCode="&quot;$&quot;#,##0.00"/>
+    <numFmt numFmtId="168" formatCode="0.0%"/>
   </numFmts>
   <fonts count="14" x14ac:knownFonts="1">
     <font>
@@ -989,7 +990,7 @@
     <xf numFmtId="0" fontId="10" fillId="6" borderId="0"/>
     <xf numFmtId="0" fontId="13" fillId="7" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="61">
+  <cellXfs count="63">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="1" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyAlignment="1">
@@ -1147,6 +1148,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="168" fontId="1" fillId="2" borderId="1" xfId="1" applyNumberFormat="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="8">
     <cellStyle name="genBOE" xfId="1" xr:uid="{00000000-0005-0000-0000-000000000000}"/>
@@ -4343,7 +4348,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0000-000000000000}" name="PivotTable7" cacheId="9" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="3" minRefreshableVersion="3" showCalcMbrs="0" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="3" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0000-000000000000}" name="PivotTable7" cacheId="33" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="3" minRefreshableVersion="3" showCalcMbrs="0" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="3" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
   <location ref="A3:N33" firstHeaderRow="1" firstDataRow="1" firstDataCol="14"/>
   <pivotFields count="14">
     <pivotField axis="axisRow" compact="0" outline="0" showAll="0" insertBlankRow="1" defaultSubtotal="0">
@@ -4692,7 +4697,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0200-000000000000}" name="PivotTable9" cacheId="10" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="3" minRefreshableVersion="3" showCalcMbrs="0" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="3" indent="0" compact="0" compactData="0" multipleFieldFilters="0" rowHeaderCaption="Type">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0200-000000000000}" name="PivotTable9" cacheId="34" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="3" minRefreshableVersion="3" showCalcMbrs="0" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="3" indent="0" compact="0" compactData="0" multipleFieldFilters="0" rowHeaderCaption="Type">
   <location ref="A3:H11" firstHeaderRow="1" firstDataRow="1" firstDataCol="8"/>
   <pivotFields count="19">
     <pivotField axis="axisRow" compact="0" outline="0" showAll="0" defaultSubtotal="0">
@@ -4901,7 +4906,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0300-000000000000}" name="PivotTable4" cacheId="11" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" missingCaption="_" updatedVersion="3" minRefreshableVersion="3" showCalcMbrs="0" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="3" indent="0" compact="0" compactData="0" multipleFieldFilters="0" rowHeaderCaption="BOE ID">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0300-000000000000}" name="PivotTable4" cacheId="35" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" missingCaption="_" updatedVersion="3" minRefreshableVersion="3" showCalcMbrs="0" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="3" indent="0" compact="0" compactData="0" multipleFieldFilters="0" rowHeaderCaption="BOE ID">
   <location ref="A3:T33" firstHeaderRow="1" firstDataRow="1" firstDataCol="20"/>
   <pivotFields count="20">
     <pivotField axis="axisRow" compact="0" outline="0" showAll="0" insertBlankRow="1" defaultSubtotal="0">
@@ -6306,7 +6311,7 @@
   <cols>
     <col min="1" max="1" width="40.85546875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="24.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.140625" style="62" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -6316,7 +6321,7 @@
       <c r="B1" s="5" t="s">
         <v>138</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="C1" s="61" t="s">
         <v>139</v>
       </c>
     </row>
@@ -9376,28 +9381,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance">
-  <documentManagement>
-    <Unity_Description xmlns="D75E00DB-06CE-4005-B397-8C0860A4229B" xsi:nil="true"/>
-    <Unity_Tag xmlns="D75E00DB-06CE-4005-B397-8C0860A4229B" xsi:nil="true"/>
-    <Capabilities xmlns="d75e00db-06ce-4005-b397-8c0860a4229b" xsi:nil="true"/>
-    <SipLabel xmlns="372b77af-8063-48a8-888c-73c0edf01dea">
-      <Value>2</Value>
-    </SipLabel>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Custom Document" ma:contentTypeID="0x010100E6322E8F405D4D9EA89D8C83B7E1048B001BB96E1BE0ACBB41BF00782ED0412411" ma:contentTypeVersion="3" ma:contentTypeDescription="Custom Document" ma:contentTypeScope="" ma:versionID="3c14126572fa3c0d4c677ac1f3ba4426">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="D75E00DB-06CE-4005-B397-8C0860A4229B" xmlns:ns3="372b77af-8063-48a8-888c-73c0edf01dea" xmlns:ns4="d75e00db-06ce-4005-b397-8c0860a4229b" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="9e89026a025b72b85b9543506e7af3e1" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="D75E00DB-06CE-4005-B397-8C0860A4229B"/>
@@ -9500,10 +9483,43 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance">
+  <documentManagement>
+    <Unity_Description xmlns="D75E00DB-06CE-4005-B397-8C0860A4229B" xsi:nil="true"/>
+    <Unity_Tag xmlns="D75E00DB-06CE-4005-B397-8C0860A4229B" xsi:nil="true"/>
+    <Capabilities xmlns="d75e00db-06ce-4005-b397-8c0860a4229b" xsi:nil="true"/>
+    <SipLabel xmlns="372b77af-8063-48a8-888c-73c0edf01dea">
+      <Value>2</Value>
+    </SipLabel>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2653FDDC-5C81-4B5A-A42F-7A63208AFFF7}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1DE4120D-B400-435F-B862-B3B8683830A5}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="D75E00DB-06CE-4005-B397-8C0860A4229B"/>
+    <ds:schemaRef ds:uri="372b77af-8063-48a8-888c-73c0edf01dea"/>
+    <ds:schemaRef ds:uri="d75e00db-06ce-4005-b397-8c0860a4229b"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/internal/2005/internalDocumentation"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -9526,20 +9542,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1DE4120D-B400-435F-B862-B3B8683830A5}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2653FDDC-5C81-4B5A-A42F-7A63208AFFF7}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="D75E00DB-06CE-4005-B397-8C0860A4229B"/>
-    <ds:schemaRef ds:uri="372b77af-8063-48a8-888c-73c0edf01dea"/>
-    <ds:schemaRef ds:uri="d75e00db-06ce-4005-b397-8c0860a4229b"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/internal/2005/internalDocumentation"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
4972 - Remove MOQ Type Selection from the Resource Types, Remove "location" for CER/PE/AR MOQ Types, Remove MOQ Summary from Workspce Data export
</commit_message>
<xml_diff>
--- a/GenBOE/GenBOE.Web/Templates/Export/WorkspaceDataMST.xlsx
+++ b/GenBOE/GenBOE.Web/Templates/Export/WorkspaceDataMST.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ranzalon\Source\repos\IES\GenBOE\GenBOE.Web\Templates\Export\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9C4AECB-FEE8-49D8-A00A-246A93C2370B}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE39FAC7-A498-44DA-9819-C44D307D47E9}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="25080" yWindow="-120" windowWidth="25440" windowHeight="15990" firstSheet="5" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3120" yWindow="345" windowWidth="18900" windowHeight="11055" firstSheet="5" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="BOE3 Pivot" sheetId="19" state="hidden" r:id="rId1"/>
@@ -24,17 +24,16 @@
     <sheet name="Resource Spreads" sheetId="41" r:id="rId9"/>
     <sheet name="MOQ by BOE by Task" sheetId="45" r:id="rId10"/>
     <sheet name="MOQ Table Data" sheetId="46" r:id="rId11"/>
-    <sheet name="MOQ Summary" sheetId="47" r:id="rId12"/>
-    <sheet name="WBS" sheetId="24" r:id="rId13"/>
-    <sheet name="CLINs" sheetId="25" r:id="rId14"/>
-    <sheet name="User Permissions" sheetId="39" r:id="rId15"/>
-    <sheet name="Workspace Identification" sheetId="40" r:id="rId16"/>
-    <sheet name="Travel Unit Cost" sheetId="43" r:id="rId17"/>
-    <sheet name="Travel Extended Cost" sheetId="44" r:id="rId18"/>
+    <sheet name="WBS" sheetId="24" r:id="rId12"/>
+    <sheet name="CLINs" sheetId="25" r:id="rId13"/>
+    <sheet name="User Permissions" sheetId="39" r:id="rId14"/>
+    <sheet name="Workspace Identification" sheetId="40" r:id="rId15"/>
+    <sheet name="Travel Unit Cost" sheetId="43" r:id="rId16"/>
+    <sheet name="Travel Extended Cost" sheetId="44" r:id="rId17"/>
   </sheets>
   <externalReferences>
+    <externalReference r:id="rId18"/>
     <externalReference r:id="rId19"/>
-    <externalReference r:id="rId20"/>
   </externalReferences>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'BOE &amp; Resource Combo'!$A$1:$AP$1</definedName>
@@ -54,9 +53,9 @@
   </definedNames>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="33" r:id="rId21"/>
-    <pivotCache cacheId="34" r:id="rId22"/>
-    <pivotCache cacheId="35" r:id="rId23"/>
+    <pivotCache cacheId="0" r:id="rId20"/>
+    <pivotCache cacheId="1" r:id="rId21"/>
+    <pivotCache cacheId="2" r:id="rId22"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -321,7 +320,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="877" uniqueCount="140">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="874" uniqueCount="138">
   <si>
     <t>Start Date</t>
   </si>
@@ -735,24 +734,17 @@
   </si>
   <si>
     <t>Total Relevant Hours After Additional Query Filters Applied</t>
-  </si>
-  <si>
-    <t>MOQ Hours Bid/Spread</t>
-  </si>
-  <si>
-    <t>% of total</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="5">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="m/yyyy"/>
     <numFmt numFmtId="165" formatCode="m/d/yyyy;@"/>
     <numFmt numFmtId="166" formatCode="0.000"/>
     <numFmt numFmtId="167" formatCode="&quot;$&quot;#,##0.00"/>
-    <numFmt numFmtId="168" formatCode="0.0%"/>
   </numFmts>
   <fonts count="14" x14ac:knownFonts="1">
     <font>
@@ -990,7 +982,7 @@
     <xf numFmtId="0" fontId="10" fillId="6" borderId="0"/>
     <xf numFmtId="0" fontId="13" fillId="7" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="63">
+  <cellXfs count="61">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="1" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyAlignment="1">
@@ -1148,10 +1140,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="168" fontId="1" fillId="2" borderId="1" xfId="1" applyNumberFormat="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="8">
     <cellStyle name="genBOE" xfId="1" xr:uid="{00000000-0005-0000-0000-000000000000}"/>
@@ -4348,7 +4336,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0000-000000000000}" name="PivotTable7" cacheId="33" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="3" minRefreshableVersion="3" showCalcMbrs="0" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="3" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0000-000000000000}" name="PivotTable7" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="3" minRefreshableVersion="3" showCalcMbrs="0" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="3" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
   <location ref="A3:N33" firstHeaderRow="1" firstDataRow="1" firstDataCol="14"/>
   <pivotFields count="14">
     <pivotField axis="axisRow" compact="0" outline="0" showAll="0" insertBlankRow="1" defaultSubtotal="0">
@@ -4697,7 +4685,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0200-000000000000}" name="PivotTable9" cacheId="34" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="3" minRefreshableVersion="3" showCalcMbrs="0" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="3" indent="0" compact="0" compactData="0" multipleFieldFilters="0" rowHeaderCaption="Type">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0200-000000000000}" name="PivotTable9" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="3" minRefreshableVersion="3" showCalcMbrs="0" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="3" indent="0" compact="0" compactData="0" multipleFieldFilters="0" rowHeaderCaption="Type">
   <location ref="A3:H11" firstHeaderRow="1" firstDataRow="1" firstDataCol="8"/>
   <pivotFields count="19">
     <pivotField axis="axisRow" compact="0" outline="0" showAll="0" defaultSubtotal="0">
@@ -4906,7 +4894,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0300-000000000000}" name="PivotTable4" cacheId="35" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" missingCaption="_" updatedVersion="3" minRefreshableVersion="3" showCalcMbrs="0" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="3" indent="0" compact="0" compactData="0" multipleFieldFilters="0" rowHeaderCaption="BOE ID">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0300-000000000000}" name="PivotTable4" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" missingCaption="_" updatedVersion="3" minRefreshableVersion="3" showCalcMbrs="0" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="3" indent="0" compact="0" compactData="0" multipleFieldFilters="0" rowHeaderCaption="BOE ID">
   <location ref="A3:T33" firstHeaderRow="1" firstDataRow="1" firstDataCol="20"/>
   <pivotFields count="20">
     <pivotField axis="axisRow" compact="0" outline="0" showAll="0" insertBlankRow="1" defaultSubtotal="0">
@@ -6305,33 +6293,6 @@
 </file>
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C5C2B818-1ECD-43FE-AA03-6B27248B8CDB}">
-  <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="40.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="24.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.140625" style="62" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="5" t="s">
-        <v>84</v>
-      </c>
-      <c r="B1" s="5" t="s">
-        <v>138</v>
-      </c>
-      <c r="C1" s="61" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
   <dimension ref="A1:E2"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
@@ -6367,7 +6328,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
   <dimension ref="A1:E2"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
@@ -6404,7 +6365,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0B00-000000000000}">
   <dimension ref="A1:I2"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -6456,7 +6417,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0C00-000000000000}">
   <dimension ref="A1:A16"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -6542,7 +6503,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1E9E49D2-B4A1-426D-8F6A-B85DD2E6A5AA}">
   <dimension ref="A1:AA7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -6763,7 +6724,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00BB237A-2FF2-450F-81EE-9A098F6C7133}">
   <dimension ref="A1:AA6"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -9381,6 +9342,19 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance">
+  <documentManagement>
+    <Unity_Description xmlns="D75E00DB-06CE-4005-B397-8C0860A4229B" xsi:nil="true"/>
+    <Unity_Tag xmlns="D75E00DB-06CE-4005-B397-8C0860A4229B" xsi:nil="true"/>
+    <Capabilities xmlns="d75e00db-06ce-4005-b397-8c0860a4229b" xsi:nil="true"/>
+    <SipLabel xmlns="372b77af-8063-48a8-888c-73c0edf01dea">
+      <Value>2</Value>
+    </SipLabel>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Custom Document" ma:contentTypeID="0x010100E6322E8F405D4D9EA89D8C83B7E1048B001BB96E1BE0ACBB41BF00782ED0412411" ma:contentTypeVersion="3" ma:contentTypeDescription="Custom Document" ma:contentTypeScope="" ma:versionID="3c14126572fa3c0d4c677ac1f3ba4426">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="D75E00DB-06CE-4005-B397-8C0860A4229B" xmlns:ns3="372b77af-8063-48a8-888c-73c0edf01dea" xmlns:ns4="d75e00db-06ce-4005-b397-8c0860a4229b" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="9e89026a025b72b85b9543506e7af3e1" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="D75E00DB-06CE-4005-B397-8C0860A4229B"/>
@@ -9483,19 +9457,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance">
-  <documentManagement>
-    <Unity_Description xmlns="D75E00DB-06CE-4005-B397-8C0860A4229B" xsi:nil="true"/>
-    <Unity_Tag xmlns="D75E00DB-06CE-4005-B397-8C0860A4229B" xsi:nil="true"/>
-    <Capabilities xmlns="d75e00db-06ce-4005-b397-8c0860a4229b" xsi:nil="true"/>
-    <SipLabel xmlns="372b77af-8063-48a8-888c-73c0edf01dea">
-      <Value>2</Value>
-    </SipLabel>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -9506,6 +9467,23 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{268822B0-DCAE-4D2C-8340-AB7554C48D72}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="D75E00DB-06CE-4005-B397-8C0860A4229B"/>
+    <ds:schemaRef ds:uri="372b77af-8063-48a8-888c-73c0edf01dea"/>
+    <ds:schemaRef ds:uri="d75e00db-06ce-4005-b397-8c0860a4229b"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1DE4120D-B400-435F-B862-B3B8683830A5}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -9524,23 +9502,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{268822B0-DCAE-4D2C-8340-AB7554C48D72}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="D75E00DB-06CE-4005-B397-8C0860A4229B"/>
-    <ds:schemaRef ds:uri="372b77af-8063-48a8-888c-73c0edf01dea"/>
-    <ds:schemaRef ds:uri="d75e00db-06ce-4005-b397-8c0860a4229b"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2653FDDC-5C81-4B5A-A42F-7A63208AFFF7}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
BOEJ-5005: Fixing minor issues w/ templates;
</commit_message>
<xml_diff>
--- a/GenBOE/GenBOE.Web/Templates/Export/WorkspaceDataMST.xlsx
+++ b/GenBOE/GenBOE.Web/Templates/Export/WorkspaceDataMST.xlsx
@@ -5,12 +5,12 @@
   <workbookPr showPivotChartFilter="1" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ranzalon\Source\repos\IES\GenBOE\GenBOE.Web\Templates\Export\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\gitBOE\GenBOE\GenBOE.Web\Templates\Export\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE39FAC7-A498-44DA-9819-C44D307D47E9}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1EAF9FDB-E7F5-4174-B18A-3DDDB98D8D97}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3120" yWindow="345" windowWidth="18900" windowHeight="11055" firstSheet="5" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="975" yWindow="-120" windowWidth="27945" windowHeight="16440" firstSheet="5" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="BOE3 Pivot" sheetId="19" state="hidden" r:id="rId1"/>
@@ -40,7 +40,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">BOEs!$A$1:$AQ$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'BOEs (2)'!$B$1:$T$16</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'BOEs (3)'!$A$1:$N$16</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'MOQ by BOE by Task'!$A$1:$G$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'MOQ by BOE by Task'!$A$1:$F$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'MOQ Table Data'!$A$1:$O$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Resource Spreads'!$A$1:$N$2</definedName>
     <definedName name="Approvers">'[1]Options Lists'!$D$2:$D$4</definedName>
@@ -53,9 +53,9 @@
   </definedNames>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="0" r:id="rId20"/>
-    <pivotCache cacheId="1" r:id="rId21"/>
-    <pivotCache cacheId="2" r:id="rId22"/>
+    <pivotCache cacheId="3" r:id="rId20"/>
+    <pivotCache cacheId="4" r:id="rId21"/>
+    <pivotCache cacheId="5" r:id="rId22"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -320,7 +320,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="874" uniqueCount="138">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="873" uniqueCount="137">
   <si>
     <t>Start Date</t>
   </si>
@@ -701,9 +701,6 @@
   </si>
   <si>
     <t xml:space="preserve"> </t>
-  </si>
-  <si>
-    <t>Total MOQ Hours</t>
   </si>
   <si>
     <t>Table Name</t>
@@ -4336,7 +4333,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0000-000000000000}" name="PivotTable7" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="3" minRefreshableVersion="3" showCalcMbrs="0" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="3" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0000-000000000000}" name="PivotTable7" cacheId="3" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="3" minRefreshableVersion="3" showCalcMbrs="0" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="3" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
   <location ref="A3:N33" firstHeaderRow="1" firstDataRow="1" firstDataCol="14"/>
   <pivotFields count="14">
     <pivotField axis="axisRow" compact="0" outline="0" showAll="0" insertBlankRow="1" defaultSubtotal="0">
@@ -4685,7 +4682,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0200-000000000000}" name="PivotTable9" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="3" minRefreshableVersion="3" showCalcMbrs="0" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="3" indent="0" compact="0" compactData="0" multipleFieldFilters="0" rowHeaderCaption="Type">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0200-000000000000}" name="PivotTable9" cacheId="4" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="3" minRefreshableVersion="3" showCalcMbrs="0" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="3" indent="0" compact="0" compactData="0" multipleFieldFilters="0" rowHeaderCaption="Type">
   <location ref="A3:H11" firstHeaderRow="1" firstDataRow="1" firstDataCol="8"/>
   <pivotFields count="19">
     <pivotField axis="axisRow" compact="0" outline="0" showAll="0" defaultSubtotal="0">
@@ -4894,7 +4891,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0300-000000000000}" name="PivotTable4" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" missingCaption="_" updatedVersion="3" minRefreshableVersion="3" showCalcMbrs="0" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="3" indent="0" compact="0" compactData="0" multipleFieldFilters="0" rowHeaderCaption="BOE ID">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0300-000000000000}" name="PivotTable4" cacheId="5" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" missingCaption="_" updatedVersion="3" minRefreshableVersion="3" showCalcMbrs="0" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="3" indent="0" compact="0" compactData="0" multipleFieldFilters="0" rowHeaderCaption="BOE ID">
   <location ref="A3:T33" firstHeaderRow="1" firstDataRow="1" firstDataCol="20"/>
   <pivotFields count="20">
     <pivotField axis="axisRow" compact="0" outline="0" showAll="0" insertBlankRow="1" defaultSubtotal="0">
@@ -6175,18 +6172,17 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3DA6D2FB-3F32-46E9-963C-DCD2D761F967}">
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.140625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="13.28515625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="11.42578125" bestFit="1" customWidth="1"/>
     <col min="4" max="5" width="24" customWidth="1"/>
-    <col min="6" max="6" width="21.140625" customWidth="1"/>
-    <col min="7" max="7" width="40.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="40.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
         <v>70</v>
       </c>
@@ -6203,15 +6199,12 @@
         <v>119</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>127</v>
-      </c>
-      <c r="G1" s="5" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
+    <row r="2" spans="1:6" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
   </sheetData>
-  <autoFilter ref="A1:G1" xr:uid="{1E7471F8-87B8-4A9F-A5C2-80CE50F530C1}"/>
+  <autoFilter ref="A1:F1" xr:uid="{1E7471F8-87B8-4A9F-A5C2-80CE50F530C1}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -6255,34 +6248,34 @@
         <v>84</v>
       </c>
       <c r="F1" s="5" t="s">
+        <v>127</v>
+      </c>
+      <c r="G1" s="5" t="s">
         <v>128</v>
       </c>
-      <c r="G1" s="5" t="s">
+      <c r="H1" s="5" t="s">
         <v>129</v>
       </c>
-      <c r="H1" s="5" t="s">
+      <c r="I1" s="5" t="s">
         <v>130</v>
       </c>
-      <c r="I1" s="5" t="s">
+      <c r="J1" s="5" t="s">
         <v>131</v>
       </c>
-      <c r="J1" s="5" t="s">
+      <c r="K1" s="5" t="s">
         <v>132</v>
       </c>
-      <c r="K1" s="5" t="s">
+      <c r="L1" s="5" t="s">
         <v>133</v>
       </c>
-      <c r="L1" s="5" t="s">
+      <c r="M1" s="5" t="s">
         <v>134</v>
       </c>
-      <c r="M1" s="5" t="s">
+      <c r="N1" s="5" t="s">
         <v>135</v>
       </c>
-      <c r="N1" s="5" t="s">
+      <c r="O1" s="5" t="s">
         <v>136</v>
-      </c>
-      <c r="O1" s="5" t="s">
-        <v>137</v>
       </c>
     </row>
     <row r="2" spans="1:15" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
@@ -9342,16 +9335,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance">
-  <documentManagement>
-    <Unity_Description xmlns="D75E00DB-06CE-4005-B397-8C0860A4229B" xsi:nil="true"/>
-    <Unity_Tag xmlns="D75E00DB-06CE-4005-B397-8C0860A4229B" xsi:nil="true"/>
-    <Capabilities xmlns="d75e00db-06ce-4005-b397-8c0860a4229b" xsi:nil="true"/>
-    <SipLabel xmlns="372b77af-8063-48a8-888c-73c0edf01dea">
-      <Value>2</Value>
-    </SipLabel>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -9458,27 +9447,22 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance">
+  <documentManagement>
+    <Unity_Description xmlns="D75E00DB-06CE-4005-B397-8C0860A4229B" xsi:nil="true"/>
+    <Unity_Tag xmlns="D75E00DB-06CE-4005-B397-8C0860A4229B" xsi:nil="true"/>
+    <Capabilities xmlns="d75e00db-06ce-4005-b397-8c0860a4229b" xsi:nil="true"/>
+    <SipLabel xmlns="372b77af-8063-48a8-888c-73c0edf01dea">
+      <Value>2</Value>
+    </SipLabel>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{268822B0-DCAE-4D2C-8340-AB7554C48D72}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2653FDDC-5C81-4B5A-A42F-7A63208AFFF7}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="D75E00DB-06CE-4005-B397-8C0860A4229B"/>
-    <ds:schemaRef ds:uri="372b77af-8063-48a8-888c-73c0edf01dea"/>
-    <ds:schemaRef ds:uri="d75e00db-06ce-4005-b397-8c0860a4229b"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -9503,9 +9487,18 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2653FDDC-5C81-4B5A-A42F-7A63208AFFF7}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{268822B0-DCAE-4D2C-8340-AB7554C48D72}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="D75E00DB-06CE-4005-B397-8C0860A4229B"/>
+    <ds:schemaRef ds:uri="372b77af-8063-48a8-888c-73c0edf01dea"/>
+    <ds:schemaRef ds:uri="d75e00db-06ce-4005-b397-8c0860a4229b"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
4900 - Move custom fields before filters field in UI, Word Export, Excel Export
</commit_message>
<xml_diff>
--- a/GenBOE/GenBOE.Web/Templates/Export/WorkspaceDataMST.xlsx
+++ b/GenBOE/GenBOE.Web/Templates/Export/WorkspaceDataMST.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ranzalon\Source\repos\IES\GenBOE\GenBOE.Web\Templates\Export\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B136B4E5-D192-4CEF-96E3-6D3EC645AA2A}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C80882E1-1D37-4462-B8D3-2843B4CCF992}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="25080" yWindow="-120" windowWidth="25440" windowHeight="15990" firstSheet="5" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="25440" windowHeight="15390" firstSheet="5" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="BOE3 Pivot" sheetId="19" state="hidden" r:id="rId1"/>
@@ -41,7 +41,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'BOEs (2)'!$B$1:$T$16</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'BOEs (3)'!$A$1:$N$16</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'MOQ by BOE by Task'!$A$1:$F$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'MOQ Table Data'!$A$1:$P$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10">'MOQ Table Data'!$A$1:$P$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Resource Spreads'!$A$1:$N$2</definedName>
     <definedName name="Approvers">'[1]Options Lists'!$D$2:$D$4</definedName>
     <definedName name="Authors">'[1]Options Lists'!$C$2:$C$4</definedName>
@@ -6230,9 +6230,9 @@
     <col min="11" max="11" width="42" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="41.140625" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="35.28515625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="57.85546875" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="61.42578125" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="28.42578125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="28.42578125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="57.85546875" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="61.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:16" s="5" customFormat="1" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -6276,13 +6276,13 @@
         <v>134</v>
       </c>
       <c r="N1" s="5" t="s">
+        <v>137</v>
+      </c>
+      <c r="O1" s="5" t="s">
         <v>135</v>
       </c>
-      <c r="O1" s="5" t="s">
+      <c r="P1" s="5" t="s">
         <v>136</v>
-      </c>
-      <c r="P1" s="5" t="s">
-        <v>137</v>
       </c>
     </row>
     <row r="2" spans="1:16" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
@@ -9342,16 +9342,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance">
-  <documentManagement>
-    <Unity_Description xmlns="D75E00DB-06CE-4005-B397-8C0860A4229B" xsi:nil="true"/>
-    <Unity_Tag xmlns="D75E00DB-06CE-4005-B397-8C0860A4229B" xsi:nil="true"/>
-    <Capabilities xmlns="d75e00db-06ce-4005-b397-8c0860a4229b" xsi:nil="true"/>
-    <SipLabel xmlns="372b77af-8063-48a8-888c-73c0edf01dea">
-      <Value>2</Value>
-    </SipLabel>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -9458,27 +9454,22 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance">
+  <documentManagement>
+    <Unity_Description xmlns="D75E00DB-06CE-4005-B397-8C0860A4229B" xsi:nil="true"/>
+    <Unity_Tag xmlns="D75E00DB-06CE-4005-B397-8C0860A4229B" xsi:nil="true"/>
+    <Capabilities xmlns="d75e00db-06ce-4005-b397-8c0860a4229b" xsi:nil="true"/>
+    <SipLabel xmlns="372b77af-8063-48a8-888c-73c0edf01dea">
+      <Value>2</Value>
+    </SipLabel>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{268822B0-DCAE-4D2C-8340-AB7554C48D72}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2653FDDC-5C81-4B5A-A42F-7A63208AFFF7}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="D75E00DB-06CE-4005-B397-8C0860A4229B"/>
-    <ds:schemaRef ds:uri="372b77af-8063-48a8-888c-73c0edf01dea"/>
-    <ds:schemaRef ds:uri="d75e00db-06ce-4005-b397-8c0860a4229b"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -9503,9 +9494,18 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2653FDDC-5C81-4B5A-A42F-7A63208AFFF7}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{268822B0-DCAE-4D2C-8340-AB7554C48D72}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="D75E00DB-06CE-4005-B397-8C0860A4229B"/>
+    <ds:schemaRef ds:uri="372b77af-8063-48a8-888c-73c0edf01dea"/>
+    <ds:schemaRef ds:uri="d75e00db-06ce-4005-b397-8c0860a4229b"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
BOEJ-5045: Moving custom fields to the back of the spreadsheet
</commit_message>
<xml_diff>
--- a/GenBOE/GenBOE.Web/Templates/Export/WorkspaceDataMST.xlsx
+++ b/GenBOE/GenBOE.Web/Templates/Export/WorkspaceDataMST.xlsx
@@ -5,12 +5,12 @@
   <workbookPr showPivotChartFilter="1" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ranzalon\Source\repos\IES\GenBOE\GenBOE.Web\Templates\Export\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\gitBoe\GenBOE\GenBOE.Web\Templates\Export\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C80882E1-1D37-4462-B8D3-2843B4CCF992}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7CCB59E5-9CBC-49E2-B052-1CACA0BAADC3}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="25440" windowHeight="15390" firstSheet="5" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1050" yWindow="-120" windowWidth="27870" windowHeight="16440" firstSheet="5" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="BOE3 Pivot" sheetId="19" state="hidden" r:id="rId1"/>
@@ -41,7 +41,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'BOEs (2)'!$B$1:$T$16</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'BOEs (3)'!$A$1:$N$16</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'MOQ by BOE by Task'!$A$1:$F$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="10">'MOQ Table Data'!$A$1:$P$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10">'MOQ Table Data'!$A$1:$O$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Resource Spreads'!$A$1:$N$2</definedName>
     <definedName name="Approvers">'[1]Options Lists'!$D$2:$D$4</definedName>
     <definedName name="Authors">'[1]Options Lists'!$C$2:$C$4</definedName>
@@ -53,9 +53,9 @@
   </definedNames>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="0" r:id="rId20"/>
-    <pivotCache cacheId="1" r:id="rId21"/>
-    <pivotCache cacheId="2" r:id="rId22"/>
+    <pivotCache cacheId="3" r:id="rId20"/>
+    <pivotCache cacheId="4" r:id="rId21"/>
+    <pivotCache cacheId="5" r:id="rId22"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -4336,7 +4336,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0000-000000000000}" name="PivotTable7" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="3" minRefreshableVersion="3" showCalcMbrs="0" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="3" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0000-000000000000}" name="PivotTable7" cacheId="3" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="3" minRefreshableVersion="3" showCalcMbrs="0" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="3" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
   <location ref="A3:N33" firstHeaderRow="1" firstDataRow="1" firstDataCol="14"/>
   <pivotFields count="14">
     <pivotField axis="axisRow" compact="0" outline="0" showAll="0" insertBlankRow="1" defaultSubtotal="0">
@@ -4685,7 +4685,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0200-000000000000}" name="PivotTable9" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="3" minRefreshableVersion="3" showCalcMbrs="0" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="3" indent="0" compact="0" compactData="0" multipleFieldFilters="0" rowHeaderCaption="Type">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0200-000000000000}" name="PivotTable9" cacheId="4" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="3" minRefreshableVersion="3" showCalcMbrs="0" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="3" indent="0" compact="0" compactData="0" multipleFieldFilters="0" rowHeaderCaption="Type">
   <location ref="A3:H11" firstHeaderRow="1" firstDataRow="1" firstDataCol="8"/>
   <pivotFields count="19">
     <pivotField axis="axisRow" compact="0" outline="0" showAll="0" defaultSubtotal="0">
@@ -4894,7 +4894,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0300-000000000000}" name="PivotTable4" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" missingCaption="_" updatedVersion="3" minRefreshableVersion="3" showCalcMbrs="0" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="3" indent="0" compact="0" compactData="0" multipleFieldFilters="0" rowHeaderCaption="BOE ID">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0300-000000000000}" name="PivotTable4" cacheId="5" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" missingCaption="_" updatedVersion="3" minRefreshableVersion="3" showCalcMbrs="0" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="3" indent="0" compact="0" compactData="0" multipleFieldFilters="0" rowHeaderCaption="BOE ID">
   <location ref="A3:T33" firstHeaderRow="1" firstDataRow="1" firstDataCol="20"/>
   <pivotFields count="20">
     <pivotField axis="axisRow" compact="0" outline="0" showAll="0" insertBlankRow="1" defaultSubtotal="0">
@@ -6217,22 +6217,22 @@
   <dimension ref="A1:P2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.42578125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="24" customWidth="1"/>
-    <col min="5" max="5" width="42.28515625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="15.85546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="18.85546875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="28.85546875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="21.140625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="23" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="24" style="1" customWidth="1"/>
+    <col min="5" max="5" width="42.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="18.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="28.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="21.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="23" style="1" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="42" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="41.140625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="35.28515625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="28.42578125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="57.85546875" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="61.42578125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="35.28515625" style="33" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="57.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="61.42578125" style="33" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="28.42578125" style="1" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:16" s="5" customFormat="1" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -6272,22 +6272,22 @@
       <c r="L1" s="5" t="s">
         <v>133</v>
       </c>
-      <c r="M1" s="5" t="s">
+      <c r="M1" s="32" t="s">
         <v>134</v>
       </c>
       <c r="N1" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="O1" s="32" t="s">
+        <v>136</v>
+      </c>
+      <c r="P1" s="5" t="s">
         <v>137</v>
-      </c>
-      <c r="O1" s="5" t="s">
-        <v>135</v>
-      </c>
-      <c r="P1" s="5" t="s">
-        <v>136</v>
       </c>
     </row>
     <row r="2" spans="1:16" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
   </sheetData>
-  <autoFilter ref="A1:P1" xr:uid="{1ED341D2-1636-4B33-8C24-31F8903C1E1B}"/>
+  <autoFilter ref="A1:O1" xr:uid="{1ED341D2-1636-4B33-8C24-31F8903C1E1B}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -9342,12 +9342,16 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance">
+  <documentManagement>
+    <Unity_Description xmlns="D75E00DB-06CE-4005-B397-8C0860A4229B" xsi:nil="true"/>
+    <Unity_Tag xmlns="D75E00DB-06CE-4005-B397-8C0860A4229B" xsi:nil="true"/>
+    <Capabilities xmlns="d75e00db-06ce-4005-b397-8c0860a4229b" xsi:nil="true"/>
+    <SipLabel xmlns="372b77af-8063-48a8-888c-73c0edf01dea">
+      <Value>2</Value>
+    </SipLabel>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -9454,22 +9458,27 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance">
-  <documentManagement>
-    <Unity_Description xmlns="D75E00DB-06CE-4005-B397-8C0860A4229B" xsi:nil="true"/>
-    <Unity_Tag xmlns="D75E00DB-06CE-4005-B397-8C0860A4229B" xsi:nil="true"/>
-    <Capabilities xmlns="d75e00db-06ce-4005-b397-8c0860a4229b" xsi:nil="true"/>
-    <SipLabel xmlns="372b77af-8063-48a8-888c-73c0edf01dea">
-      <Value>2</Value>
-    </SipLabel>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2653FDDC-5C81-4B5A-A42F-7A63208AFFF7}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{268822B0-DCAE-4D2C-8340-AB7554C48D72}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="D75E00DB-06CE-4005-B397-8C0860A4229B"/>
+    <ds:schemaRef ds:uri="372b77af-8063-48a8-888c-73c0edf01dea"/>
+    <ds:schemaRef ds:uri="d75e00db-06ce-4005-b397-8c0860a4229b"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -9494,18 +9503,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{268822B0-DCAE-4D2C-8340-AB7554C48D72}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2653FDDC-5C81-4B5A-A42F-7A63208AFFF7}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="D75E00DB-06CE-4005-B397-8C0860A4229B"/>
-    <ds:schemaRef ds:uri="372b77af-8063-48a8-888c-73c0edf01dea"/>
-    <ds:schemaRef ds:uri="d75e00db-06ce-4005-b397-8c0860a4229b"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Update the workspace data export
</commit_message>
<xml_diff>
--- a/GenBOE/GenBOE.Web/Templates/Export/WorkspaceDataMST.xlsx
+++ b/GenBOE/GenBOE.Web/Templates/Export/WorkspaceDataMST.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24931"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25601"/>
   <workbookPr showPivotChartFilter="1" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ranzalon\Source\repos\IES\GenBOE\GenBOE.Web\Templates\Export\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\e405721\Desktop\Code-Repos\IES\GenBOE\GenBOE.Web\Templates\Export\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C63EE7C8-C81F-4A65-B93B-F47B3B8CED03}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE1FFCCF-476B-49B4-A8EB-69A7C572A320}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="25080" yWindow="-120" windowWidth="25440" windowHeight="15990" firstSheet="5" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21240" firstSheet="6" activeTab="14" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="BOE3 Pivot" sheetId="19" state="hidden" r:id="rId1"/>
@@ -320,7 +320,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="875" uniqueCount="139">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="876" uniqueCount="140">
   <si>
     <t>Start Date</t>
   </si>
@@ -737,6 +737,9 @@
   </si>
   <si>
     <t>Period of Performance (PoP): Months</t>
+  </si>
+  <si>
+    <t>SAP Connection Enabled</t>
   </si>
 </sst>
 </file>
@@ -985,7 +988,7 @@
     <xf numFmtId="0" fontId="10" fillId="6" borderId="0"/>
     <xf numFmtId="0" fontId="13" fillId="7" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="61">
+  <cellXfs count="60">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="1" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyAlignment="1">
@@ -1038,9 +1041,6 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="49" fontId="1" fillId="2" borderId="3" xfId="1" applyNumberFormat="1" applyBorder="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="1" applyNumberFormat="1">
@@ -6232,10 +6232,10 @@
     <col min="10" max="10" width="23" style="1" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="42" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="41.140625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="41.140625" style="33" customWidth="1"/>
-    <col min="14" max="14" width="35.28515625" style="33" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="41.140625" style="32" customWidth="1"/>
+    <col min="14" max="14" width="35.28515625" style="32" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="57.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="61.42578125" style="33" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="61.42578125" style="32" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="28.42578125" style="1" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -6276,16 +6276,16 @@
       <c r="L1" s="5" t="s">
         <v>133</v>
       </c>
-      <c r="M1" s="32" t="s">
+      <c r="M1" s="31" t="s">
         <v>138</v>
       </c>
-      <c r="N1" s="32" t="s">
+      <c r="N1" s="31" t="s">
         <v>134</v>
       </c>
       <c r="O1" s="5" t="s">
         <v>135</v>
       </c>
-      <c r="P1" s="32" t="s">
+      <c r="P1" s="31" t="s">
         <v>136</v>
       </c>
       <c r="Q1" s="5" t="s">
@@ -6500,11 +6500,11 @@
       </c>
     </row>
     <row r="15" spans="1:1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="20"/>
-    </row>
-    <row r="16" spans="1:1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="20"/>
-    </row>
+      <c r="A15" s="19" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -6523,206 +6523,206 @@
     <col min="5" max="5" width="12.28515625" customWidth="1"/>
     <col min="6" max="6" width="16" customWidth="1"/>
     <col min="7" max="7" width="20.5703125" customWidth="1"/>
-    <col min="8" max="8" width="10.5703125" style="40" customWidth="1"/>
-    <col min="9" max="11" width="8.85546875" style="40"/>
-    <col min="12" max="12" width="12.85546875" style="40" customWidth="1"/>
-    <col min="13" max="13" width="8.85546875" style="40"/>
-    <col min="14" max="14" width="15.5703125" style="57" customWidth="1"/>
-    <col min="15" max="15" width="19.140625" style="57" customWidth="1"/>
-    <col min="16" max="16" width="15.7109375" style="57" customWidth="1"/>
-    <col min="17" max="17" width="19.28515625" style="57" customWidth="1"/>
-    <col min="18" max="18" width="13.7109375" style="57" customWidth="1"/>
-    <col min="19" max="19" width="17.85546875" style="57" customWidth="1"/>
+    <col min="8" max="8" width="10.5703125" style="39" customWidth="1"/>
+    <col min="9" max="11" width="8.85546875" style="39"/>
+    <col min="12" max="12" width="12.85546875" style="39" customWidth="1"/>
+    <col min="13" max="13" width="8.85546875" style="39"/>
+    <col min="14" max="14" width="15.5703125" style="56" customWidth="1"/>
+    <col min="15" max="15" width="19.140625" style="56" customWidth="1"/>
+    <col min="16" max="16" width="15.7109375" style="56" customWidth="1"/>
+    <col min="17" max="17" width="19.28515625" style="56" customWidth="1"/>
+    <col min="18" max="18" width="13.7109375" style="56" customWidth="1"/>
+    <col min="19" max="19" width="17.85546875" style="56" customWidth="1"/>
     <col min="20" max="20" width="17.7109375" customWidth="1"/>
     <col min="21" max="21" width="15.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:27" s="45" customFormat="1" ht="20.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="41"/>
-      <c r="B1" s="42"/>
-      <c r="C1" s="42"/>
-      <c r="D1" s="42"/>
-      <c r="E1" s="42"/>
-      <c r="F1" s="42"/>
-      <c r="G1" s="42"/>
-      <c r="H1" s="43"/>
-      <c r="I1" s="43"/>
-      <c r="J1" s="43"/>
-      <c r="K1" s="43"/>
-      <c r="L1" s="43"/>
-      <c r="M1" s="43"/>
-      <c r="N1" s="44"/>
-      <c r="O1" s="44"/>
-      <c r="P1" s="44"/>
-      <c r="R1" s="46"/>
-      <c r="S1" s="47"/>
+    <row r="1" spans="1:27" s="44" customFormat="1" ht="20.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="40"/>
+      <c r="B1" s="41"/>
+      <c r="C1" s="41"/>
+      <c r="D1" s="41"/>
+      <c r="E1" s="41"/>
+      <c r="F1" s="41"/>
+      <c r="G1" s="41"/>
+      <c r="H1" s="42"/>
+      <c r="I1" s="42"/>
+      <c r="J1" s="42"/>
+      <c r="K1" s="42"/>
+      <c r="L1" s="42"/>
+      <c r="M1" s="42"/>
+      <c r="N1" s="43"/>
+      <c r="O1" s="43"/>
+      <c r="P1" s="43"/>
+      <c r="R1" s="45"/>
+      <c r="S1" s="46"/>
       <c r="T1"/>
-      <c r="U1" s="53"/>
-      <c r="V1" s="54"/>
-      <c r="W1" s="54"/>
-      <c r="X1" s="54"/>
-      <c r="Y1" s="54"/>
-      <c r="Z1" s="54"/>
-      <c r="AA1" s="54"/>
-    </row>
-    <row r="2" spans="1:27" s="45" customFormat="1" ht="19.5" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="41"/>
-      <c r="B2" s="42"/>
-      <c r="C2" s="42"/>
-      <c r="D2" s="42"/>
-      <c r="E2" s="42"/>
-      <c r="F2" s="42"/>
-      <c r="G2" s="42"/>
-      <c r="H2" s="43"/>
-      <c r="I2" s="43"/>
-      <c r="J2" s="43"/>
-      <c r="K2" s="43"/>
-      <c r="L2" s="43"/>
-      <c r="M2" s="43"/>
-      <c r="N2" s="44"/>
-      <c r="O2" s="44"/>
-      <c r="P2" s="44"/>
-      <c r="Q2" s="44"/>
-      <c r="R2" s="44"/>
-      <c r="S2" s="44"/>
+      <c r="U1" s="52"/>
+      <c r="V1" s="53"/>
+      <c r="W1" s="53"/>
+      <c r="X1" s="53"/>
+      <c r="Y1" s="53"/>
+      <c r="Z1" s="53"/>
+      <c r="AA1" s="53"/>
+    </row>
+    <row r="2" spans="1:27" s="44" customFormat="1" ht="19.5" thickTop="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="40"/>
+      <c r="B2" s="41"/>
+      <c r="C2" s="41"/>
+      <c r="D2" s="41"/>
+      <c r="E2" s="41"/>
+      <c r="F2" s="41"/>
+      <c r="G2" s="41"/>
+      <c r="H2" s="42"/>
+      <c r="I2" s="42"/>
+      <c r="J2" s="42"/>
+      <c r="K2" s="42"/>
+      <c r="L2" s="42"/>
+      <c r="M2" s="42"/>
+      <c r="N2" s="43"/>
+      <c r="O2" s="43"/>
+      <c r="P2" s="43"/>
+      <c r="Q2" s="43"/>
+      <c r="R2" s="43"/>
+      <c r="S2" s="43"/>
       <c r="T2"/>
-      <c r="U2" s="55"/>
-      <c r="V2" s="54"/>
-      <c r="W2" s="54"/>
-      <c r="X2" s="54"/>
-      <c r="Y2" s="54"/>
-      <c r="Z2" s="54"/>
-      <c r="AA2" s="54"/>
-    </row>
-    <row r="3" spans="1:27" s="45" customFormat="1" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A3" s="41"/>
-      <c r="B3" s="42"/>
-      <c r="C3" s="42"/>
-      <c r="D3" s="42"/>
-      <c r="E3" s="42"/>
-      <c r="F3" s="42"/>
-      <c r="G3" s="42"/>
-      <c r="H3" s="43"/>
-      <c r="I3" s="43"/>
-      <c r="J3" s="43"/>
-      <c r="K3" s="43"/>
-      <c r="L3" s="43"/>
-      <c r="M3" s="43"/>
-      <c r="N3" s="44"/>
-      <c r="O3" s="44"/>
-      <c r="P3" s="44"/>
-      <c r="Q3" s="44"/>
-      <c r="R3" s="44"/>
-      <c r="S3" s="44"/>
+      <c r="U2" s="54"/>
+      <c r="V2" s="53"/>
+      <c r="W2" s="53"/>
+      <c r="X2" s="53"/>
+      <c r="Y2" s="53"/>
+      <c r="Z2" s="53"/>
+      <c r="AA2" s="53"/>
+    </row>
+    <row r="3" spans="1:27" s="44" customFormat="1" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A3" s="40"/>
+      <c r="B3" s="41"/>
+      <c r="C3" s="41"/>
+      <c r="D3" s="41"/>
+      <c r="E3" s="41"/>
+      <c r="F3" s="41"/>
+      <c r="G3" s="41"/>
+      <c r="H3" s="42"/>
+      <c r="I3" s="42"/>
+      <c r="J3" s="42"/>
+      <c r="K3" s="42"/>
+      <c r="L3" s="42"/>
+      <c r="M3" s="42"/>
+      <c r="N3" s="43"/>
+      <c r="O3" s="43"/>
+      <c r="P3" s="43"/>
+      <c r="Q3" s="43"/>
+      <c r="R3" s="43"/>
+      <c r="S3" s="43"/>
       <c r="T3"/>
-      <c r="U3" s="55"/>
-      <c r="V3" s="54"/>
-      <c r="W3" s="54"/>
-      <c r="X3" s="54"/>
-      <c r="Y3" s="54"/>
-      <c r="Z3" s="54"/>
-      <c r="AA3" s="54"/>
-    </row>
-    <row r="4" spans="1:27" s="45" customFormat="1" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A4" s="41"/>
-      <c r="B4" s="42"/>
-      <c r="C4" s="42"/>
-      <c r="D4" s="42"/>
-      <c r="E4" s="42"/>
-      <c r="F4" s="42"/>
-      <c r="G4" s="42"/>
-      <c r="H4" s="43"/>
-      <c r="I4" s="43"/>
-      <c r="J4" s="43"/>
-      <c r="K4" s="43"/>
-      <c r="L4" s="43"/>
-      <c r="M4" s="43"/>
-      <c r="N4" s="44"/>
-      <c r="O4" s="44"/>
-      <c r="P4" s="44"/>
-      <c r="Q4" s="44"/>
-      <c r="R4" s="44"/>
-      <c r="S4" s="44"/>
+      <c r="U3" s="54"/>
+      <c r="V3" s="53"/>
+      <c r="W3" s="53"/>
+      <c r="X3" s="53"/>
+      <c r="Y3" s="53"/>
+      <c r="Z3" s="53"/>
+      <c r="AA3" s="53"/>
+    </row>
+    <row r="4" spans="1:27" s="44" customFormat="1" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A4" s="40"/>
+      <c r="B4" s="41"/>
+      <c r="C4" s="41"/>
+      <c r="D4" s="41"/>
+      <c r="E4" s="41"/>
+      <c r="F4" s="41"/>
+      <c r="G4" s="41"/>
+      <c r="H4" s="42"/>
+      <c r="I4" s="42"/>
+      <c r="J4" s="42"/>
+      <c r="K4" s="42"/>
+      <c r="L4" s="42"/>
+      <c r="M4" s="42"/>
+      <c r="N4" s="43"/>
+      <c r="O4" s="43"/>
+      <c r="P4" s="43"/>
+      <c r="Q4" s="43"/>
+      <c r="R4" s="43"/>
+      <c r="S4" s="43"/>
       <c r="T4"/>
-      <c r="U4" s="55"/>
-      <c r="V4" s="54"/>
-      <c r="W4" s="54"/>
-      <c r="X4" s="54"/>
-      <c r="Y4" s="54"/>
-      <c r="Z4" s="54"/>
-      <c r="AA4" s="54"/>
-    </row>
-    <row r="5" spans="1:27" s="45" customFormat="1" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A5" s="55"/>
-      <c r="B5" s="42"/>
-      <c r="C5" s="42"/>
-      <c r="D5" s="42"/>
-      <c r="E5" s="42"/>
-      <c r="F5" s="42"/>
-      <c r="G5" s="42"/>
-      <c r="H5" s="43"/>
-      <c r="I5" s="43"/>
-      <c r="J5" s="43"/>
-      <c r="K5" s="43"/>
-      <c r="L5" s="43"/>
-      <c r="M5" s="43"/>
-      <c r="N5" s="44"/>
-      <c r="O5" s="44"/>
-      <c r="P5" s="44"/>
-      <c r="Q5" s="44"/>
-      <c r="R5" s="44"/>
-      <c r="S5" s="44"/>
+      <c r="U4" s="54"/>
+      <c r="V4" s="53"/>
+      <c r="W4" s="53"/>
+      <c r="X4" s="53"/>
+      <c r="Y4" s="53"/>
+      <c r="Z4" s="53"/>
+      <c r="AA4" s="53"/>
+    </row>
+    <row r="5" spans="1:27" s="44" customFormat="1" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A5" s="54"/>
+      <c r="B5" s="41"/>
+      <c r="C5" s="41"/>
+      <c r="D5" s="41"/>
+      <c r="E5" s="41"/>
+      <c r="F5" s="41"/>
+      <c r="G5" s="41"/>
+      <c r="H5" s="42"/>
+      <c r="I5" s="42"/>
+      <c r="J5" s="42"/>
+      <c r="K5" s="42"/>
+      <c r="L5" s="42"/>
+      <c r="M5" s="42"/>
+      <c r="N5" s="43"/>
+      <c r="O5" s="43"/>
+      <c r="P5" s="43"/>
+      <c r="Q5" s="43"/>
+      <c r="R5" s="43"/>
+      <c r="S5" s="43"/>
       <c r="T5"/>
-      <c r="U5" s="55"/>
-      <c r="V5" s="54"/>
-      <c r="W5" s="54"/>
-      <c r="X5" s="54"/>
-      <c r="Y5" s="54"/>
-      <c r="Z5" s="54"/>
-      <c r="AA5" s="54"/>
-    </row>
-    <row r="6" spans="1:27" s="45" customFormat="1" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A6" s="55"/>
-      <c r="B6" s="56"/>
-      <c r="C6" s="56"/>
-      <c r="D6" s="56"/>
-      <c r="E6" s="56"/>
-      <c r="F6" s="56"/>
-      <c r="G6" s="56"/>
-      <c r="H6" s="43"/>
-      <c r="I6" s="43"/>
-      <c r="J6" s="43"/>
-      <c r="K6" s="43"/>
-      <c r="L6" s="43"/>
-      <c r="M6" s="43"/>
-      <c r="N6" s="44"/>
-      <c r="O6" s="44"/>
-      <c r="P6" s="44"/>
-      <c r="Q6" s="44"/>
-      <c r="R6" s="44"/>
-      <c r="S6" s="44"/>
+      <c r="U5" s="54"/>
+      <c r="V5" s="53"/>
+      <c r="W5" s="53"/>
+      <c r="X5" s="53"/>
+      <c r="Y5" s="53"/>
+      <c r="Z5" s="53"/>
+      <c r="AA5" s="53"/>
+    </row>
+    <row r="6" spans="1:27" s="44" customFormat="1" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A6" s="54"/>
+      <c r="B6" s="55"/>
+      <c r="C6" s="55"/>
+      <c r="D6" s="55"/>
+      <c r="E6" s="55"/>
+      <c r="F6" s="55"/>
+      <c r="G6" s="55"/>
+      <c r="H6" s="42"/>
+      <c r="I6" s="42"/>
+      <c r="J6" s="42"/>
+      <c r="K6" s="42"/>
+      <c r="L6" s="42"/>
+      <c r="M6" s="42"/>
+      <c r="N6" s="43"/>
+      <c r="O6" s="43"/>
+      <c r="P6" s="43"/>
+      <c r="Q6" s="43"/>
+      <c r="R6" s="43"/>
+      <c r="S6" s="43"/>
       <c r="T6"/>
-      <c r="U6" s="55"/>
-      <c r="V6" s="54"/>
-      <c r="W6" s="54"/>
-      <c r="X6" s="54"/>
-      <c r="Y6" s="54"/>
-      <c r="Z6" s="54"/>
-      <c r="AA6" s="54"/>
-    </row>
-    <row r="7" spans="1:27" s="55" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="H7" s="43"/>
-      <c r="I7" s="43"/>
-      <c r="J7" s="43"/>
-      <c r="K7" s="43"/>
-      <c r="L7" s="43"/>
-      <c r="M7" s="43"/>
-      <c r="N7" s="44"/>
-      <c r="O7" s="44"/>
-      <c r="P7" s="44"/>
-      <c r="Q7" s="44"/>
-      <c r="R7" s="44"/>
-      <c r="S7" s="44" t="s">
+      <c r="U6" s="54"/>
+      <c r="V6" s="53"/>
+      <c r="W6" s="53"/>
+      <c r="X6" s="53"/>
+      <c r="Y6" s="53"/>
+      <c r="Z6" s="53"/>
+      <c r="AA6" s="53"/>
+    </row>
+    <row r="7" spans="1:27" s="54" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="H7" s="42"/>
+      <c r="I7" s="42"/>
+      <c r="J7" s="42"/>
+      <c r="K7" s="42"/>
+      <c r="L7" s="42"/>
+      <c r="M7" s="42"/>
+      <c r="N7" s="43"/>
+      <c r="O7" s="43"/>
+      <c r="P7" s="43"/>
+      <c r="Q7" s="43"/>
+      <c r="R7" s="43"/>
+      <c r="S7" s="43" t="s">
         <v>126</v>
       </c>
       <c r="T7"/>
@@ -6737,199 +6737,199 @@
   <dimension ref="A1:AA6"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.7109375" style="58" customWidth="1"/>
-    <col min="2" max="2" width="7.140625" style="58" customWidth="1"/>
-    <col min="3" max="3" width="29.42578125" style="58" customWidth="1"/>
-    <col min="4" max="4" width="26.85546875" style="58" customWidth="1"/>
-    <col min="5" max="5" width="12.28515625" style="58" customWidth="1"/>
-    <col min="6" max="6" width="16" style="58" customWidth="1"/>
-    <col min="7" max="7" width="20.5703125" style="58" customWidth="1"/>
-    <col min="8" max="8" width="10.5703125" style="59" customWidth="1"/>
-    <col min="9" max="13" width="9.140625" style="59"/>
-    <col min="14" max="14" width="15.5703125" style="57" customWidth="1"/>
-    <col min="15" max="15" width="24.5703125" style="57" customWidth="1"/>
-    <col min="16" max="16" width="15.7109375" style="57" customWidth="1"/>
-    <col min="17" max="17" width="19.28515625" style="57" customWidth="1"/>
-    <col min="18" max="18" width="13.7109375" style="57" customWidth="1"/>
-    <col min="19" max="19" width="17.85546875" style="57" customWidth="1"/>
-    <col min="20" max="20" width="17.7109375" style="57" customWidth="1"/>
-    <col min="21" max="21" width="15.28515625" style="57" customWidth="1"/>
-    <col min="22" max="16384" width="9.140625" style="60"/>
+    <col min="1" max="1" width="11.7109375" style="57" customWidth="1"/>
+    <col min="2" max="2" width="7.140625" style="57" customWidth="1"/>
+    <col min="3" max="3" width="29.42578125" style="57" customWidth="1"/>
+    <col min="4" max="4" width="26.85546875" style="57" customWidth="1"/>
+    <col min="5" max="5" width="12.28515625" style="57" customWidth="1"/>
+    <col min="6" max="6" width="16" style="57" customWidth="1"/>
+    <col min="7" max="7" width="20.5703125" style="57" customWidth="1"/>
+    <col min="8" max="8" width="10.5703125" style="58" customWidth="1"/>
+    <col min="9" max="13" width="9.140625" style="58"/>
+    <col min="14" max="14" width="15.5703125" style="56" customWidth="1"/>
+    <col min="15" max="15" width="24.5703125" style="56" customWidth="1"/>
+    <col min="16" max="16" width="15.7109375" style="56" customWidth="1"/>
+    <col min="17" max="17" width="19.28515625" style="56" customWidth="1"/>
+    <col min="18" max="18" width="13.7109375" style="56" customWidth="1"/>
+    <col min="19" max="19" width="17.85546875" style="56" customWidth="1"/>
+    <col min="20" max="20" width="17.7109375" style="56" customWidth="1"/>
+    <col min="21" max="21" width="15.28515625" style="56" customWidth="1"/>
+    <col min="22" max="16384" width="9.140625" style="59"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:27" s="52" customFormat="1" ht="20.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="42"/>
-      <c r="B1" s="42"/>
-      <c r="C1" s="42"/>
-      <c r="D1" s="42"/>
-      <c r="E1" s="42"/>
-      <c r="F1" s="42"/>
-      <c r="G1" s="42"/>
-      <c r="H1" s="48"/>
-      <c r="I1" s="48"/>
-      <c r="J1" s="48"/>
-      <c r="K1" s="48"/>
-      <c r="L1" s="48"/>
-      <c r="M1" s="48"/>
-      <c r="N1" s="44"/>
-      <c r="O1" s="44"/>
-      <c r="P1" s="44"/>
-      <c r="Q1" s="44"/>
-      <c r="R1" s="49"/>
-      <c r="S1" s="44"/>
-      <c r="T1" s="46"/>
-      <c r="U1" s="50"/>
-      <c r="V1" s="51"/>
-      <c r="W1" s="51"/>
-      <c r="X1" s="51"/>
-      <c r="Y1" s="51"/>
-      <c r="Z1" s="51"/>
-      <c r="AA1" s="51"/>
-    </row>
-    <row r="2" spans="1:27" s="52" customFormat="1" ht="19.5" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="42"/>
-      <c r="B2" s="42"/>
-      <c r="C2" s="42"/>
-      <c r="D2" s="42"/>
-      <c r="E2" s="42"/>
-      <c r="F2" s="42"/>
-      <c r="G2" s="42"/>
-      <c r="H2" s="48"/>
-      <c r="I2" s="48"/>
-      <c r="J2" s="48"/>
-      <c r="K2" s="48"/>
-      <c r="L2" s="48"/>
-      <c r="M2" s="48"/>
-      <c r="N2" s="44"/>
-      <c r="O2" s="44"/>
-      <c r="P2" s="44"/>
-      <c r="Q2" s="44"/>
-      <c r="R2" s="44"/>
-      <c r="S2" s="44"/>
-      <c r="T2" s="44"/>
-      <c r="U2" s="44"/>
-      <c r="V2" s="51"/>
-      <c r="W2" s="51"/>
-      <c r="X2" s="51"/>
-      <c r="Y2" s="51"/>
-      <c r="Z2" s="51"/>
-      <c r="AA2" s="51"/>
-    </row>
-    <row r="3" spans="1:27" s="52" customFormat="1" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A3" s="42"/>
-      <c r="B3" s="42"/>
-      <c r="C3" s="42"/>
-      <c r="D3" s="42"/>
-      <c r="E3" s="42"/>
-      <c r="F3" s="42"/>
-      <c r="G3" s="42"/>
-      <c r="H3" s="48"/>
-      <c r="I3" s="48"/>
-      <c r="J3" s="48"/>
-      <c r="K3" s="48"/>
-      <c r="L3" s="48"/>
-      <c r="M3" s="48"/>
-      <c r="N3" s="44"/>
-      <c r="O3" s="44"/>
-      <c r="P3" s="44"/>
-      <c r="Q3" s="44"/>
-      <c r="R3" s="44"/>
-      <c r="S3" s="44"/>
-      <c r="T3" s="44"/>
-      <c r="U3" s="44"/>
-      <c r="V3" s="51"/>
-      <c r="W3" s="51"/>
-      <c r="X3" s="51"/>
-      <c r="Y3" s="51"/>
-      <c r="Z3" s="51"/>
-      <c r="AA3" s="51"/>
-    </row>
-    <row r="4" spans="1:27" s="52" customFormat="1" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A4" s="42"/>
-      <c r="B4" s="42"/>
-      <c r="C4" s="42"/>
-      <c r="D4" s="42"/>
-      <c r="E4" s="42"/>
-      <c r="F4" s="42"/>
-      <c r="G4" s="42"/>
-      <c r="H4" s="48"/>
-      <c r="I4" s="48"/>
-      <c r="J4" s="48"/>
-      <c r="K4" s="48"/>
-      <c r="L4" s="48"/>
-      <c r="M4" s="48"/>
-      <c r="N4" s="44"/>
-      <c r="O4" s="44"/>
-      <c r="P4" s="44"/>
-      <c r="Q4" s="44"/>
-      <c r="R4" s="44"/>
-      <c r="S4" s="44"/>
-      <c r="T4" s="44"/>
-      <c r="U4" s="44"/>
-      <c r="V4" s="51"/>
-      <c r="W4" s="51"/>
-      <c r="X4" s="51"/>
-      <c r="Y4" s="51"/>
-      <c r="Z4" s="51"/>
-      <c r="AA4" s="51"/>
-    </row>
-    <row r="5" spans="1:27" s="52" customFormat="1" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A5" s="42"/>
-      <c r="B5" s="42"/>
-      <c r="C5" s="42"/>
-      <c r="D5" s="42"/>
-      <c r="E5" s="42"/>
-      <c r="F5" s="42"/>
-      <c r="G5" s="42"/>
-      <c r="H5" s="48"/>
-      <c r="I5" s="48"/>
-      <c r="J5" s="48"/>
-      <c r="K5" s="48"/>
-      <c r="L5" s="48"/>
-      <c r="M5" s="48"/>
-      <c r="N5" s="44"/>
-      <c r="O5" s="44"/>
-      <c r="P5" s="44"/>
-      <c r="Q5" s="44"/>
-      <c r="R5" s="44"/>
-      <c r="S5" s="44"/>
-      <c r="T5" s="44"/>
-      <c r="U5" s="44"/>
-      <c r="V5" s="51"/>
-      <c r="W5" s="51"/>
-      <c r="X5" s="51"/>
-      <c r="Y5" s="51"/>
-      <c r="Z5" s="51"/>
-      <c r="AA5" s="51"/>
-    </row>
-    <row r="6" spans="1:27" s="45" customFormat="1" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A6" s="56"/>
-      <c r="B6" s="56"/>
-      <c r="C6" s="56"/>
-      <c r="D6" s="56"/>
-      <c r="E6" s="56"/>
-      <c r="F6" s="56"/>
-      <c r="G6" s="56"/>
-      <c r="H6" s="43"/>
-      <c r="I6" s="43"/>
-      <c r="J6" s="43"/>
-      <c r="K6" s="43"/>
-      <c r="L6" s="43"/>
-      <c r="M6" s="43"/>
-      <c r="N6" s="44"/>
-      <c r="O6" s="44"/>
-      <c r="P6" s="44"/>
-      <c r="Q6" s="44"/>
-      <c r="R6" s="44"/>
-      <c r="S6" s="44"/>
-      <c r="T6" s="44"/>
-      <c r="U6" s="44"/>
-      <c r="V6" s="54"/>
-      <c r="W6" s="54"/>
-      <c r="X6" s="54"/>
-      <c r="Y6" s="54"/>
-      <c r="Z6" s="54"/>
-      <c r="AA6" s="54"/>
+    <row r="1" spans="1:27" s="51" customFormat="1" ht="20.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="41"/>
+      <c r="B1" s="41"/>
+      <c r="C1" s="41"/>
+      <c r="D1" s="41"/>
+      <c r="E1" s="41"/>
+      <c r="F1" s="41"/>
+      <c r="G1" s="41"/>
+      <c r="H1" s="47"/>
+      <c r="I1" s="47"/>
+      <c r="J1" s="47"/>
+      <c r="K1" s="47"/>
+      <c r="L1" s="47"/>
+      <c r="M1" s="47"/>
+      <c r="N1" s="43"/>
+      <c r="O1" s="43"/>
+      <c r="P1" s="43"/>
+      <c r="Q1" s="43"/>
+      <c r="R1" s="48"/>
+      <c r="S1" s="43"/>
+      <c r="T1" s="45"/>
+      <c r="U1" s="49"/>
+      <c r="V1" s="50"/>
+      <c r="W1" s="50"/>
+      <c r="X1" s="50"/>
+      <c r="Y1" s="50"/>
+      <c r="Z1" s="50"/>
+      <c r="AA1" s="50"/>
+    </row>
+    <row r="2" spans="1:27" s="51" customFormat="1" ht="19.5" thickTop="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="41"/>
+      <c r="B2" s="41"/>
+      <c r="C2" s="41"/>
+      <c r="D2" s="41"/>
+      <c r="E2" s="41"/>
+      <c r="F2" s="41"/>
+      <c r="G2" s="41"/>
+      <c r="H2" s="47"/>
+      <c r="I2" s="47"/>
+      <c r="J2" s="47"/>
+      <c r="K2" s="47"/>
+      <c r="L2" s="47"/>
+      <c r="M2" s="47"/>
+      <c r="N2" s="43"/>
+      <c r="O2" s="43"/>
+      <c r="P2" s="43"/>
+      <c r="Q2" s="43"/>
+      <c r="R2" s="43"/>
+      <c r="S2" s="43"/>
+      <c r="T2" s="43"/>
+      <c r="U2" s="43"/>
+      <c r="V2" s="50"/>
+      <c r="W2" s="50"/>
+      <c r="X2" s="50"/>
+      <c r="Y2" s="50"/>
+      <c r="Z2" s="50"/>
+      <c r="AA2" s="50"/>
+    </row>
+    <row r="3" spans="1:27" s="51" customFormat="1" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A3" s="41"/>
+      <c r="B3" s="41"/>
+      <c r="C3" s="41"/>
+      <c r="D3" s="41"/>
+      <c r="E3" s="41"/>
+      <c r="F3" s="41"/>
+      <c r="G3" s="41"/>
+      <c r="H3" s="47"/>
+      <c r="I3" s="47"/>
+      <c r="J3" s="47"/>
+      <c r="K3" s="47"/>
+      <c r="L3" s="47"/>
+      <c r="M3" s="47"/>
+      <c r="N3" s="43"/>
+      <c r="O3" s="43"/>
+      <c r="P3" s="43"/>
+      <c r="Q3" s="43"/>
+      <c r="R3" s="43"/>
+      <c r="S3" s="43"/>
+      <c r="T3" s="43"/>
+      <c r="U3" s="43"/>
+      <c r="V3" s="50"/>
+      <c r="W3" s="50"/>
+      <c r="X3" s="50"/>
+      <c r="Y3" s="50"/>
+      <c r="Z3" s="50"/>
+      <c r="AA3" s="50"/>
+    </row>
+    <row r="4" spans="1:27" s="51" customFormat="1" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A4" s="41"/>
+      <c r="B4" s="41"/>
+      <c r="C4" s="41"/>
+      <c r="D4" s="41"/>
+      <c r="E4" s="41"/>
+      <c r="F4" s="41"/>
+      <c r="G4" s="41"/>
+      <c r="H4" s="47"/>
+      <c r="I4" s="47"/>
+      <c r="J4" s="47"/>
+      <c r="K4" s="47"/>
+      <c r="L4" s="47"/>
+      <c r="M4" s="47"/>
+      <c r="N4" s="43"/>
+      <c r="O4" s="43"/>
+      <c r="P4" s="43"/>
+      <c r="Q4" s="43"/>
+      <c r="R4" s="43"/>
+      <c r="S4" s="43"/>
+      <c r="T4" s="43"/>
+      <c r="U4" s="43"/>
+      <c r="V4" s="50"/>
+      <c r="W4" s="50"/>
+      <c r="X4" s="50"/>
+      <c r="Y4" s="50"/>
+      <c r="Z4" s="50"/>
+      <c r="AA4" s="50"/>
+    </row>
+    <row r="5" spans="1:27" s="51" customFormat="1" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A5" s="41"/>
+      <c r="B5" s="41"/>
+      <c r="C5" s="41"/>
+      <c r="D5" s="41"/>
+      <c r="E5" s="41"/>
+      <c r="F5" s="41"/>
+      <c r="G5" s="41"/>
+      <c r="H5" s="47"/>
+      <c r="I5" s="47"/>
+      <c r="J5" s="47"/>
+      <c r="K5" s="47"/>
+      <c r="L5" s="47"/>
+      <c r="M5" s="47"/>
+      <c r="N5" s="43"/>
+      <c r="O5" s="43"/>
+      <c r="P5" s="43"/>
+      <c r="Q5" s="43"/>
+      <c r="R5" s="43"/>
+      <c r="S5" s="43"/>
+      <c r="T5" s="43"/>
+      <c r="U5" s="43"/>
+      <c r="V5" s="50"/>
+      <c r="W5" s="50"/>
+      <c r="X5" s="50"/>
+      <c r="Y5" s="50"/>
+      <c r="Z5" s="50"/>
+      <c r="AA5" s="50"/>
+    </row>
+    <row r="6" spans="1:27" s="44" customFormat="1" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A6" s="55"/>
+      <c r="B6" s="55"/>
+      <c r="C6" s="55"/>
+      <c r="D6" s="55"/>
+      <c r="E6" s="55"/>
+      <c r="F6" s="55"/>
+      <c r="G6" s="55"/>
+      <c r="H6" s="42"/>
+      <c r="I6" s="42"/>
+      <c r="J6" s="42"/>
+      <c r="K6" s="42"/>
+      <c r="L6" s="42"/>
+      <c r="M6" s="42"/>
+      <c r="N6" s="43"/>
+      <c r="O6" s="43"/>
+      <c r="P6" s="43"/>
+      <c r="Q6" s="43"/>
+      <c r="R6" s="43"/>
+      <c r="S6" s="43"/>
+      <c r="T6" s="43"/>
+      <c r="U6" s="43"/>
+      <c r="V6" s="53"/>
+      <c r="W6" s="53"/>
+      <c r="X6" s="53"/>
+      <c r="Y6" s="53"/>
+      <c r="Z6" s="53"/>
+      <c r="AA6" s="53"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -8857,19 +8857,19 @@
     <col min="12" max="12" width="19.7109375" style="1" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="10.5703125" style="1" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="13.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="13.42578125" style="38" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="12.5703125" style="38" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="13.42578125" style="37" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="12.5703125" style="37" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="21.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="20.140625" style="33" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="18.7109375" style="31" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="20.140625" style="32" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="18.7109375" style="30" bestFit="1" customWidth="1"/>
     <col min="20" max="20" width="17.140625" style="1" bestFit="1" customWidth="1"/>
     <col min="21" max="21" width="20.28515625" style="1" bestFit="1" customWidth="1"/>
     <col min="22" max="22" width="21.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="13.7109375" style="38" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="12.85546875" style="38" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="13.7109375" style="37" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="12.85546875" style="37" bestFit="1" customWidth="1"/>
     <col min="25" max="25" width="21.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="20.42578125" style="33" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="19" style="31" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="20.42578125" style="32" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="19" style="30" bestFit="1" customWidth="1"/>
     <col min="28" max="28" width="20" style="1" bestFit="1" customWidth="1"/>
     <col min="29" max="29" width="24.7109375" style="1" bestFit="1" customWidth="1"/>
     <col min="30" max="30" width="18.28515625" style="1" bestFit="1" customWidth="1"/>
@@ -8877,14 +8877,14 @@
     <col min="32" max="32" width="18.85546875" style="1" bestFit="1" customWidth="1"/>
     <col min="33" max="33" width="23.85546875" style="1" bestFit="1" customWidth="1"/>
     <col min="34" max="34" width="16.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="35" max="35" width="13" style="35" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="17" style="33" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="15.7109375" style="31" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="13" style="34" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="17" style="32" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="15.7109375" style="30" bestFit="1" customWidth="1"/>
     <col min="38" max="38" width="26.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="39" max="39" width="8.7109375" style="40" customWidth="1"/>
-    <col min="40" max="40" width="10.5703125" style="40" bestFit="1" customWidth="1"/>
-    <col min="41" max="41" width="10" style="33" bestFit="1" customWidth="1"/>
-    <col min="42" max="42" width="8.7109375" style="31" customWidth="1"/>
+    <col min="39" max="39" width="8.7109375" style="39" customWidth="1"/>
+    <col min="40" max="40" width="10.5703125" style="39" bestFit="1" customWidth="1"/>
+    <col min="41" max="41" width="10" style="32" bestFit="1" customWidth="1"/>
+    <col min="42" max="42" width="8.7109375" style="30" customWidth="1"/>
     <col min="43" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
@@ -8931,19 +8931,19 @@
       <c r="N1" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="O1" s="37" t="s">
+      <c r="O1" s="36" t="s">
         <v>31</v>
       </c>
-      <c r="P1" s="37" t="s">
+      <c r="P1" s="36" t="s">
         <v>32</v>
       </c>
       <c r="Q1" s="5" t="s">
         <v>94</v>
       </c>
-      <c r="R1" s="32" t="s">
+      <c r="R1" s="31" t="s">
         <v>86</v>
       </c>
-      <c r="S1" s="26" t="s">
+      <c r="S1" s="25" t="s">
         <v>100</v>
       </c>
       <c r="T1" s="5" t="s">
@@ -8955,19 +8955,19 @@
       <c r="V1" s="5" t="s">
         <v>92</v>
       </c>
-      <c r="W1" s="37" t="s">
+      <c r="W1" s="36" t="s">
         <v>4</v>
       </c>
-      <c r="X1" s="37" t="s">
+      <c r="X1" s="36" t="s">
         <v>5</v>
       </c>
       <c r="Y1" s="5" t="s">
         <v>95</v>
       </c>
-      <c r="Z1" s="32" t="s">
+      <c r="Z1" s="31" t="s">
         <v>85</v>
       </c>
-      <c r="AA1" s="26" t="s">
+      <c r="AA1" s="25" t="s">
         <v>102</v>
       </c>
       <c r="AB1" s="5" t="s">
@@ -8991,28 +8991,28 @@
       <c r="AH1" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="AI1" s="34" t="s">
+      <c r="AI1" s="33" t="s">
         <v>14</v>
       </c>
-      <c r="AJ1" s="32" t="s">
+      <c r="AJ1" s="31" t="s">
         <v>15</v>
       </c>
-      <c r="AK1" s="26" t="s">
+      <c r="AK1" s="25" t="s">
         <v>109</v>
       </c>
       <c r="AL1" s="5" t="s">
         <v>99</v>
       </c>
-      <c r="AM1" s="39" t="s">
+      <c r="AM1" s="38" t="s">
         <v>90</v>
       </c>
-      <c r="AN1" s="39" t="s">
+      <c r="AN1" s="38" t="s">
         <v>91</v>
       </c>
-      <c r="AO1" s="36" t="s">
+      <c r="AO1" s="35" t="s">
         <v>110</v>
       </c>
-      <c r="AP1" s="29" t="s">
+      <c r="AP1" s="28" t="s">
         <v>111</v>
       </c>
     </row>
@@ -9038,8 +9038,8 @@
     <col min="8" max="8" width="13.42578125" style="3" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="12.5703125" style="3" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="21.42578125" style="3" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="20.140625" style="22" bestFit="1" customWidth="1"/>
-    <col min="12" max="13" width="20.140625" style="27" customWidth="1"/>
+    <col min="11" max="11" width="20.140625" style="21" bestFit="1" customWidth="1"/>
+    <col min="12" max="13" width="20.140625" style="26" customWidth="1"/>
     <col min="14" max="14" width="20.140625" style="3" customWidth="1"/>
     <col min="15" max="15" width="11.42578125" style="3" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="13.5703125" style="3" bestFit="1" customWidth="1"/>
@@ -9051,8 +9051,8 @@
     <col min="22" max="22" width="13.7109375" style="3" bestFit="1" customWidth="1"/>
     <col min="23" max="23" width="12.85546875" style="3" bestFit="1" customWidth="1"/>
     <col min="24" max="24" width="21.7109375" style="3" customWidth="1"/>
-    <col min="25" max="25" width="20.42578125" style="22" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="20.42578125" style="27" customWidth="1"/>
+    <col min="25" max="25" width="20.42578125" style="21" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="20.42578125" style="26" customWidth="1"/>
     <col min="27" max="27" width="20.42578125" style="3" customWidth="1"/>
     <col min="28" max="28" width="24.7109375" style="3" bestFit="1" customWidth="1"/>
     <col min="29" max="31" width="24.7109375" style="3" customWidth="1"/>
@@ -9062,8 +9062,8 @@
     <col min="38" max="38" width="13" style="3" bestFit="1" customWidth="1"/>
     <col min="39" max="39" width="16.85546875" style="3" bestFit="1" customWidth="1"/>
     <col min="40" max="40" width="13" style="18" bestFit="1" customWidth="1"/>
-    <col min="41" max="41" width="13" style="22" customWidth="1"/>
-    <col min="42" max="42" width="17" style="27" bestFit="1" customWidth="1"/>
+    <col min="41" max="41" width="13" style="21" customWidth="1"/>
+    <col min="42" max="42" width="17" style="26" bestFit="1" customWidth="1"/>
     <col min="43" max="43" width="24.85546875" style="3" bestFit="1" customWidth="1"/>
     <col min="44" max="16384" width="9.140625" style="3"/>
   </cols>
@@ -9099,13 +9099,13 @@
       <c r="J1" s="5" t="s">
         <v>94</v>
       </c>
-      <c r="K1" s="21" t="s">
+      <c r="K1" s="20" t="s">
         <v>86</v>
       </c>
-      <c r="L1" s="26" t="s">
+      <c r="L1" s="25" t="s">
         <v>100</v>
       </c>
-      <c r="M1" s="26" t="s">
+      <c r="M1" s="25" t="s">
         <v>124</v>
       </c>
       <c r="N1" s="5" t="s">
@@ -9141,10 +9141,10 @@
       <c r="X1" s="5" t="s">
         <v>95</v>
       </c>
-      <c r="Y1" s="21" t="s">
+      <c r="Y1" s="20" t="s">
         <v>85</v>
       </c>
-      <c r="Z1" s="26" t="s">
+      <c r="Z1" s="25" t="s">
         <v>102</v>
       </c>
       <c r="AA1" s="5" t="s">
@@ -9189,10 +9189,10 @@
       <c r="AN1" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="AO1" s="21" t="s">
+      <c r="AO1" s="20" t="s">
         <v>15</v>
       </c>
-      <c r="AP1" s="26" t="s">
+      <c r="AP1" s="25" t="s">
         <v>109</v>
       </c>
       <c r="AQ1" s="5" t="s">
@@ -9218,8 +9218,8 @@
     <col min="4" max="4" width="20.7109375" style="7" customWidth="1"/>
     <col min="5" max="5" width="25.7109375" style="7" customWidth="1"/>
     <col min="6" max="7" width="15.7109375" style="7" customWidth="1"/>
-    <col min="8" max="8" width="13.140625" style="23" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.140625" style="28" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.140625" style="22" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13.140625" style="27" bestFit="1" customWidth="1"/>
     <col min="10" max="11" width="25.7109375" style="7" customWidth="1"/>
     <col min="12" max="13" width="15.42578125" style="7" customWidth="1"/>
     <col min="14" max="14" width="11" style="7" customWidth="1"/>
@@ -9248,10 +9248,10 @@
       <c r="G1" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="H1" s="21" t="s">
+      <c r="H1" s="20" t="s">
         <v>6</v>
       </c>
-      <c r="I1" s="26" t="s">
+      <c r="I1" s="25" t="s">
         <v>113</v>
       </c>
       <c r="J1" s="9" t="s">
@@ -9292,8 +9292,8 @@
     <col min="9" max="9" width="18.140625" style="16" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="18.85546875" style="16" bestFit="1" customWidth="1"/>
     <col min="11" max="12" width="10.7109375" style="17" customWidth="1"/>
-    <col min="13" max="13" width="20.7109375" style="25" customWidth="1"/>
-    <col min="14" max="14" width="20.7109375" style="30" customWidth="1"/>
+    <col min="13" max="13" width="20.7109375" style="24" customWidth="1"/>
+    <col min="14" max="14" width="20.7109375" style="29" customWidth="1"/>
     <col min="15" max="16384" width="9.140625" style="16"/>
   </cols>
   <sheetData>
@@ -9334,10 +9334,10 @@
       <c r="L1" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="M1" s="24" t="s">
+      <c r="M1" s="23" t="s">
         <v>110</v>
       </c>
-      <c r="N1" s="29" t="s">
+      <c r="N1" s="28" t="s">
         <v>111</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Merged PR 1136: ACV-226: Add Source to MOQ Table Data in Workspace Data Report
Added the Source Column to the MOQ Table Data in Workspace Data Report Export.

**This change is only needed for RMS.**

Screenshot:
![sourceadded.png](https://idetfs01/Estimating/ec33f0ce-06e6-4674-9d97-643c8eb6e517/_apis/git/repositories/c962790d-14a5-4524-9fe8-35b4cce33cc3/pullRequests/1136/attachments/sourceadded.png)
</commit_message>
<xml_diff>
--- a/GenBOE/GenBOE.Web/Templates/Export/WorkspaceDataMST.xlsx
+++ b/GenBOE/GenBOE.Web/Templates/Export/WorkspaceDataMST.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\e405721\Desktop\Code-Repos\IES\GenBOE\GenBOE.Web\Templates\Export\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE1FFCCF-476B-49B4-A8EB-69A7C572A320}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C0A9B38D-3E45-4BE5-83D1-9441DA857D8F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21240" firstSheet="6" activeTab="14" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="3825" windowWidth="29040" windowHeight="15840" firstSheet="6" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="BOE3 Pivot" sheetId="19" state="hidden" r:id="rId1"/>
@@ -320,7 +320,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="876" uniqueCount="140">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="877" uniqueCount="141">
   <si>
     <t>Start Date</t>
   </si>
@@ -740,6 +740,9 @@
   </si>
   <si>
     <t>SAP Connection Enabled</t>
+  </si>
+  <si>
+    <t>Source</t>
   </si>
 </sst>
 </file>
@@ -6217,7 +6220,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EDDB750B-2EAA-4C67-B526-87C6863613C3}">
-  <dimension ref="A1:Q2"/>
+  <dimension ref="A1:R2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.140625" style="1" bestFit="1" customWidth="1"/>
@@ -6237,9 +6240,10 @@
     <col min="15" max="15" width="57.85546875" style="1" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="61.42578125" style="32" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="28.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="27.28515625" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" s="5" customFormat="1" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:18" s="5" customFormat="1" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
         <v>70</v>
       </c>
@@ -6289,10 +6293,13 @@
         <v>136</v>
       </c>
       <c r="Q1" s="5" t="s">
+        <v>140</v>
+      </c>
+      <c r="R1" s="5" t="s">
         <v>137</v>
       </c>
     </row>
-    <row r="2" spans="1:17" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
+    <row r="2" spans="1:18" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <autoFilter ref="A1:Q1" xr:uid="{EDDB750B-2EAA-4C67-B526-87C6863613C3}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Merged PR 1153: ACV-304: Workspace Data Report Multi-Selected Tabs Fix
Fixed an issue where the **BOE & Resource Combo** tab and **MOQ Table Data** tab were both selected on opening.

The reason why this was the case was pretty silly... long story short DONT save the template when you have another tab selected. Since Excel saves the meta-data of what cell you have selected, which worksheet you have open, scroll positioning, etc.

**_Screenshot of the issue:_**

![image-2023-02-09-15-43-12-182.png](https://idetfs01/Estimating/ec33f0ce-06e6-4674-9d97-643c8eb6e517/_apis/git/repositories/c962790d-14a5-4524-9fe8-35b4cce33cc3/pullRequests/1153/attachments/image-2023-02-09-15-43-12-182.png)
</commit_message>
<xml_diff>
--- a/GenBOE/GenBOE.Web/Templates/Export/WorkspaceDataMST.xlsx
+++ b/GenBOE/GenBOE.Web/Templates/Export/WorkspaceDataMST.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\e405721\Desktop\Code-Repos\IES\GenBOE\GenBOE.Web\Templates\Export\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C0A9B38D-3E45-4BE5-83D1-9441DA857D8F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E131BEF6-88B5-4C73-A51C-BE44A80E72BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="3825" windowWidth="29040" windowHeight="15840" firstSheet="6" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21240" firstSheet="5" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="BOE3 Pivot" sheetId="19" state="hidden" r:id="rId1"/>

</xml_diff>

<commit_message>
consolidated templates and added empty brc cols for odc
</commit_message>
<xml_diff>
--- a/GenBOE/GenBOE.Web/Templates/Export/WorkspaceDataMST.xlsx
+++ b/GenBOE/GenBOE.Web/Templates/Export/WorkspaceDataMST.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25601"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26130"/>
   <workbookPr showPivotChartFilter="1" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\e405721\Desktop\Code-Repos\IES\GenBOE\GenBOE.Web\Templates\Export\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\e302876\proph\IES\GenBOE\GenBOE.Web\Templates\Export\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E131BEF6-88B5-4C73-A51C-BE44A80E72BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA71204E-83A7-40B4-A06D-78329F08D05A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21240" firstSheet="5" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" firstSheet="5" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="BOE3 Pivot" sheetId="19" state="hidden" r:id="rId1"/>
@@ -36,13 +36,13 @@
     <externalReference r:id="rId19"/>
   </externalReferences>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'BOE &amp; Resource Combo'!$A$1:$AP$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">BOEs!$A$1:$AQ$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'BOE &amp; Resource Combo'!$A$1:$AT$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">BOEs!$A$1:$AU$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'BOEs (2)'!$B$1:$T$16</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'BOEs (3)'!$A$1:$N$16</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'MOQ by BOE by Task'!$A$1:$F$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'MOQ Table Data'!$A$1:$Q$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Resource Spreads'!$A$1:$N$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Resource Spreads'!$A$1:$P$2</definedName>
     <definedName name="Approvers">'[1]Options Lists'!$D$2:$D$4</definedName>
     <definedName name="Authors">'[1]Options Lists'!$C$2:$C$4</definedName>
     <definedName name="CLINs">'[1]Options Lists'!$B$2:$B$5</definedName>
@@ -53,10 +53,11 @@
   </definedNames>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="0" r:id="rId20"/>
-    <pivotCache cacheId="1" r:id="rId21"/>
-    <pivotCache cacheId="2" r:id="rId22"/>
+    <pivotCache cacheId="3" r:id="rId20"/>
+    <pivotCache cacheId="4" r:id="rId21"/>
+    <pivotCache cacheId="5" r:id="rId22"/>
   </pivotCaches>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -320,7 +321,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="877" uniqueCount="141">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="887" uniqueCount="145">
   <si>
     <t>Start Date</t>
   </si>
@@ -743,6 +744,18 @@
   </si>
   <si>
     <t>Source</t>
+  </si>
+  <si>
+    <t>BRC</t>
+  </si>
+  <si>
+    <t>BRC Description</t>
+  </si>
+  <si>
+    <t>BRC Type</t>
+  </si>
+  <si>
+    <t>BRC Segment Region</t>
   </si>
 </sst>
 </file>
@@ -3138,7 +3151,7 @@
 <file path=xl/pivotCache/pivotCacheDefinition2.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="Lindsay Yorks" refreshedDate="40653.729487847224" createdVersion="3" refreshedVersion="3" minRefreshableVersion="3" recordCount="15" xr:uid="{00000000-000A-0000-FFFF-FFFF01000000}">
   <cacheSource type="worksheet">
-    <worksheetSource ref="C1:AP1" sheet="BOEs"/>
+    <worksheetSource ref="C1:AT1" sheet="BOEs"/>
   </cacheSource>
   <cacheFields count="19">
     <cacheField name="Type" numFmtId="49">
@@ -4342,7 +4355,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0000-000000000000}" name="PivotTable7" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="3" minRefreshableVersion="3" showCalcMbrs="0" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="3" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0000-000000000000}" name="PivotTable7" cacheId="3" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="3" minRefreshableVersion="3" showCalcMbrs="0" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="3" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
   <location ref="A3:N33" firstHeaderRow="1" firstDataRow="1" firstDataCol="14"/>
   <pivotFields count="14">
     <pivotField axis="axisRow" compact="0" outline="0" showAll="0" insertBlankRow="1" defaultSubtotal="0">
@@ -4691,7 +4704,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0200-000000000000}" name="PivotTable9" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="3" minRefreshableVersion="3" showCalcMbrs="0" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="3" indent="0" compact="0" compactData="0" multipleFieldFilters="0" rowHeaderCaption="Type">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0200-000000000000}" name="PivotTable9" cacheId="4" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="3" minRefreshableVersion="3" showCalcMbrs="0" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="3" indent="0" compact="0" compactData="0" multipleFieldFilters="0" rowHeaderCaption="Type">
   <location ref="A3:H11" firstHeaderRow="1" firstDataRow="1" firstDataCol="8"/>
   <pivotFields count="19">
     <pivotField axis="axisRow" compact="0" outline="0" showAll="0" defaultSubtotal="0">
@@ -4900,7 +4913,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0300-000000000000}" name="PivotTable4" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" missingCaption="_" updatedVersion="3" minRefreshableVersion="3" showCalcMbrs="0" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="3" indent="0" compact="0" compactData="0" multipleFieldFilters="0" rowHeaderCaption="BOE ID">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0300-000000000000}" name="PivotTable4" cacheId="5" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" missingCaption="_" updatedVersion="3" minRefreshableVersion="3" showCalcMbrs="0" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="3" indent="0" compact="0" compactData="0" multipleFieldFilters="0" rowHeaderCaption="BOE ID">
   <location ref="A3:T33" firstHeaderRow="1" firstDataRow="1" firstDataCol="20"/>
   <pivotFields count="20">
     <pivotField axis="axisRow" compact="0" outline="0" showAll="0" insertBlankRow="1" defaultSubtotal="0">
@@ -5664,25 +5677,25 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A3:N32"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="22.5703125" customWidth="1"/>
-    <col min="2" max="2" width="11.42578125" customWidth="1"/>
-    <col min="3" max="3" width="10.5703125" customWidth="1"/>
+    <col min="1" max="1" width="22.5546875" customWidth="1"/>
+    <col min="2" max="2" width="11.44140625" customWidth="1"/>
+    <col min="3" max="3" width="10.5546875" customWidth="1"/>
     <col min="4" max="4" width="15" customWidth="1"/>
-    <col min="5" max="5" width="11.7109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.85546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13.140625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.88671875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.44140625" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="17" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="12" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="11.140625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="11.109375" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="15" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="11.44140625" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="15" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
         <v>33</v>
       </c>
@@ -5726,7 +5739,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>59</v>
       </c>
@@ -5770,7 +5783,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.3">
       <c r="G6" t="s">
         <v>57</v>
       </c>
@@ -5796,7 +5809,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:14" x14ac:dyDescent="0.3">
       <c r="H8" t="s">
         <v>43</v>
       </c>
@@ -5819,7 +5832,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:14" x14ac:dyDescent="0.3">
       <c r="D10" t="s">
         <v>62</v>
       </c>
@@ -5854,7 +5867,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:14" x14ac:dyDescent="0.3">
       <c r="G12" t="s">
         <v>57</v>
       </c>
@@ -5880,7 +5893,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:14" x14ac:dyDescent="0.3">
       <c r="H14" t="s">
         <v>43</v>
       </c>
@@ -5903,7 +5916,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:14" x14ac:dyDescent="0.3">
       <c r="D16" t="s">
         <v>57</v>
       </c>
@@ -5938,7 +5951,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="18" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>60</v>
       </c>
@@ -5982,7 +5995,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="20" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:14" x14ac:dyDescent="0.3">
       <c r="G20" t="s">
         <v>57</v>
       </c>
@@ -6008,7 +6021,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="22" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:14" x14ac:dyDescent="0.3">
       <c r="H22" t="s">
         <v>43</v>
       </c>
@@ -6031,7 +6044,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="24" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:14" x14ac:dyDescent="0.3">
       <c r="H24" t="s">
         <v>55</v>
       </c>
@@ -6054,7 +6067,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="26" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:14" x14ac:dyDescent="0.3">
       <c r="H26" t="s">
         <v>51</v>
       </c>
@@ -6077,7 +6090,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="28" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:14" x14ac:dyDescent="0.3">
       <c r="D28" t="s">
         <v>64</v>
       </c>
@@ -6112,7 +6125,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="30" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:14" x14ac:dyDescent="0.3">
       <c r="G30" t="s">
         <v>57</v>
       </c>
@@ -6138,7 +6151,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="32" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:14" x14ac:dyDescent="0.3">
       <c r="D32" t="s">
         <v>62</v>
       </c>
@@ -6176,22 +6189,26 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId2"/>
+  <headerFooter>
+    <oddHeader>&amp;C&amp;"Calibri"&amp;10&amp;K000000 Lockheed Martin Proprietary Information&amp;1#_x000D_</oddHeader>
+    <oddFooter>&amp;C_x000D_&amp;1#&amp;"Calibri"&amp;10&amp;K000000 Lockheed Martin Proprietary Information</oddFooter>
+  </headerFooter>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3DA6D2FB-3F32-46E9-963C-DCD2D761F967}">
   <dimension ref="A1:F2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="11.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.44140625" bestFit="1" customWidth="1"/>
     <col min="4" max="5" width="24" customWidth="1"/>
-    <col min="6" max="6" width="40.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="40.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" ht="16.8" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="5" t="s">
         <v>70</v>
       </c>
@@ -6211,39 +6228,43 @@
         <v>84</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
+    <row r="2" spans="1:6" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <autoFilter ref="A1:F1" xr:uid="{1E7471F8-87B8-4A9F-A5C2-80CE50F530C1}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter>
+    <oddHeader>&amp;C&amp;"Calibri"&amp;10&amp;K000000 Lockheed Martin Proprietary Information&amp;1#_x000D_</oddHeader>
+    <oddFooter>&amp;C_x000D_&amp;1#&amp;"Calibri"&amp;10&amp;K000000 Lockheed Martin Proprietary Information</oddFooter>
+  </headerFooter>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EDDB750B-2EAA-4C67-B526-87C6863613C3}">
   <dimension ref="A1:R2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="11.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.44140625" style="1" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="24" style="1" customWidth="1"/>
-    <col min="5" max="5" width="42.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="15.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="18.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="28.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="21.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="42.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.88671875" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="18.88671875" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="28.88671875" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="21.109375" style="1" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="23" style="1" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="42" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="41.140625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="41.140625" style="32" customWidth="1"/>
-    <col min="14" max="14" width="35.28515625" style="32" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="57.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="61.42578125" style="32" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="28.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="27.28515625" style="1" customWidth="1"/>
+    <col min="12" max="12" width="41.109375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="41.109375" style="32" customWidth="1"/>
+    <col min="14" max="14" width="35.33203125" style="32" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="57.88671875" style="1" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="61.44140625" style="32" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="28.44140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="27.33203125" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" s="5" customFormat="1" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:18" s="5" customFormat="1" ht="16.8" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="5" t="s">
         <v>70</v>
       </c>
@@ -6299,26 +6320,30 @@
         <v>137</v>
       </c>
     </row>
-    <row r="2" spans="1:18" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
+    <row r="2" spans="1:18" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <autoFilter ref="A1:Q1" xr:uid="{EDDB750B-2EAA-4C67-B526-87C6863613C3}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
+  <headerFooter>
+    <oddHeader>&amp;C&amp;"Calibri"&amp;10&amp;K000000 Lockheed Martin Proprietary Information&amp;1#_x000D_</oddHeader>
+    <oddFooter>&amp;C_x000D_&amp;1#&amp;"Calibri"&amp;10&amp;K000000 Lockheed Martin Proprietary Information</oddFooter>
+  </headerFooter>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
   <dimension ref="A1:E2"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="13.8" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="30.7109375" style="6" hidden="1" customWidth="1"/>
-    <col min="2" max="4" width="30.7109375" style="8" customWidth="1"/>
-    <col min="5" max="5" width="33.140625" style="7" customWidth="1"/>
-    <col min="6" max="16384" width="9.140625" style="7"/>
+    <col min="1" max="1" width="30.6640625" style="6" hidden="1" customWidth="1"/>
+    <col min="2" max="4" width="30.6640625" style="8" customWidth="1"/>
+    <col min="5" max="5" width="33.109375" style="7" customWidth="1"/>
+    <col min="6" max="16384" width="9.109375" style="7"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="5" customFormat="1" ht="20.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" s="5" customFormat="1" ht="20.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="5" t="s">
         <v>68</v>
       </c>
@@ -6335,10 +6360,14 @@
         <v>114</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="13.5" thickTop="1" x14ac:dyDescent="0.2"/>
+    <row r="2" spans="1:5" ht="14.4" thickTop="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
+  <headerFooter>
+    <oddHeader>&amp;C&amp;"Calibri"&amp;10&amp;K000000 Lockheed Martin Proprietary Information&amp;1#_x000D_</oddHeader>
+    <oddFooter>&amp;C_x000D_&amp;1#&amp;"Calibri"&amp;10&amp;K000000 Lockheed Martin Proprietary Information</oddFooter>
+  </headerFooter>
   <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
@@ -6346,16 +6375,16 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
   <dimension ref="A1:E2"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="13.8" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="13.140625" style="6" hidden="1" customWidth="1"/>
-    <col min="2" max="2" width="30.7109375" style="8" customWidth="1"/>
-    <col min="3" max="3" width="50.7109375" style="8" customWidth="1"/>
-    <col min="4" max="5" width="20.7109375" style="8" customWidth="1"/>
-    <col min="6" max="16384" width="9.140625" style="7"/>
+    <col min="1" max="1" width="13.109375" style="6" hidden="1" customWidth="1"/>
+    <col min="2" max="2" width="30.6640625" style="8" customWidth="1"/>
+    <col min="3" max="3" width="50.6640625" style="8" customWidth="1"/>
+    <col min="4" max="5" width="20.6640625" style="8" customWidth="1"/>
+    <col min="6" max="16384" width="9.109375" style="7"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="5" customFormat="1" ht="20.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" s="5" customFormat="1" ht="20.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="5" t="s">
         <v>98</v>
       </c>
@@ -6372,10 +6401,14 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="13.5" thickTop="1" x14ac:dyDescent="0.2"/>
+    <row r="2" spans="1:5" ht="14.4" thickTop="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
+  <headerFooter>
+    <oddHeader>&amp;C&amp;"Calibri"&amp;10&amp;K000000 Lockheed Martin Proprietary Information&amp;1#_x000D_</oddHeader>
+    <oddFooter>&amp;C_x000D_&amp;1#&amp;"Calibri"&amp;10&amp;K000000 Lockheed Martin Proprietary Information</oddFooter>
+  </headerFooter>
   <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
@@ -6383,20 +6416,20 @@
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0B00-000000000000}">
   <dimension ref="A1:I2"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="18.85546875" style="15" customWidth="1"/>
-    <col min="2" max="3" width="35.7109375" style="15" customWidth="1"/>
-    <col min="4" max="4" width="26.140625" style="15" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.5703125" style="15" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="22.140625" style="15" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="10.85546875" style="15" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="13.140625" style="15" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="21.85546875" style="15" bestFit="1" customWidth="1"/>
-    <col min="10" max="16384" width="9.140625" style="15"/>
+    <col min="1" max="1" width="18.88671875" style="15" customWidth="1"/>
+    <col min="2" max="3" width="35.6640625" style="15" customWidth="1"/>
+    <col min="4" max="4" width="26.109375" style="15" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.5546875" style="15" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="22.109375" style="15" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.88671875" style="15" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.109375" style="15" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="21.88671875" style="15" bestFit="1" customWidth="1"/>
+    <col min="10" max="16384" width="9.109375" style="15"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" s="14" customFormat="1" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" s="14" customFormat="1" ht="16.8" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>71</v>
       </c>
@@ -6425,126 +6458,134 @@
         <v>125</v>
       </c>
     </row>
-    <row r="2" spans="1:9" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
+    <row r="2" spans="1:9" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
+  <headerFooter>
+    <oddHeader>&amp;C&amp;"Calibri"&amp;10&amp;K000000 Lockheed Martin Proprietary Information&amp;1#_x000D_</oddHeader>
+    <oddFooter>&amp;C_x000D_&amp;1#&amp;"Calibri"&amp;10&amp;K000000 Lockheed Martin Proprietary Information</oddFooter>
+  </headerFooter>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0C00-000000000000}">
   <dimension ref="A1:A16"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="28" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="82.140625" style="1" customWidth="1"/>
-    <col min="3" max="16384" width="9.140625" style="1"/>
+    <col min="2" max="2" width="82.109375" style="1" customWidth="1"/>
+    <col min="3" max="16384" width="9.109375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="2" spans="1:1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" hidden="1" x14ac:dyDescent="0.3"/>
+    <row r="2" spans="1:1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="10" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="3" spans="1:1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="10" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="4" spans="1:1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="10" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="5" spans="1:1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="10"/>
     </row>
-    <row r="6" spans="1:1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="10" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="7" spans="1:1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="10" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="8" spans="1:1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="11" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="9" spans="1:1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="11" t="s">
         <v>122</v>
       </c>
     </row>
-    <row r="10" spans="1:1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="11" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="11" spans="1:1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="12" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="12" spans="1:1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="12" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="13" spans="1:1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="10" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="14" spans="1:1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="19" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="15" spans="1:1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="19" t="s">
         <v>139</v>
       </c>
     </row>
-    <row r="16" spans="1:1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="16" spans="1:1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
+  <headerFooter>
+    <oddHeader>&amp;C&amp;"Calibri"&amp;10&amp;K000000 Lockheed Martin Proprietary Information&amp;1#_x000D_</oddHeader>
+    <oddFooter>&amp;C_x000D_&amp;1#&amp;"Calibri"&amp;10&amp;K000000 Lockheed Martin Proprietary Information</oddFooter>
+  </headerFooter>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1E9E49D2-B4A1-426D-8F6A-B85DD2E6A5AA}">
   <dimension ref="A1:AA7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
-    <col min="2" max="2" width="7.140625" customWidth="1"/>
-    <col min="3" max="3" width="29.42578125" customWidth="1"/>
-    <col min="4" max="4" width="26.85546875" customWidth="1"/>
-    <col min="5" max="5" width="12.28515625" customWidth="1"/>
+    <col min="2" max="2" width="7.109375" customWidth="1"/>
+    <col min="3" max="3" width="29.44140625" customWidth="1"/>
+    <col min="4" max="4" width="26.88671875" customWidth="1"/>
+    <col min="5" max="5" width="12.33203125" customWidth="1"/>
     <col min="6" max="6" width="16" customWidth="1"/>
-    <col min="7" max="7" width="20.5703125" customWidth="1"/>
-    <col min="8" max="8" width="10.5703125" style="39" customWidth="1"/>
-    <col min="9" max="11" width="8.85546875" style="39"/>
-    <col min="12" max="12" width="12.85546875" style="39" customWidth="1"/>
-    <col min="13" max="13" width="8.85546875" style="39"/>
-    <col min="14" max="14" width="15.5703125" style="56" customWidth="1"/>
-    <col min="15" max="15" width="19.140625" style="56" customWidth="1"/>
-    <col min="16" max="16" width="15.7109375" style="56" customWidth="1"/>
-    <col min="17" max="17" width="19.28515625" style="56" customWidth="1"/>
-    <col min="18" max="18" width="13.7109375" style="56" customWidth="1"/>
-    <col min="19" max="19" width="17.85546875" style="56" customWidth="1"/>
-    <col min="20" max="20" width="17.7109375" customWidth="1"/>
-    <col min="21" max="21" width="15.28515625" customWidth="1"/>
+    <col min="7" max="7" width="20.5546875" customWidth="1"/>
+    <col min="8" max="8" width="10.5546875" style="39" customWidth="1"/>
+    <col min="9" max="11" width="8.88671875" style="39"/>
+    <col min="12" max="12" width="12.88671875" style="39" customWidth="1"/>
+    <col min="13" max="13" width="8.88671875" style="39"/>
+    <col min="14" max="14" width="15.5546875" style="56" customWidth="1"/>
+    <col min="15" max="15" width="19.109375" style="56" customWidth="1"/>
+    <col min="16" max="16" width="15.6640625" style="56" customWidth="1"/>
+    <col min="17" max="17" width="19.33203125" style="56" customWidth="1"/>
+    <col min="18" max="18" width="13.6640625" style="56" customWidth="1"/>
+    <col min="19" max="19" width="17.88671875" style="56" customWidth="1"/>
+    <col min="20" max="20" width="17.6640625" customWidth="1"/>
+    <col min="21" max="21" width="15.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:27" s="44" customFormat="1" ht="20.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:27" s="44" customFormat="1" ht="19.2" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A1" s="40"/>
       <c r="B1" s="41"/>
       <c r="C1" s="41"/>
@@ -6572,7 +6613,7 @@
       <c r="Z1" s="53"/>
       <c r="AA1" s="53"/>
     </row>
-    <row r="2" spans="1:27" s="44" customFormat="1" ht="19.5" thickTop="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:27" s="44" customFormat="1" ht="18.600000000000001" thickTop="1" x14ac:dyDescent="0.35">
       <c r="A2" s="40"/>
       <c r="B2" s="41"/>
       <c r="C2" s="41"/>
@@ -6601,7 +6642,7 @@
       <c r="Z2" s="53"/>
       <c r="AA2" s="53"/>
     </row>
-    <row r="3" spans="1:27" s="44" customFormat="1" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:27" s="44" customFormat="1" ht="18" x14ac:dyDescent="0.35">
       <c r="A3" s="40"/>
       <c r="B3" s="41"/>
       <c r="C3" s="41"/>
@@ -6630,7 +6671,7 @@
       <c r="Z3" s="53"/>
       <c r="AA3" s="53"/>
     </row>
-    <row r="4" spans="1:27" s="44" customFormat="1" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:27" s="44" customFormat="1" ht="18" x14ac:dyDescent="0.35">
       <c r="A4" s="40"/>
       <c r="B4" s="41"/>
       <c r="C4" s="41"/>
@@ -6659,7 +6700,7 @@
       <c r="Z4" s="53"/>
       <c r="AA4" s="53"/>
     </row>
-    <row r="5" spans="1:27" s="44" customFormat="1" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:27" s="44" customFormat="1" ht="18" x14ac:dyDescent="0.35">
       <c r="A5" s="54"/>
       <c r="B5" s="41"/>
       <c r="C5" s="41"/>
@@ -6688,7 +6729,7 @@
       <c r="Z5" s="53"/>
       <c r="AA5" s="53"/>
     </row>
-    <row r="6" spans="1:27" s="44" customFormat="1" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:27" s="44" customFormat="1" ht="18" x14ac:dyDescent="0.35">
       <c r="A6" s="54"/>
       <c r="B6" s="55"/>
       <c r="C6" s="55"/>
@@ -6717,7 +6758,7 @@
       <c r="Z6" s="53"/>
       <c r="AA6" s="53"/>
     </row>
-    <row r="7" spans="1:27" s="54" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:27" s="54" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="H7" s="42"/>
       <c r="I7" s="42"/>
       <c r="J7" s="42"/>
@@ -6736,35 +6777,39 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter>
+    <oddHeader>&amp;C&amp;"Calibri"&amp;10&amp;K000000 Lockheed Martin Proprietary Information&amp;1#_x000D_</oddHeader>
+    <oddFooter>&amp;C_x000D_&amp;1#&amp;"Calibri"&amp;10&amp;K000000 Lockheed Martin Proprietary Information</oddFooter>
+  </headerFooter>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00BB237A-2FF2-450F-81EE-9A098F6C7133}">
   <dimension ref="A1:AA6"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="11.7109375" style="57" customWidth="1"/>
-    <col min="2" max="2" width="7.140625" style="57" customWidth="1"/>
-    <col min="3" max="3" width="29.42578125" style="57" customWidth="1"/>
-    <col min="4" max="4" width="26.85546875" style="57" customWidth="1"/>
-    <col min="5" max="5" width="12.28515625" style="57" customWidth="1"/>
+    <col min="1" max="1" width="11.6640625" style="57" customWidth="1"/>
+    <col min="2" max="2" width="7.109375" style="57" customWidth="1"/>
+    <col min="3" max="3" width="29.44140625" style="57" customWidth="1"/>
+    <col min="4" max="4" width="26.88671875" style="57" customWidth="1"/>
+    <col min="5" max="5" width="12.33203125" style="57" customWidth="1"/>
     <col min="6" max="6" width="16" style="57" customWidth="1"/>
-    <col min="7" max="7" width="20.5703125" style="57" customWidth="1"/>
-    <col min="8" max="8" width="10.5703125" style="58" customWidth="1"/>
-    <col min="9" max="13" width="9.140625" style="58"/>
-    <col min="14" max="14" width="15.5703125" style="56" customWidth="1"/>
-    <col min="15" max="15" width="24.5703125" style="56" customWidth="1"/>
-    <col min="16" max="16" width="15.7109375" style="56" customWidth="1"/>
-    <col min="17" max="17" width="19.28515625" style="56" customWidth="1"/>
-    <col min="18" max="18" width="13.7109375" style="56" customWidth="1"/>
-    <col min="19" max="19" width="17.85546875" style="56" customWidth="1"/>
-    <col min="20" max="20" width="17.7109375" style="56" customWidth="1"/>
-    <col min="21" max="21" width="15.28515625" style="56" customWidth="1"/>
-    <col min="22" max="16384" width="9.140625" style="59"/>
+    <col min="7" max="7" width="20.5546875" style="57" customWidth="1"/>
+    <col min="8" max="8" width="10.5546875" style="58" customWidth="1"/>
+    <col min="9" max="13" width="9.109375" style="58"/>
+    <col min="14" max="14" width="15.5546875" style="56" customWidth="1"/>
+    <col min="15" max="15" width="24.5546875" style="56" customWidth="1"/>
+    <col min="16" max="16" width="15.6640625" style="56" customWidth="1"/>
+    <col min="17" max="17" width="19.33203125" style="56" customWidth="1"/>
+    <col min="18" max="18" width="13.6640625" style="56" customWidth="1"/>
+    <col min="19" max="19" width="17.88671875" style="56" customWidth="1"/>
+    <col min="20" max="20" width="17.6640625" style="56" customWidth="1"/>
+    <col min="21" max="21" width="15.33203125" style="56" customWidth="1"/>
+    <col min="22" max="16384" width="9.109375" style="59"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:27" s="51" customFormat="1" ht="20.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:27" s="51" customFormat="1" ht="19.2" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A1" s="41"/>
       <c r="B1" s="41"/>
       <c r="C1" s="41"/>
@@ -6793,7 +6838,7 @@
       <c r="Z1" s="50"/>
       <c r="AA1" s="50"/>
     </row>
-    <row r="2" spans="1:27" s="51" customFormat="1" ht="19.5" thickTop="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:27" s="51" customFormat="1" ht="18.600000000000001" thickTop="1" x14ac:dyDescent="0.35">
       <c r="A2" s="41"/>
       <c r="B2" s="41"/>
       <c r="C2" s="41"/>
@@ -6822,7 +6867,7 @@
       <c r="Z2" s="50"/>
       <c r="AA2" s="50"/>
     </row>
-    <row r="3" spans="1:27" s="51" customFormat="1" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:27" s="51" customFormat="1" ht="18" x14ac:dyDescent="0.35">
       <c r="A3" s="41"/>
       <c r="B3" s="41"/>
       <c r="C3" s="41"/>
@@ -6851,7 +6896,7 @@
       <c r="Z3" s="50"/>
       <c r="AA3" s="50"/>
     </row>
-    <row r="4" spans="1:27" s="51" customFormat="1" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:27" s="51" customFormat="1" ht="18" x14ac:dyDescent="0.35">
       <c r="A4" s="41"/>
       <c r="B4" s="41"/>
       <c r="C4" s="41"/>
@@ -6880,7 +6925,7 @@
       <c r="Z4" s="50"/>
       <c r="AA4" s="50"/>
     </row>
-    <row r="5" spans="1:27" s="51" customFormat="1" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:27" s="51" customFormat="1" ht="18" x14ac:dyDescent="0.35">
       <c r="A5" s="41"/>
       <c r="B5" s="41"/>
       <c r="C5" s="41"/>
@@ -6909,7 +6954,7 @@
       <c r="Z5" s="50"/>
       <c r="AA5" s="50"/>
     </row>
-    <row r="6" spans="1:27" s="44" customFormat="1" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:27" s="44" customFormat="1" ht="18" x14ac:dyDescent="0.35">
       <c r="A6" s="55"/>
       <c r="B6" s="55"/>
       <c r="C6" s="55"/>
@@ -6940,34 +6985,38 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter>
+    <oddHeader>&amp;C&amp;"Calibri"&amp;10&amp;K000000 Lockheed Martin Proprietary Information&amp;1#_x000D_</oddHeader>
+    <oddFooter>&amp;C_x000D_&amp;1#&amp;"Calibri"&amp;10&amp;K000000 Lockheed Martin Proprietary Information</oddFooter>
+  </headerFooter>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:N16"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="16.85546875" style="3" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.42578125" style="3" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.5703125" style="3" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.42578125" style="3" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.7109375" style="3" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.85546875" style="3" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="15.42578125" style="3" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="13.140625" style="3" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="18.85546875" style="3" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="13.85546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.88671875" style="3" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.44140625" style="3" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.5546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.44140625" style="3" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.6640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.88671875" style="3" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.44140625" style="3" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.109375" style="3" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="18.88671875" style="3" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="13.88671875" style="3" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="13" style="3" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="16.85546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="16.88671875" style="3" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="13" style="3" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="17" style="3" bestFit="1" customWidth="1"/>
-    <col min="15" max="17" width="13.5703125" style="3" customWidth="1"/>
-    <col min="18" max="18" width="15.42578125" style="3" bestFit="1" customWidth="1"/>
-    <col min="19" max="16384" width="9.140625" style="3"/>
+    <col min="15" max="17" width="13.5546875" style="3" customWidth="1"/>
+    <col min="18" max="18" width="15.44140625" style="3" bestFit="1" customWidth="1"/>
+    <col min="19" max="16384" width="9.109375" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:14" ht="16.8" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>33</v>
       </c>
@@ -7011,7 +7060,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="2" spans="1:14" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:14" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
         <v>59</v>
       </c>
@@ -7022,7 +7071,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
         <v>59</v>
       </c>
@@ -7045,7 +7094,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
         <v>59</v>
       </c>
@@ -7086,7 +7135,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
         <v>59</v>
       </c>
@@ -7127,7 +7176,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
         <v>59</v>
       </c>
@@ -7150,7 +7199,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
         <v>59</v>
       </c>
@@ -7191,7 +7240,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A8" s="3" t="s">
         <v>59</v>
       </c>
@@ -7232,7 +7281,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A9" s="3" t="s">
         <v>60</v>
       </c>
@@ -7252,7 +7301,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A10" s="3" t="s">
         <v>60</v>
       </c>
@@ -7275,7 +7324,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A11" s="3" t="s">
         <v>60</v>
       </c>
@@ -7316,7 +7365,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A12" s="3" t="s">
         <v>60</v>
       </c>
@@ -7357,7 +7406,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A13" s="3" t="s">
         <v>60</v>
       </c>
@@ -7398,7 +7447,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A14" s="3" t="s">
         <v>60</v>
       </c>
@@ -7439,7 +7488,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A15" s="3" t="s">
         <v>60</v>
       </c>
@@ -7462,7 +7511,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A16" s="3" t="s">
         <v>60</v>
       </c>
@@ -7507,26 +7556,30 @@
   <autoFilter ref="A1:N16" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
+  <headerFooter>
+    <oddHeader>&amp;C&amp;"Calibri"&amp;10&amp;K000000 Lockheed Martin Proprietary Information&amp;1#_x000D_</oddHeader>
+    <oddFooter>&amp;C_x000D_&amp;1#&amp;"Calibri"&amp;10&amp;K000000 Lockheed Martin Proprietary Information</oddFooter>
+  </headerFooter>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A3:H11"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="7.5703125" customWidth="1"/>
-    <col min="2" max="2" width="8.85546875" customWidth="1"/>
-    <col min="3" max="3" width="11.85546875" customWidth="1"/>
-    <col min="4" max="4" width="8.7109375" customWidth="1"/>
-    <col min="5" max="5" width="11.7109375" customWidth="1"/>
-    <col min="6" max="6" width="11.42578125" customWidth="1"/>
-    <col min="7" max="7" width="10.5703125" customWidth="1"/>
-    <col min="8" max="8" width="9.42578125" customWidth="1"/>
+    <col min="1" max="1" width="7.5546875" customWidth="1"/>
+    <col min="2" max="2" width="8.88671875" customWidth="1"/>
+    <col min="3" max="3" width="11.88671875" customWidth="1"/>
+    <col min="4" max="4" width="8.6640625" customWidth="1"/>
+    <col min="5" max="5" width="11.6640625" customWidth="1"/>
+    <col min="6" max="6" width="11.44140625" customWidth="1"/>
+    <col min="7" max="7" width="10.5546875" customWidth="1"/>
+    <col min="8" max="8" width="9.44140625" customWidth="1"/>
     <col min="9" max="19" width="15" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
         <v>26</v>
       </c>
@@ -7552,7 +7605,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>33</v>
       </c>
@@ -7578,7 +7631,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="B5" t="s">
         <v>45</v>
       </c>
@@ -7586,7 +7639,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>12</v>
       </c>
@@ -7612,12 +7665,12 @@
         <v>38</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
       <c r="H7" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="B8" t="s">
         <v>45</v>
       </c>
@@ -7625,7 +7678,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>34</v>
       </c>
@@ -7651,12 +7704,12 @@
         <v>38</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
       <c r="H10" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
       <c r="B11" t="s">
         <v>45</v>
       </c>
@@ -7667,35 +7720,39 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId2"/>
+  <headerFooter>
+    <oddHeader>&amp;C&amp;"Calibri"&amp;10&amp;K000000 Lockheed Martin Proprietary Information&amp;1#_x000D_</oddHeader>
+    <oddFooter>&amp;C_x000D_&amp;1#&amp;"Calibri"&amp;10&amp;K000000 Lockheed Martin Proprietary Information</oddFooter>
+  </headerFooter>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A3:T32"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="22.42578125" customWidth="1"/>
-    <col min="2" max="2" width="12.42578125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.7109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.42578125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="11.7109375" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="10.85546875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.140625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="22.44140625" customWidth="1"/>
+    <col min="2" max="2" width="12.44140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.88671875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.44140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.5546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="9.44140625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.5546875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="10.88671875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="13.109375" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="11.44140625" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="17" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="12" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.140625" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.109375" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="15" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="11.44140625" bestFit="1" customWidth="1"/>
     <col min="20" max="20" width="15" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
         <v>70</v>
       </c>
@@ -7757,7 +7814,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="4" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>58</v>
       </c>
@@ -7819,7 +7876,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="6" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:20" x14ac:dyDescent="0.3">
       <c r="B6" t="s">
         <v>34</v>
       </c>
@@ -7878,7 +7935,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="8" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:20" x14ac:dyDescent="0.3">
       <c r="I8" t="s">
         <v>40</v>
       </c>
@@ -7916,7 +7973,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="10" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:20" x14ac:dyDescent="0.3">
       <c r="B10" t="s">
         <v>12</v>
       </c>
@@ -7975,7 +8032,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="12" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:20" x14ac:dyDescent="0.3">
       <c r="R12" t="s">
         <v>20</v>
       </c>
@@ -7986,7 +8043,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="14" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:20" x14ac:dyDescent="0.3">
       <c r="N14" t="s">
         <v>43</v>
       </c>
@@ -8009,7 +8066,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="16" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:20" x14ac:dyDescent="0.3">
       <c r="O16" t="s">
         <v>53</v>
       </c>
@@ -8029,7 +8086,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="18" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>45</v>
       </c>
@@ -8091,7 +8148,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="20" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:20" x14ac:dyDescent="0.3">
       <c r="B20" t="s">
         <v>34</v>
       </c>
@@ -8150,7 +8207,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="22" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:20" x14ac:dyDescent="0.3">
       <c r="I22" t="s">
         <v>49</v>
       </c>
@@ -8188,7 +8245,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="24" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:20" x14ac:dyDescent="0.3">
       <c r="B24" t="s">
         <v>12</v>
       </c>
@@ -8247,7 +8304,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="26" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:20" x14ac:dyDescent="0.3">
       <c r="O26" t="s">
         <v>52</v>
       </c>
@@ -8267,7 +8324,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="28" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:20" x14ac:dyDescent="0.3">
       <c r="N28" t="s">
         <v>43</v>
       </c>
@@ -8290,7 +8347,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="30" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:20" x14ac:dyDescent="0.3">
       <c r="N30" t="s">
         <v>55</v>
       </c>
@@ -8313,7 +8370,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="32" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:20" x14ac:dyDescent="0.3">
       <c r="N32" t="s">
         <v>51</v>
       </c>
@@ -8339,39 +8396,43 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId2"/>
+  <headerFooter>
+    <oddHeader>&amp;C&amp;"Calibri"&amp;10&amp;K000000 Lockheed Martin Proprietary Information&amp;1#_x000D_</oddHeader>
+    <oddFooter>&amp;C_x000D_&amp;1#&amp;"Calibri"&amp;10&amp;K000000 Lockheed Martin Proprietary Information</oddFooter>
+  </headerFooter>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:T16"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="9.140625" style="3"/>
-    <col min="2" max="3" width="10.5703125" style="3" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.5703125" style="3" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.5703125" style="3" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.5703125" style="3" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13.42578125" style="3" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="12.5703125" style="3" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="11.42578125" style="3" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="13.5703125" style="3" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="13.7109375" style="3" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="12.85546875" style="3" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="15.42578125" style="3" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="13.140625" style="3" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="18.85546875" style="3" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="13.85546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.109375" style="3"/>
+    <col min="2" max="3" width="10.5546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.5546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.5546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.5546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.44140625" style="3" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12.5546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="11.44140625" style="3" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="13.5546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="13.6640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="12.88671875" style="3" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="15.44140625" style="3" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="13.109375" style="3" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="18.88671875" style="3" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="13.88671875" style="3" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="13" style="3" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="16.85546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="16.88671875" style="3" bestFit="1" customWidth="1"/>
     <col min="19" max="19" width="13" style="3" bestFit="1" customWidth="1"/>
     <col min="20" max="20" width="17" style="3" bestFit="1" customWidth="1"/>
-    <col min="21" max="23" width="13.5703125" style="3" customWidth="1"/>
-    <col min="24" max="24" width="15.42578125" style="3" bestFit="1" customWidth="1"/>
-    <col min="25" max="16384" width="9.140625" style="3"/>
+    <col min="21" max="23" width="13.5546875" style="3" customWidth="1"/>
+    <col min="24" max="24" width="15.44140625" style="3" bestFit="1" customWidth="1"/>
+    <col min="25" max="16384" width="9.109375" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:20" ht="16.8" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>70</v>
       </c>
@@ -8433,7 +8494,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="2" spans="1:20" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:20" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
         <v>58</v>
       </c>
@@ -8459,7 +8520,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="3" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
         <v>58</v>
       </c>
@@ -8482,7 +8543,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="4" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
         <v>58</v>
       </c>
@@ -8511,7 +8572,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="5" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
         <v>58</v>
       </c>
@@ -8540,7 +8601,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="6" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
         <v>58</v>
       </c>
@@ -8563,7 +8624,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="7" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
         <v>58</v>
       </c>
@@ -8592,7 +8653,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="8" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A8" s="3" t="s">
         <v>58</v>
       </c>
@@ -8621,7 +8682,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="9" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A9" s="3" t="s">
         <v>45</v>
       </c>
@@ -8647,7 +8708,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="10" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A10" s="3" t="s">
         <v>45</v>
       </c>
@@ -8670,7 +8731,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="11" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A11" s="3" t="s">
         <v>45</v>
       </c>
@@ -8699,7 +8760,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="12" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A12" s="3" t="s">
         <v>45</v>
       </c>
@@ -8728,7 +8789,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="13" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A13" s="3" t="s">
         <v>45</v>
       </c>
@@ -8757,7 +8818,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="14" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A14" s="3" t="s">
         <v>45</v>
       </c>
@@ -8786,7 +8847,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="15" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A15" s="3" t="s">
         <v>45</v>
       </c>
@@ -8809,7 +8870,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="16" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A16" s="3" t="s">
         <v>45</v>
       </c>
@@ -8842,60 +8903,65 @@
   <autoFilter ref="B1:T16" xr:uid="{00000000-0009-0000-0000-000004000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
+  <headerFooter>
+    <oddHeader>&amp;C&amp;"Calibri"&amp;10&amp;K000000 Lockheed Martin Proprietary Information&amp;1#_x000D_</oddHeader>
+    <oddFooter>&amp;C_x000D_&amp;1#&amp;"Calibri"&amp;10&amp;K000000 Lockheed Martin Proprietary Information</oddFooter>
+  </headerFooter>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
-  <dimension ref="A1:AP2"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:AT2"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="11.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.85546875" style="1" customWidth="1"/>
-    <col min="4" max="4" width="11.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="18.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="19.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="19.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="10.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="13.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="19.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="10.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="13.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="13.42578125" style="37" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="12.5703125" style="37" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="21.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="20.140625" style="32" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="18.7109375" style="30" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="20.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="21.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="13.7109375" style="37" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="12.85546875" style="37" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="21.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="20.42578125" style="32" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.88671875" style="1" customWidth="1"/>
+    <col min="4" max="4" width="11.44140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.5546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="18.44140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.5546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="19.109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="19.88671875" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="10.5546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="13.5546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="19.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="10.5546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="13.5546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="13.44140625" style="37" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="12.5546875" style="37" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="21.44140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="20.109375" style="32" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="18.6640625" style="30" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="17.109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="20.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="21.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="13.6640625" style="37" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="12.88671875" style="37" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="21.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="20.44140625" style="32" bestFit="1" customWidth="1"/>
     <col min="27" max="27" width="19" style="30" bestFit="1" customWidth="1"/>
     <col min="28" max="28" width="20" style="1" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="24.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="18.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="18.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="18.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="23.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="16.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="35" max="35" width="13" style="34" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="17" style="32" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="15.7109375" style="30" bestFit="1" customWidth="1"/>
-    <col min="38" max="38" width="26.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="39" max="39" width="8.7109375" style="39" customWidth="1"/>
-    <col min="40" max="40" width="10.5703125" style="39" bestFit="1" customWidth="1"/>
-    <col min="41" max="41" width="10" style="32" bestFit="1" customWidth="1"/>
-    <col min="42" max="42" width="8.7109375" style="30" customWidth="1"/>
-    <col min="43" max="16384" width="9.140625" style="1"/>
+    <col min="29" max="29" width="24.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="18.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="18.5546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="32" max="35" width="18.5546875" style="1" customWidth="1"/>
+    <col min="36" max="36" width="18.88671875" style="1" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="23.88671875" style="1" bestFit="1" customWidth="1"/>
+    <col min="38" max="38" width="16.88671875" style="1" bestFit="1" customWidth="1"/>
+    <col min="39" max="39" width="13" style="34" bestFit="1" customWidth="1"/>
+    <col min="40" max="40" width="17" style="32" bestFit="1" customWidth="1"/>
+    <col min="41" max="41" width="15.6640625" style="30" bestFit="1" customWidth="1"/>
+    <col min="42" max="42" width="26.109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="43" max="43" width="8.6640625" style="39" customWidth="1"/>
+    <col min="44" max="44" width="10.5546875" style="39" bestFit="1" customWidth="1"/>
+    <col min="45" max="45" width="10" style="32" bestFit="1" customWidth="1"/>
+    <col min="46" max="46" width="8.6640625" style="30" customWidth="1"/>
+    <col min="47" max="16384" width="9.109375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:42" s="5" customFormat="1" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:46" s="5" customFormat="1" ht="16.8" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="5" t="s">
         <v>70</v>
       </c>
@@ -8990,92 +9056,109 @@
         <v>105</v>
       </c>
       <c r="AF1" s="5" t="s">
+        <v>141</v>
+      </c>
+      <c r="AG1" s="5" t="s">
+        <v>142</v>
+      </c>
+      <c r="AH1" s="5" t="s">
+        <v>143</v>
+      </c>
+      <c r="AI1" s="5" t="s">
+        <v>144</v>
+      </c>
+      <c r="AJ1" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="AG1" s="5" t="s">
+      <c r="AK1" s="5" t="s">
         <v>93</v>
       </c>
-      <c r="AH1" s="5" t="s">
+      <c r="AL1" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="AI1" s="33" t="s">
+      <c r="AM1" s="33" t="s">
         <v>14</v>
       </c>
-      <c r="AJ1" s="31" t="s">
+      <c r="AN1" s="31" t="s">
         <v>15</v>
       </c>
-      <c r="AK1" s="25" t="s">
+      <c r="AO1" s="25" t="s">
         <v>109</v>
       </c>
-      <c r="AL1" s="5" t="s">
+      <c r="AP1" s="5" t="s">
         <v>99</v>
       </c>
-      <c r="AM1" s="38" t="s">
+      <c r="AQ1" s="38" t="s">
         <v>90</v>
       </c>
-      <c r="AN1" s="38" t="s">
+      <c r="AR1" s="38" t="s">
         <v>91</v>
       </c>
-      <c r="AO1" s="35" t="s">
+      <c r="AS1" s="35" t="s">
         <v>110</v>
       </c>
-      <c r="AP1" s="28" t="s">
+      <c r="AT1" s="28" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="2" spans="1:42" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
+    <row r="2" spans="1:46" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
   </sheetData>
-  <autoFilter ref="A1:AP1" xr:uid="{00000000-0009-0000-0000-000005000000}"/>
+  <autoFilter ref="A1:AT1" xr:uid="{00000000-0009-0000-0000-000005000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
+  <headerFooter>
+    <oddHeader>&amp;C&amp;"Calibri"&amp;10&amp;K000000 Lockheed Martin Proprietary Information&amp;1#_x000D_</oddHeader>
+    <oddFooter>&amp;C_x000D_&amp;1#&amp;"Calibri"&amp;10&amp;K000000 Lockheed Martin Proprietary Information</oddFooter>
+  </headerFooter>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
-  <dimension ref="A1:AQ2"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:AU2"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="11.42578125" style="3" customWidth="1"/>
-    <col min="2" max="2" width="13.28515625" style="3" bestFit="1" customWidth="1"/>
-    <col min="3" max="4" width="10.5703125" style="3" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.5703125" style="3" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.5703125" style="3" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13.5703125" style="3" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="13.42578125" style="3" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="12.5703125" style="3" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="21.42578125" style="3" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="20.140625" style="21" bestFit="1" customWidth="1"/>
-    <col min="12" max="13" width="20.140625" style="26" customWidth="1"/>
-    <col min="14" max="14" width="20.140625" style="3" customWidth="1"/>
-    <col min="15" max="15" width="11.42578125" style="3" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="13.5703125" style="3" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="20.140625" style="3" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="18.42578125" style="3" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="23.85546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.44140625" style="3" customWidth="1"/>
+    <col min="2" max="2" width="13.33203125" style="3" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="10.5546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.5546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.5546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.5546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.44140625" style="3" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12.5546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="21.44140625" style="3" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="20.109375" style="21" bestFit="1" customWidth="1"/>
+    <col min="12" max="13" width="20.109375" style="26" customWidth="1"/>
+    <col min="14" max="14" width="20.109375" style="3" customWidth="1"/>
+    <col min="15" max="15" width="11.44140625" style="3" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="13.5546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="20.109375" style="3" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="18.44140625" style="3" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="23.88671875" style="3" bestFit="1" customWidth="1"/>
     <col min="20" max="20" width="19" style="3" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="21.140625" style="3" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="13.7109375" style="3" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="12.85546875" style="3" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="21.7109375" style="3" customWidth="1"/>
-    <col min="25" max="25" width="20.42578125" style="21" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="20.42578125" style="26" customWidth="1"/>
-    <col min="27" max="27" width="20.42578125" style="3" customWidth="1"/>
-    <col min="28" max="28" width="24.7109375" style="3" bestFit="1" customWidth="1"/>
-    <col min="29" max="31" width="24.7109375" style="3" customWidth="1"/>
-    <col min="32" max="32" width="18.85546875" style="3" bestFit="1" customWidth="1"/>
-    <col min="33" max="36" width="18.85546875" style="3" customWidth="1"/>
-    <col min="37" max="37" width="13.85546875" style="3" bestFit="1" customWidth="1"/>
-    <col min="38" max="38" width="13" style="3" bestFit="1" customWidth="1"/>
-    <col min="39" max="39" width="16.85546875" style="3" bestFit="1" customWidth="1"/>
-    <col min="40" max="40" width="13" style="18" bestFit="1" customWidth="1"/>
-    <col min="41" max="41" width="13" style="21" customWidth="1"/>
-    <col min="42" max="42" width="17" style="26" bestFit="1" customWidth="1"/>
-    <col min="43" max="43" width="24.85546875" style="3" bestFit="1" customWidth="1"/>
-    <col min="44" max="16384" width="9.140625" style="3"/>
+    <col min="21" max="21" width="21.109375" style="3" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="13.6640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="12.88671875" style="3" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="21.6640625" style="3" customWidth="1"/>
+    <col min="25" max="25" width="20.44140625" style="21" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="20.44140625" style="26" customWidth="1"/>
+    <col min="27" max="27" width="20.44140625" style="3" customWidth="1"/>
+    <col min="28" max="28" width="24.6640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="29" max="31" width="24.6640625" style="3" customWidth="1"/>
+    <col min="32" max="35" width="18.5546875" style="1" customWidth="1"/>
+    <col min="36" max="36" width="18.88671875" style="3" bestFit="1" customWidth="1"/>
+    <col min="37" max="40" width="18.88671875" style="3" customWidth="1"/>
+    <col min="41" max="41" width="13.88671875" style="3" bestFit="1" customWidth="1"/>
+    <col min="42" max="42" width="13" style="3" bestFit="1" customWidth="1"/>
+    <col min="43" max="43" width="16.88671875" style="3" bestFit="1" customWidth="1"/>
+    <col min="44" max="44" width="13" style="18" bestFit="1" customWidth="1"/>
+    <col min="45" max="45" width="13" style="21" customWidth="1"/>
+    <col min="46" max="46" width="17" style="26" bestFit="1" customWidth="1"/>
+    <col min="47" max="47" width="24.88671875" style="3" bestFit="1" customWidth="1"/>
+    <col min="48" max="16384" width="9.109375" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:43" s="5" customFormat="1" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:47" s="5" customFormat="1" ht="16.8" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="5" t="s">
         <v>70</v>
       </c>
@@ -9170,47 +9253,63 @@
         <v>105</v>
       </c>
       <c r="AF1" s="5" t="s">
+        <v>141</v>
+      </c>
+      <c r="AG1" s="5" t="s">
+        <v>142</v>
+      </c>
+      <c r="AH1" s="5" t="s">
+        <v>143</v>
+      </c>
+      <c r="AI1" s="5" t="s">
+        <v>144</v>
+      </c>
+      <c r="AJ1" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="AG1" s="5" t="s">
+      <c r="AK1" s="5" t="s">
         <v>93</v>
       </c>
-      <c r="AH1" s="5" t="s">
+      <c r="AL1" s="5" t="s">
         <v>106</v>
       </c>
-      <c r="AI1" s="5" t="s">
+      <c r="AM1" s="5" t="s">
         <v>107</v>
       </c>
-      <c r="AJ1" s="5" t="s">
+      <c r="AN1" s="5" t="s">
         <v>108</v>
       </c>
-      <c r="AK1" s="5" t="s">
+      <c r="AO1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="AL1" s="5" t="s">
+      <c r="AP1" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="AM1" s="5" t="s">
+      <c r="AQ1" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="AN1" s="5" t="s">
+      <c r="AR1" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="AO1" s="20" t="s">
+      <c r="AS1" s="20" t="s">
         <v>15</v>
       </c>
-      <c r="AP1" s="25" t="s">
+      <c r="AT1" s="25" t="s">
         <v>109</v>
       </c>
-      <c r="AQ1" s="5" t="s">
+      <c r="AU1" s="5" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="2" spans="1:43" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
+    <row r="2" spans="1:47" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
   </sheetData>
-  <autoFilter ref="A1:AQ1" xr:uid="{00000000-0009-0000-0000-000006000000}"/>
+  <autoFilter ref="A1:AU1" xr:uid="{00000000-0009-0000-0000-000006000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
+  <headerFooter>
+    <oddHeader>&amp;C&amp;"Calibri"&amp;10&amp;K000000 Lockheed Martin Proprietary Information&amp;1#_x000D_</oddHeader>
+    <oddFooter>&amp;C_x000D_&amp;1#&amp;"Calibri"&amp;10&amp;K000000 Lockheed Martin Proprietary Information</oddFooter>
+  </headerFooter>
   <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
@@ -9218,22 +9317,22 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1:N2"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="13.8" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="20.7109375" style="7" customWidth="1"/>
-    <col min="2" max="3" width="25.7109375" style="7" customWidth="1"/>
-    <col min="4" max="4" width="20.7109375" style="7" customWidth="1"/>
-    <col min="5" max="5" width="25.7109375" style="7" customWidth="1"/>
-    <col min="6" max="7" width="15.7109375" style="7" customWidth="1"/>
-    <col min="8" max="8" width="13.140625" style="22" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.140625" style="27" bestFit="1" customWidth="1"/>
-    <col min="10" max="11" width="25.7109375" style="7" customWidth="1"/>
-    <col min="12" max="13" width="15.42578125" style="7" customWidth="1"/>
+    <col min="1" max="1" width="20.6640625" style="7" customWidth="1"/>
+    <col min="2" max="3" width="25.6640625" style="7" customWidth="1"/>
+    <col min="4" max="4" width="20.6640625" style="7" customWidth="1"/>
+    <col min="5" max="5" width="25.6640625" style="7" customWidth="1"/>
+    <col min="6" max="7" width="15.6640625" style="7" customWidth="1"/>
+    <col min="8" max="8" width="13.109375" style="22" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13.109375" style="27" bestFit="1" customWidth="1"/>
+    <col min="10" max="11" width="25.6640625" style="7" customWidth="1"/>
+    <col min="12" max="13" width="15.44140625" style="7" customWidth="1"/>
     <col min="14" max="14" width="11" style="7" customWidth="1"/>
-    <col min="15" max="16384" width="9.140625" style="7"/>
+    <col min="15" max="16384" width="9.109375" style="7"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" s="9" customFormat="1" ht="20.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:14" s="9" customFormat="1" ht="20.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="9" t="s">
         <v>27</v>
       </c>
@@ -9277,34 +9376,39 @@
         <v>112</v>
       </c>
     </row>
-    <row r="2" spans="1:14" ht="13.5" thickTop="1" x14ac:dyDescent="0.2"/>
+    <row r="2" spans="1:14" ht="14.4" thickTop="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
+  <headerFooter>
+    <oddHeader>&amp;C&amp;"Calibri"&amp;10&amp;K000000 Lockheed Martin Proprietary Information&amp;1#_x000D_</oddHeader>
+    <oddFooter>&amp;C_x000D_&amp;1#&amp;"Calibri"&amp;10&amp;K000000 Lockheed Martin Proprietary Information</oddFooter>
+  </headerFooter>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
-  <dimension ref="A1:N2"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:P2"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12" style="16" customWidth="1"/>
     <col min="2" max="2" width="24" style="16" customWidth="1"/>
-    <col min="3" max="3" width="25.5703125" style="16" customWidth="1"/>
-    <col min="4" max="4" width="10.5703125" style="16" customWidth="1"/>
-    <col min="5" max="6" width="10.5703125" style="16" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="10.5703125" style="16" customWidth="1"/>
-    <col min="8" max="8" width="20.42578125" style="16" customWidth="1"/>
-    <col min="9" max="9" width="18.140625" style="16" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="18.85546875" style="16" bestFit="1" customWidth="1"/>
-    <col min="11" max="12" width="10.7109375" style="17" customWidth="1"/>
-    <col min="13" max="13" width="20.7109375" style="24" customWidth="1"/>
-    <col min="14" max="14" width="20.7109375" style="29" customWidth="1"/>
-    <col min="15" max="16384" width="9.140625" style="16"/>
+    <col min="3" max="3" width="25.5546875" style="16" customWidth="1"/>
+    <col min="4" max="4" width="10.5546875" style="16" customWidth="1"/>
+    <col min="5" max="6" width="10.5546875" style="16" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.5546875" style="16" customWidth="1"/>
+    <col min="8" max="8" width="20.44140625" style="16" customWidth="1"/>
+    <col min="9" max="9" width="18.109375" style="16" bestFit="1" customWidth="1"/>
+    <col min="10" max="11" width="18.109375" style="16" customWidth="1"/>
+    <col min="12" max="12" width="18.88671875" style="16" bestFit="1" customWidth="1"/>
+    <col min="13" max="14" width="10.6640625" style="17" customWidth="1"/>
+    <col min="15" max="15" width="20.6640625" style="24" customWidth="1"/>
+    <col min="16" max="16" width="20.6640625" style="29" customWidth="1"/>
+    <col min="17" max="16384" width="9.109375" style="16"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" s="2" customFormat="1" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:16" s="2" customFormat="1" ht="16.8" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>2</v>
       </c>
@@ -9332,27 +9436,37 @@
       <c r="I1" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="J1" s="5" t="s">
+        <v>143</v>
+      </c>
+      <c r="K1" s="5" t="s">
+        <v>144</v>
+      </c>
+      <c r="L1" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="K1" s="2" t="s">
+      <c r="M1" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="L1" s="2" t="s">
+      <c r="N1" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="M1" s="23" t="s">
+      <c r="O1" s="23" t="s">
         <v>110</v>
       </c>
-      <c r="N1" s="28" t="s">
+      <c r="P1" s="28" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="2" spans="1:14" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
+    <row r="2" spans="1:16" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
   </sheetData>
-  <autoFilter ref="A1:N2" xr:uid="{00000000-0009-0000-0000-000008000000}"/>
+  <autoFilter ref="A1:P2" xr:uid="{00000000-0009-0000-0000-000008000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
+  <headerFooter>
+    <oddHeader>&amp;C&amp;"Calibri"&amp;10&amp;K000000 Lockheed Martin Proprietary Information&amp;1#_x000D_</oddHeader>
+    <oddFooter>&amp;C_x000D_&amp;1#&amp;"Calibri"&amp;10&amp;K000000 Lockheed Martin Proprietary Information</oddFooter>
+  </headerFooter>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
fixed template focus and A19
</commit_message>
<xml_diff>
--- a/GenBOE/GenBOE.Web/Templates/Export/WorkspaceDataMST.xlsx
+++ b/GenBOE/GenBOE.Web/Templates/Export/WorkspaceDataMST.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26130"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26731"/>
   <workbookPr showPivotChartFilter="1" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\e302876\proph\IES\GenBOE\GenBOE.Web\Templates\Export\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA71204E-83A7-40B4-A06D-78329F08D05A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B303C56-67D7-4CA4-969E-3E3728B93C9B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" firstSheet="5" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" firstSheet="5" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="BOE3 Pivot" sheetId="19" state="hidden" r:id="rId1"/>
@@ -53,11 +53,10 @@
   </definedNames>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="3" r:id="rId20"/>
-    <pivotCache cacheId="4" r:id="rId21"/>
-    <pivotCache cacheId="5" r:id="rId22"/>
+    <pivotCache cacheId="0" r:id="rId20"/>
+    <pivotCache cacheId="1" r:id="rId21"/>
+    <pivotCache cacheId="2" r:id="rId22"/>
   </pivotCaches>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -1184,7 +1183,7 @@
 </file>
 
 <file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="BOEs"/>
@@ -1265,7 +1264,7 @@
 </file>
 
 <file path=xl/externalLinks/externalLink2.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="Labor Types"/>
@@ -4355,7 +4354,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0000-000000000000}" name="PivotTable7" cacheId="3" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="3" minRefreshableVersion="3" showCalcMbrs="0" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="3" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0000-000000000000}" name="PivotTable7" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="3" minRefreshableVersion="3" showCalcMbrs="0" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="3" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
   <location ref="A3:N33" firstHeaderRow="1" firstDataRow="1" firstDataCol="14"/>
   <pivotFields count="14">
     <pivotField axis="axisRow" compact="0" outline="0" showAll="0" insertBlankRow="1" defaultSubtotal="0">
@@ -4704,7 +4703,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0200-000000000000}" name="PivotTable9" cacheId="4" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="3" minRefreshableVersion="3" showCalcMbrs="0" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="3" indent="0" compact="0" compactData="0" multipleFieldFilters="0" rowHeaderCaption="Type">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0200-000000000000}" name="PivotTable9" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="3" minRefreshableVersion="3" showCalcMbrs="0" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="3" indent="0" compact="0" compactData="0" multipleFieldFilters="0" rowHeaderCaption="Type">
   <location ref="A3:H11" firstHeaderRow="1" firstDataRow="1" firstDataCol="8"/>
   <pivotFields count="19">
     <pivotField axis="axisRow" compact="0" outline="0" showAll="0" defaultSubtotal="0">
@@ -4913,7 +4912,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0300-000000000000}" name="PivotTable4" cacheId="5" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" missingCaption="_" updatedVersion="3" minRefreshableVersion="3" showCalcMbrs="0" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="3" indent="0" compact="0" compactData="0" multipleFieldFilters="0" rowHeaderCaption="BOE ID">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0300-000000000000}" name="PivotTable4" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" missingCaption="_" updatedVersion="3" minRefreshableVersion="3" showCalcMbrs="0" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="3" indent="0" compact="0" compactData="0" multipleFieldFilters="0" rowHeaderCaption="BOE ID">
   <location ref="A3:T33" firstHeaderRow="1" firstDataRow="1" firstDataCol="20"/>
   <pivotFields count="20">
     <pivotField axis="axisRow" compact="0" outline="0" showAll="0" insertBlankRow="1" defaultSubtotal="0">
@@ -5356,9 +5355,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -5396,9 +5395,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
-        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -5431,26 +5430,9 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -5483,26 +5465,9 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -6496,59 +6461,61 @@
       </c>
     </row>
     <row r="5" spans="1:1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="10"/>
+      <c r="A5" s="10" t="s">
+        <v>79</v>
+      </c>
     </row>
     <row r="6" spans="1:1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="10" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
     </row>
     <row r="7" spans="1:1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="10" t="s">
-        <v>80</v>
+      <c r="A7" s="11" t="s">
+        <v>81</v>
       </c>
     </row>
     <row r="8" spans="1:1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="11" t="s">
-        <v>81</v>
+        <v>122</v>
       </c>
     </row>
     <row r="9" spans="1:1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="11" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
     </row>
     <row r="10" spans="1:1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="11" t="s">
-        <v>123</v>
+      <c r="A10" s="12" t="s">
+        <v>121</v>
       </c>
     </row>
     <row r="11" spans="1:1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="12" t="s">
-        <v>121</v>
+        <v>82</v>
       </c>
     </row>
     <row r="12" spans="1:1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="12" t="s">
-        <v>82</v>
+      <c r="A12" s="10" t="s">
+        <v>96</v>
       </c>
     </row>
     <row r="13" spans="1:1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="10" t="s">
-        <v>96</v>
+      <c r="A13" s="19" t="s">
+        <v>97</v>
       </c>
     </row>
     <row r="14" spans="1:1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="19" t="s">
-        <v>97</v>
+        <v>139</v>
       </c>
     </row>
     <row r="15" spans="1:1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="19" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="16" spans="1:1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3"/>
+      <c r="A15" s="19"/>
+    </row>
+    <row r="16" spans="1:1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="19"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -9471,28 +9438,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance">
-  <documentManagement>
-    <Unity_Description xmlns="D75E00DB-06CE-4005-B397-8C0860A4229B" xsi:nil="true"/>
-    <Unity_Tag xmlns="D75E00DB-06CE-4005-B397-8C0860A4229B" xsi:nil="true"/>
-    <Capabilities xmlns="d75e00db-06ce-4005-b397-8c0860a4229b" xsi:nil="true"/>
-    <SipLabel xmlns="372b77af-8063-48a8-888c-73c0edf01dea">
-      <Value>2</Value>
-    </SipLabel>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Custom Document" ma:contentTypeID="0x010100E6322E8F405D4D9EA89D8C83B7E1048B001BB96E1BE0ACBB41BF00782ED0412411" ma:contentTypeVersion="3" ma:contentTypeDescription="Custom Document" ma:contentTypeScope="" ma:versionID="3c14126572fa3c0d4c677ac1f3ba4426">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="D75E00DB-06CE-4005-B397-8C0860A4229B" xmlns:ns3="372b77af-8063-48a8-888c-73c0edf01dea" xmlns:ns4="d75e00db-06ce-4005-b397-8c0860a4229b" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="9e89026a025b72b85b9543506e7af3e1" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="D75E00DB-06CE-4005-B397-8C0860A4229B"/>
@@ -9595,32 +9540,29 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2653FDDC-5C81-4B5A-A42F-7A63208AFFF7}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{268822B0-DCAE-4D2C-8340-AB7554C48D72}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="D75E00DB-06CE-4005-B397-8C0860A4229B"/>
-    <ds:schemaRef ds:uri="372b77af-8063-48a8-888c-73c0edf01dea"/>
-    <ds:schemaRef ds:uri="d75e00db-06ce-4005-b397-8c0860a4229b"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance">
+  <documentManagement>
+    <Unity_Description xmlns="D75E00DB-06CE-4005-B397-8C0860A4229B" xsi:nil="true"/>
+    <Unity_Tag xmlns="D75E00DB-06CE-4005-B397-8C0860A4229B" xsi:nil="true"/>
+    <Capabilities xmlns="d75e00db-06ce-4005-b397-8c0860a4229b" xsi:nil="true"/>
+    <SipLabel xmlns="372b77af-8063-48a8-888c-73c0edf01dea">
+      <Value>2</Value>
+    </SipLabel>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1DE4120D-B400-435F-B862-B3B8683830A5}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -9637,4 +9579,29 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/internal/2005/internalDocumentation"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2653FDDC-5C81-4B5A-A42F-7A63208AFFF7}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{268822B0-DCAE-4D2C-8340-AB7554C48D72}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="D75E00DB-06CE-4005-B397-8C0860A4229B"/>
+    <ds:schemaRef ds:uri="372b77af-8063-48a8-888c-73c0edf01dea"/>
+    <ds:schemaRef ds:uri="d75e00db-06ce-4005-b397-8c0860a4229b"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
PROPH-1778: Add rationale field into MOQ Types in Workspace Data Exporter
</commit_message>
<xml_diff>
--- a/GenBOE/GenBOE.Web/Templates/Export/WorkspaceDataMST.xlsx
+++ b/GenBOE/GenBOE.Web/Templates/Export/WorkspaceDataMST.xlsx
@@ -5,12 +5,12 @@
   <workbookPr showPivotChartFilter="1" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\e302876\proph\IES\GenBOE\GenBOE.Web\Templates\Export\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\gitBoe\GenBOE\GenBOE.Web\Templates\Export\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B303C56-67D7-4CA4-969E-3E3728B93C9B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37A2B01A-8844-4C24-8B34-A14A32448E44}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" firstSheet="5" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5190" yWindow="30" windowWidth="34035" windowHeight="21570" firstSheet="5" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="BOE3 Pivot" sheetId="19" state="hidden" r:id="rId1"/>
@@ -53,9 +53,9 @@
   </definedNames>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="0" r:id="rId20"/>
-    <pivotCache cacheId="1" r:id="rId21"/>
-    <pivotCache cacheId="2" r:id="rId22"/>
+    <pivotCache cacheId="3" r:id="rId20"/>
+    <pivotCache cacheId="4" r:id="rId21"/>
+    <pivotCache cacheId="5" r:id="rId22"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -320,7 +320,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="887" uniqueCount="145">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="888" uniqueCount="146">
   <si>
     <t>Start Date</t>
   </si>
@@ -755,6 +755,9 @@
   </si>
   <si>
     <t>BRC Segment Region</t>
+  </si>
+  <si>
+    <t>Rationale</t>
   </si>
 </sst>
 </file>
@@ -4354,7 +4357,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0000-000000000000}" name="PivotTable7" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="3" minRefreshableVersion="3" showCalcMbrs="0" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="3" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0000-000000000000}" name="PivotTable7" cacheId="3" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="3" minRefreshableVersion="3" showCalcMbrs="0" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="3" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
   <location ref="A3:N33" firstHeaderRow="1" firstDataRow="1" firstDataCol="14"/>
   <pivotFields count="14">
     <pivotField axis="axisRow" compact="0" outline="0" showAll="0" insertBlankRow="1" defaultSubtotal="0">
@@ -4703,7 +4706,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0200-000000000000}" name="PivotTable9" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="3" minRefreshableVersion="3" showCalcMbrs="0" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="3" indent="0" compact="0" compactData="0" multipleFieldFilters="0" rowHeaderCaption="Type">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0200-000000000000}" name="PivotTable9" cacheId="4" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="3" minRefreshableVersion="3" showCalcMbrs="0" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="3" indent="0" compact="0" compactData="0" multipleFieldFilters="0" rowHeaderCaption="Type">
   <location ref="A3:H11" firstHeaderRow="1" firstDataRow="1" firstDataCol="8"/>
   <pivotFields count="19">
     <pivotField axis="axisRow" compact="0" outline="0" showAll="0" defaultSubtotal="0">
@@ -4912,7 +4915,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0300-000000000000}" name="PivotTable4" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" missingCaption="_" updatedVersion="3" minRefreshableVersion="3" showCalcMbrs="0" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="3" indent="0" compact="0" compactData="0" multipleFieldFilters="0" rowHeaderCaption="BOE ID">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0300-000000000000}" name="PivotTable4" cacheId="5" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" missingCaption="_" updatedVersion="3" minRefreshableVersion="3" showCalcMbrs="0" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="3" indent="0" compact="0" compactData="0" multipleFieldFilters="0" rowHeaderCaption="BOE ID">
   <location ref="A3:T33" firstHeaderRow="1" firstDataRow="1" firstDataCol="20"/>
   <pivotFields count="20">
     <pivotField axis="axisRow" compact="0" outline="0" showAll="0" insertBlankRow="1" defaultSubtotal="0">
@@ -5642,25 +5645,25 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A3:N32"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="22.5546875" customWidth="1"/>
-    <col min="2" max="2" width="11.44140625" customWidth="1"/>
-    <col min="3" max="3" width="10.5546875" customWidth="1"/>
+    <col min="1" max="1" width="22.5703125" customWidth="1"/>
+    <col min="2" max="2" width="11.42578125" customWidth="1"/>
+    <col min="3" max="3" width="10.5703125" customWidth="1"/>
     <col min="4" max="4" width="15" customWidth="1"/>
-    <col min="5" max="5" width="11.6640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.88671875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13.109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.44140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.42578125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="17" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="12" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="11.109375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="11.140625" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="15" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="11.44140625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="11.42578125" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="15" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
         <v>33</v>
       </c>
@@ -5704,7 +5707,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>59</v>
       </c>
@@ -5748,7 +5751,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
       <c r="G6" t="s">
         <v>57</v>
       </c>
@@ -5774,7 +5777,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
       <c r="H8" t="s">
         <v>43</v>
       </c>
@@ -5797,7 +5800,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
       <c r="D10" t="s">
         <v>62</v>
       </c>
@@ -5832,7 +5835,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
       <c r="G12" t="s">
         <v>57</v>
       </c>
@@ -5858,7 +5861,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:14" x14ac:dyDescent="0.25">
       <c r="H14" t="s">
         <v>43</v>
       </c>
@@ -5881,7 +5884,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:14" x14ac:dyDescent="0.25">
       <c r="D16" t="s">
         <v>57</v>
       </c>
@@ -5916,7 +5919,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="18" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>60</v>
       </c>
@@ -5960,7 +5963,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="20" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:14" x14ac:dyDescent="0.25">
       <c r="G20" t="s">
         <v>57</v>
       </c>
@@ -5986,7 +5989,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="22" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:14" x14ac:dyDescent="0.25">
       <c r="H22" t="s">
         <v>43</v>
       </c>
@@ -6009,7 +6012,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="24" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:14" x14ac:dyDescent="0.25">
       <c r="H24" t="s">
         <v>55</v>
       </c>
@@ -6032,7 +6035,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="26" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:14" x14ac:dyDescent="0.25">
       <c r="H26" t="s">
         <v>51</v>
       </c>
@@ -6055,7 +6058,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="28" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:14" x14ac:dyDescent="0.25">
       <c r="D28" t="s">
         <v>64</v>
       </c>
@@ -6090,7 +6093,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="30" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:14" x14ac:dyDescent="0.25">
       <c r="G30" t="s">
         <v>57</v>
       </c>
@@ -6116,7 +6119,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="32" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:14" x14ac:dyDescent="0.25">
       <c r="D32" t="s">
         <v>62</v>
       </c>
@@ -6163,17 +6166,18 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3DA6D2FB-3F32-46E9-963C-DCD2D761F967}">
-  <dimension ref="A1:F2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:G2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.44140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.42578125" bestFit="1" customWidth="1"/>
     <col min="4" max="5" width="24" customWidth="1"/>
-    <col min="6" max="6" width="40.88671875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="40.85546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="64.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="16.8" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:7" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
         <v>70</v>
       </c>
@@ -6192,8 +6196,11 @@
       <c r="F1" s="5" t="s">
         <v>84</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
+      <c r="G1" s="5" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <autoFilter ref="A1:F1" xr:uid="{1E7471F8-87B8-4A9F-A5C2-80CE50F530C1}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -6207,29 +6214,29 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EDDB750B-2EAA-4C67-B526-87C6863613C3}">
   <dimension ref="A1:R2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.44140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.42578125" style="1" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="24" style="1" customWidth="1"/>
-    <col min="5" max="5" width="42.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="15.88671875" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="18.88671875" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="28.88671875" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="21.109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="42.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="18.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="28.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="21.140625" style="1" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="23" style="1" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="42" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="41.109375" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="41.109375" style="32" customWidth="1"/>
-    <col min="14" max="14" width="35.33203125" style="32" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="57.88671875" style="1" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="61.44140625" style="32" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="28.44140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="27.33203125" style="1" customWidth="1"/>
+    <col min="12" max="12" width="41.140625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="41.140625" style="32" customWidth="1"/>
+    <col min="14" max="14" width="35.28515625" style="32" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="57.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="61.42578125" style="32" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="28.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="27.28515625" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" s="5" customFormat="1" ht="16.8" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:18" s="5" customFormat="1" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
         <v>70</v>
       </c>
@@ -6285,7 +6292,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="2" spans="1:18" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
+    <row r="2" spans="1:18" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <autoFilter ref="A1:Q1" xr:uid="{EDDB750B-2EAA-4C67-B526-87C6863613C3}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -6300,15 +6307,15 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
   <dimension ref="A1:E2"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="13.8" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="30.6640625" style="6" hidden="1" customWidth="1"/>
-    <col min="2" max="4" width="30.6640625" style="8" customWidth="1"/>
-    <col min="5" max="5" width="33.109375" style="7" customWidth="1"/>
-    <col min="6" max="16384" width="9.109375" style="7"/>
+    <col min="1" max="1" width="30.7109375" style="6" hidden="1" customWidth="1"/>
+    <col min="2" max="4" width="30.7109375" style="8" customWidth="1"/>
+    <col min="5" max="5" width="33.140625" style="7" customWidth="1"/>
+    <col min="6" max="16384" width="9.140625" style="7"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="5" customFormat="1" ht="20.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" s="5" customFormat="1" ht="20.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
         <v>68</v>
       </c>
@@ -6325,7 +6332,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="14.4" thickTop="1" x14ac:dyDescent="0.3"/>
+    <row r="2" spans="1:5" ht="13.5" thickTop="1" x14ac:dyDescent="0.2"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -6340,16 +6347,16 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
   <dimension ref="A1:E2"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="13.8" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="13.109375" style="6" hidden="1" customWidth="1"/>
-    <col min="2" max="2" width="30.6640625" style="8" customWidth="1"/>
-    <col min="3" max="3" width="50.6640625" style="8" customWidth="1"/>
-    <col min="4" max="5" width="20.6640625" style="8" customWidth="1"/>
-    <col min="6" max="16384" width="9.109375" style="7"/>
+    <col min="1" max="1" width="13.140625" style="6" hidden="1" customWidth="1"/>
+    <col min="2" max="2" width="30.7109375" style="8" customWidth="1"/>
+    <col min="3" max="3" width="50.7109375" style="8" customWidth="1"/>
+    <col min="4" max="5" width="20.7109375" style="8" customWidth="1"/>
+    <col min="6" max="16384" width="9.140625" style="7"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="5" customFormat="1" ht="20.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" s="5" customFormat="1" ht="20.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
         <v>98</v>
       </c>
@@ -6366,7 +6373,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="14.4" thickTop="1" x14ac:dyDescent="0.3"/>
+    <row r="2" spans="1:5" ht="13.5" thickTop="1" x14ac:dyDescent="0.2"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -6381,20 +6388,20 @@
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0B00-000000000000}">
   <dimension ref="A1:I2"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="18.88671875" style="15" customWidth="1"/>
-    <col min="2" max="3" width="35.6640625" style="15" customWidth="1"/>
-    <col min="4" max="4" width="26.109375" style="15" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.5546875" style="15" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="22.109375" style="15" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="10.88671875" style="15" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="13.109375" style="15" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="21.88671875" style="15" bestFit="1" customWidth="1"/>
-    <col min="10" max="16384" width="9.109375" style="15"/>
+    <col min="1" max="1" width="18.85546875" style="15" customWidth="1"/>
+    <col min="2" max="3" width="35.7109375" style="15" customWidth="1"/>
+    <col min="4" max="4" width="26.140625" style="15" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.5703125" style="15" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="22.140625" style="15" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.85546875" style="15" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.140625" style="15" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="21.85546875" style="15" bestFit="1" customWidth="1"/>
+    <col min="10" max="16384" width="9.140625" style="15"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" s="14" customFormat="1" ht="16.8" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:9" s="14" customFormat="1" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>71</v>
       </c>
@@ -6423,7 +6430,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="2" spans="1:9" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
+    <row r="2" spans="1:9" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -6437,83 +6444,83 @@
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0C00-000000000000}">
   <dimension ref="A1:A16"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="28" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="82.109375" style="1" customWidth="1"/>
-    <col min="3" max="16384" width="9.109375" style="1"/>
+    <col min="2" max="2" width="82.140625" style="1" customWidth="1"/>
+    <col min="3" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" hidden="1" x14ac:dyDescent="0.3"/>
-    <row r="2" spans="1:1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:1" hidden="1" x14ac:dyDescent="0.25"/>
+    <row r="2" spans="1:1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="10" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="3" spans="1:1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="10" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="4" spans="1:1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="10" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="5" spans="1:1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="6" spans="1:1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="7" spans="1:1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="11" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="8" spans="1:1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="11" t="s">
         <v>122</v>
       </c>
     </row>
-    <row r="9" spans="1:1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="11" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="10" spans="1:1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="12" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="11" spans="1:1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="12" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="12" spans="1:1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="10" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="13" spans="1:1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="19" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="14" spans="1:1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="19" t="s">
         <v>139</v>
       </c>
     </row>
-    <row r="15" spans="1:1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="19"/>
     </row>
-    <row r="16" spans="1:1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="19"/>
     </row>
   </sheetData>
@@ -6529,30 +6536,30 @@
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1E9E49D2-B4A1-426D-8F6A-B85DD2E6A5AA}">
   <dimension ref="A1:AA7"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
-    <col min="2" max="2" width="7.109375" customWidth="1"/>
-    <col min="3" max="3" width="29.44140625" customWidth="1"/>
-    <col min="4" max="4" width="26.88671875" customWidth="1"/>
-    <col min="5" max="5" width="12.33203125" customWidth="1"/>
+    <col min="2" max="2" width="7.140625" customWidth="1"/>
+    <col min="3" max="3" width="29.42578125" customWidth="1"/>
+    <col min="4" max="4" width="26.85546875" customWidth="1"/>
+    <col min="5" max="5" width="12.28515625" customWidth="1"/>
     <col min="6" max="6" width="16" customWidth="1"/>
-    <col min="7" max="7" width="20.5546875" customWidth="1"/>
-    <col min="8" max="8" width="10.5546875" style="39" customWidth="1"/>
-    <col min="9" max="11" width="8.88671875" style="39"/>
-    <col min="12" max="12" width="12.88671875" style="39" customWidth="1"/>
-    <col min="13" max="13" width="8.88671875" style="39"/>
-    <col min="14" max="14" width="15.5546875" style="56" customWidth="1"/>
-    <col min="15" max="15" width="19.109375" style="56" customWidth="1"/>
-    <col min="16" max="16" width="15.6640625" style="56" customWidth="1"/>
-    <col min="17" max="17" width="19.33203125" style="56" customWidth="1"/>
-    <col min="18" max="18" width="13.6640625" style="56" customWidth="1"/>
-    <col min="19" max="19" width="17.88671875" style="56" customWidth="1"/>
-    <col min="20" max="20" width="17.6640625" customWidth="1"/>
-    <col min="21" max="21" width="15.33203125" customWidth="1"/>
+    <col min="7" max="7" width="20.5703125" customWidth="1"/>
+    <col min="8" max="8" width="10.5703125" style="39" customWidth="1"/>
+    <col min="9" max="11" width="8.85546875" style="39"/>
+    <col min="12" max="12" width="12.85546875" style="39" customWidth="1"/>
+    <col min="13" max="13" width="8.85546875" style="39"/>
+    <col min="14" max="14" width="15.5703125" style="56" customWidth="1"/>
+    <col min="15" max="15" width="19.140625" style="56" customWidth="1"/>
+    <col min="16" max="16" width="15.7109375" style="56" customWidth="1"/>
+    <col min="17" max="17" width="19.28515625" style="56" customWidth="1"/>
+    <col min="18" max="18" width="13.7109375" style="56" customWidth="1"/>
+    <col min="19" max="19" width="17.85546875" style="56" customWidth="1"/>
+    <col min="20" max="20" width="17.7109375" customWidth="1"/>
+    <col min="21" max="21" width="15.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:27" s="44" customFormat="1" ht="19.2" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:27" s="44" customFormat="1" ht="20.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="40"/>
       <c r="B1" s="41"/>
       <c r="C1" s="41"/>
@@ -6580,7 +6587,7 @@
       <c r="Z1" s="53"/>
       <c r="AA1" s="53"/>
     </row>
-    <row r="2" spans="1:27" s="44" customFormat="1" ht="18.600000000000001" thickTop="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:27" s="44" customFormat="1" ht="19.5" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A2" s="40"/>
       <c r="B2" s="41"/>
       <c r="C2" s="41"/>
@@ -6609,7 +6616,7 @@
       <c r="Z2" s="53"/>
       <c r="AA2" s="53"/>
     </row>
-    <row r="3" spans="1:27" s="44" customFormat="1" ht="18" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:27" s="44" customFormat="1" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A3" s="40"/>
       <c r="B3" s="41"/>
       <c r="C3" s="41"/>
@@ -6638,7 +6645,7 @@
       <c r="Z3" s="53"/>
       <c r="AA3" s="53"/>
     </row>
-    <row r="4" spans="1:27" s="44" customFormat="1" ht="18" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:27" s="44" customFormat="1" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A4" s="40"/>
       <c r="B4" s="41"/>
       <c r="C4" s="41"/>
@@ -6667,7 +6674,7 @@
       <c r="Z4" s="53"/>
       <c r="AA4" s="53"/>
     </row>
-    <row r="5" spans="1:27" s="44" customFormat="1" ht="18" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:27" s="44" customFormat="1" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A5" s="54"/>
       <c r="B5" s="41"/>
       <c r="C5" s="41"/>
@@ -6696,7 +6703,7 @@
       <c r="Z5" s="53"/>
       <c r="AA5" s="53"/>
     </row>
-    <row r="6" spans="1:27" s="44" customFormat="1" ht="18" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:27" s="44" customFormat="1" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A6" s="54"/>
       <c r="B6" s="55"/>
       <c r="C6" s="55"/>
@@ -6725,7 +6732,7 @@
       <c r="Z6" s="53"/>
       <c r="AA6" s="53"/>
     </row>
-    <row r="7" spans="1:27" s="54" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:27" s="54" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="H7" s="42"/>
       <c r="I7" s="42"/>
       <c r="J7" s="42"/>
@@ -6754,29 +6761,29 @@
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00BB237A-2FF2-450F-81EE-9A098F6C7133}">
   <dimension ref="A1:AA6"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.6640625" style="57" customWidth="1"/>
-    <col min="2" max="2" width="7.109375" style="57" customWidth="1"/>
-    <col min="3" max="3" width="29.44140625" style="57" customWidth="1"/>
-    <col min="4" max="4" width="26.88671875" style="57" customWidth="1"/>
-    <col min="5" max="5" width="12.33203125" style="57" customWidth="1"/>
+    <col min="1" max="1" width="11.7109375" style="57" customWidth="1"/>
+    <col min="2" max="2" width="7.140625" style="57" customWidth="1"/>
+    <col min="3" max="3" width="29.42578125" style="57" customWidth="1"/>
+    <col min="4" max="4" width="26.85546875" style="57" customWidth="1"/>
+    <col min="5" max="5" width="12.28515625" style="57" customWidth="1"/>
     <col min="6" max="6" width="16" style="57" customWidth="1"/>
-    <col min="7" max="7" width="20.5546875" style="57" customWidth="1"/>
-    <col min="8" max="8" width="10.5546875" style="58" customWidth="1"/>
-    <col min="9" max="13" width="9.109375" style="58"/>
-    <col min="14" max="14" width="15.5546875" style="56" customWidth="1"/>
-    <col min="15" max="15" width="24.5546875" style="56" customWidth="1"/>
-    <col min="16" max="16" width="15.6640625" style="56" customWidth="1"/>
-    <col min="17" max="17" width="19.33203125" style="56" customWidth="1"/>
-    <col min="18" max="18" width="13.6640625" style="56" customWidth="1"/>
-    <col min="19" max="19" width="17.88671875" style="56" customWidth="1"/>
-    <col min="20" max="20" width="17.6640625" style="56" customWidth="1"/>
-    <col min="21" max="21" width="15.33203125" style="56" customWidth="1"/>
-    <col min="22" max="16384" width="9.109375" style="59"/>
+    <col min="7" max="7" width="20.5703125" style="57" customWidth="1"/>
+    <col min="8" max="8" width="10.5703125" style="58" customWidth="1"/>
+    <col min="9" max="13" width="9.140625" style="58"/>
+    <col min="14" max="14" width="15.5703125" style="56" customWidth="1"/>
+    <col min="15" max="15" width="24.5703125" style="56" customWidth="1"/>
+    <col min="16" max="16" width="15.7109375" style="56" customWidth="1"/>
+    <col min="17" max="17" width="19.28515625" style="56" customWidth="1"/>
+    <col min="18" max="18" width="13.7109375" style="56" customWidth="1"/>
+    <col min="19" max="19" width="17.85546875" style="56" customWidth="1"/>
+    <col min="20" max="20" width="17.7109375" style="56" customWidth="1"/>
+    <col min="21" max="21" width="15.28515625" style="56" customWidth="1"/>
+    <col min="22" max="16384" width="9.140625" style="59"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:27" s="51" customFormat="1" ht="19.2" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:27" s="51" customFormat="1" ht="20.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="41"/>
       <c r="B1" s="41"/>
       <c r="C1" s="41"/>
@@ -6805,7 +6812,7 @@
       <c r="Z1" s="50"/>
       <c r="AA1" s="50"/>
     </row>
-    <row r="2" spans="1:27" s="51" customFormat="1" ht="18.600000000000001" thickTop="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:27" s="51" customFormat="1" ht="19.5" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A2" s="41"/>
       <c r="B2" s="41"/>
       <c r="C2" s="41"/>
@@ -6834,7 +6841,7 @@
       <c r="Z2" s="50"/>
       <c r="AA2" s="50"/>
     </row>
-    <row r="3" spans="1:27" s="51" customFormat="1" ht="18" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:27" s="51" customFormat="1" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A3" s="41"/>
       <c r="B3" s="41"/>
       <c r="C3" s="41"/>
@@ -6863,7 +6870,7 @@
       <c r="Z3" s="50"/>
       <c r="AA3" s="50"/>
     </row>
-    <row r="4" spans="1:27" s="51" customFormat="1" ht="18" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:27" s="51" customFormat="1" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A4" s="41"/>
       <c r="B4" s="41"/>
       <c r="C4" s="41"/>
@@ -6892,7 +6899,7 @@
       <c r="Z4" s="50"/>
       <c r="AA4" s="50"/>
     </row>
-    <row r="5" spans="1:27" s="51" customFormat="1" ht="18" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:27" s="51" customFormat="1" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A5" s="41"/>
       <c r="B5" s="41"/>
       <c r="C5" s="41"/>
@@ -6921,7 +6928,7 @@
       <c r="Z5" s="50"/>
       <c r="AA5" s="50"/>
     </row>
-    <row r="6" spans="1:27" s="44" customFormat="1" ht="18" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:27" s="44" customFormat="1" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A6" s="55"/>
       <c r="B6" s="55"/>
       <c r="C6" s="55"/>
@@ -6962,28 +6969,28 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:N16"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="16.88671875" style="3" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.44140625" style="3" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.5546875" style="3" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.44140625" style="3" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.6640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.88671875" style="3" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="15.44140625" style="3" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="13.109375" style="3" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="18.88671875" style="3" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="13.88671875" style="3" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.85546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.42578125" style="3" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.5703125" style="3" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.42578125" style="3" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.7109375" style="3" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.85546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.42578125" style="3" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.140625" style="3" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="18.85546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="13.85546875" style="3" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="13" style="3" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="16.88671875" style="3" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="16.85546875" style="3" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="13" style="3" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="17" style="3" bestFit="1" customWidth="1"/>
-    <col min="15" max="17" width="13.5546875" style="3" customWidth="1"/>
-    <col min="18" max="18" width="15.44140625" style="3" bestFit="1" customWidth="1"/>
-    <col min="19" max="16384" width="9.109375" style="3"/>
+    <col min="15" max="17" width="13.5703125" style="3" customWidth="1"/>
+    <col min="18" max="18" width="15.42578125" style="3" bestFit="1" customWidth="1"/>
+    <col min="19" max="16384" width="9.140625" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="16.8" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:14" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>33</v>
       </c>
@@ -7027,7 +7034,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="2" spans="1:14" ht="15" thickTop="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:14" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>59</v>
       </c>
@@ -7038,7 +7045,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>59</v>
       </c>
@@ -7061,7 +7068,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>59</v>
       </c>
@@ -7102,7 +7109,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
         <v>59</v>
       </c>
@@ -7143,7 +7150,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
         <v>59</v>
       </c>
@@ -7166,7 +7173,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
         <v>59</v>
       </c>
@@ -7207,7 +7214,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
         <v>59</v>
       </c>
@@ -7248,7 +7255,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
         <v>60</v>
       </c>
@@ -7268,7 +7275,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>60</v>
       </c>
@@ -7291,7 +7298,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
         <v>60</v>
       </c>
@@ -7332,7 +7339,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>60</v>
       </c>
@@ -7373,7 +7380,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
         <v>60</v>
       </c>
@@ -7414,7 +7421,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
         <v>60</v>
       </c>
@@ -7455,7 +7462,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
         <v>60</v>
       </c>
@@ -7478,7 +7485,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
         <v>60</v>
       </c>
@@ -7533,20 +7540,20 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A3:H11"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="7.5546875" customWidth="1"/>
-    <col min="2" max="2" width="8.88671875" customWidth="1"/>
-    <col min="3" max="3" width="11.88671875" customWidth="1"/>
-    <col min="4" max="4" width="8.6640625" customWidth="1"/>
-    <col min="5" max="5" width="11.6640625" customWidth="1"/>
-    <col min="6" max="6" width="11.44140625" customWidth="1"/>
-    <col min="7" max="7" width="10.5546875" customWidth="1"/>
-    <col min="8" max="8" width="9.44140625" customWidth="1"/>
+    <col min="1" max="1" width="7.5703125" customWidth="1"/>
+    <col min="2" max="2" width="8.85546875" customWidth="1"/>
+    <col min="3" max="3" width="11.85546875" customWidth="1"/>
+    <col min="4" max="4" width="8.7109375" customWidth="1"/>
+    <col min="5" max="5" width="11.7109375" customWidth="1"/>
+    <col min="6" max="6" width="11.42578125" customWidth="1"/>
+    <col min="7" max="7" width="10.5703125" customWidth="1"/>
+    <col min="8" max="8" width="9.42578125" customWidth="1"/>
     <col min="9" max="19" width="15" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
         <v>26</v>
       </c>
@@ -7572,7 +7579,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>33</v>
       </c>
@@ -7598,7 +7605,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
         <v>45</v>
       </c>
@@ -7606,7 +7613,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>12</v>
       </c>
@@ -7632,12 +7639,12 @@
         <v>38</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="H7" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B8" t="s">
         <v>45</v>
       </c>
@@ -7645,7 +7652,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>34</v>
       </c>
@@ -7671,12 +7678,12 @@
         <v>38</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="H10" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B11" t="s">
         <v>45</v>
       </c>
@@ -7697,29 +7704,29 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A3:T32"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="22.44140625" customWidth="1"/>
-    <col min="2" max="2" width="12.44140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.88671875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.6640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.44140625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.5546875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="9.44140625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.5546875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="11.6640625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="10.88671875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.109375" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="11.44140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="22.42578125" customWidth="1"/>
+    <col min="2" max="2" width="12.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="13.140625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="11.42578125" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="17" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="12" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.109375" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.140625" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="15" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="11.44140625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="11.42578125" bestFit="1" customWidth="1"/>
     <col min="20" max="20" width="15" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
         <v>70</v>
       </c>
@@ -7781,7 +7788,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="4" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>58</v>
       </c>
@@ -7843,7 +7850,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="6" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:20" x14ac:dyDescent="0.25">
       <c r="B6" t="s">
         <v>34</v>
       </c>
@@ -7902,7 +7909,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="8" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:20" x14ac:dyDescent="0.25">
       <c r="I8" t="s">
         <v>40</v>
       </c>
@@ -7940,7 +7947,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="10" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:20" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
         <v>12</v>
       </c>
@@ -7999,7 +8006,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="12" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:20" x14ac:dyDescent="0.25">
       <c r="R12" t="s">
         <v>20</v>
       </c>
@@ -8010,7 +8017,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="14" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:20" x14ac:dyDescent="0.25">
       <c r="N14" t="s">
         <v>43</v>
       </c>
@@ -8033,7 +8040,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="16" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:20" x14ac:dyDescent="0.25">
       <c r="O16" t="s">
         <v>53</v>
       </c>
@@ -8053,7 +8060,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="18" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>45</v>
       </c>
@@ -8115,7 +8122,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="20" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:20" x14ac:dyDescent="0.25">
       <c r="B20" t="s">
         <v>34</v>
       </c>
@@ -8174,7 +8181,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="22" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:20" x14ac:dyDescent="0.25">
       <c r="I22" t="s">
         <v>49</v>
       </c>
@@ -8212,7 +8219,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="24" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:20" x14ac:dyDescent="0.25">
       <c r="B24" t="s">
         <v>12</v>
       </c>
@@ -8271,7 +8278,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="26" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:20" x14ac:dyDescent="0.25">
       <c r="O26" t="s">
         <v>52</v>
       </c>
@@ -8291,7 +8298,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="28" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:20" x14ac:dyDescent="0.25">
       <c r="N28" t="s">
         <v>43</v>
       </c>
@@ -8314,7 +8321,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="30" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:20" x14ac:dyDescent="0.25">
       <c r="N30" t="s">
         <v>55</v>
       </c>
@@ -8337,7 +8344,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="32" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:20" x14ac:dyDescent="0.25">
       <c r="N32" t="s">
         <v>51</v>
       </c>
@@ -8373,33 +8380,33 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:T16"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.109375" style="3"/>
-    <col min="2" max="3" width="10.5546875" style="3" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.5546875" style="3" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.5546875" style="3" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.5546875" style="3" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13.44140625" style="3" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="12.5546875" style="3" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="11.44140625" style="3" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="13.5546875" style="3" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="13.6640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="12.88671875" style="3" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="15.44140625" style="3" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="13.109375" style="3" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="18.88671875" style="3" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="13.88671875" style="3" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.140625" style="3"/>
+    <col min="2" max="3" width="10.5703125" style="3" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.5703125" style="3" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.5703125" style="3" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.5703125" style="3" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.42578125" style="3" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12.5703125" style="3" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="11.42578125" style="3" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="13.5703125" style="3" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="13.7109375" style="3" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="12.85546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="15.42578125" style="3" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="13.140625" style="3" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="18.85546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="13.85546875" style="3" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="13" style="3" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="16.88671875" style="3" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="16.85546875" style="3" bestFit="1" customWidth="1"/>
     <col min="19" max="19" width="13" style="3" bestFit="1" customWidth="1"/>
     <col min="20" max="20" width="17" style="3" bestFit="1" customWidth="1"/>
-    <col min="21" max="23" width="13.5546875" style="3" customWidth="1"/>
-    <col min="24" max="24" width="15.44140625" style="3" bestFit="1" customWidth="1"/>
-    <col min="25" max="16384" width="9.109375" style="3"/>
+    <col min="21" max="23" width="13.5703125" style="3" customWidth="1"/>
+    <col min="24" max="24" width="15.42578125" style="3" bestFit="1" customWidth="1"/>
+    <col min="25" max="16384" width="9.140625" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" ht="16.8" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:20" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>70</v>
       </c>
@@ -8461,7 +8468,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="2" spans="1:20" ht="15" thickTop="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:20" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>58</v>
       </c>
@@ -8487,7 +8494,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="3" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>58</v>
       </c>
@@ -8510,7 +8517,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="4" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>58</v>
       </c>
@@ -8539,7 +8546,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="5" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
         <v>58</v>
       </c>
@@ -8568,7 +8575,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="6" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
         <v>58</v>
       </c>
@@ -8591,7 +8598,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="7" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
         <v>58</v>
       </c>
@@ -8620,7 +8627,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="8" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
         <v>58</v>
       </c>
@@ -8649,7 +8656,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="9" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
         <v>45</v>
       </c>
@@ -8675,7 +8682,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="10" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>45</v>
       </c>
@@ -8698,7 +8705,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="11" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
         <v>45</v>
       </c>
@@ -8727,7 +8734,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="12" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>45</v>
       </c>
@@ -8756,7 +8763,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="13" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
         <v>45</v>
       </c>
@@ -8785,7 +8792,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="14" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
         <v>45</v>
       </c>
@@ -8814,7 +8821,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="15" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
         <v>45</v>
       </c>
@@ -8837,7 +8844,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="16" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
         <v>45</v>
       </c>
@@ -8880,55 +8887,55 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:AT2"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.88671875" style="1" customWidth="1"/>
-    <col min="4" max="4" width="11.44140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.5546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="18.44140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.5546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="19.109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="19.88671875" style="1" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="10.5546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="13.5546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="19.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="10.5546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="13.5546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="13.44140625" style="37" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="12.5546875" style="37" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="21.44140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="20.109375" style="32" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="18.6640625" style="30" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="20.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="21.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="13.6640625" style="37" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="12.88671875" style="37" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="21.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="20.44140625" style="32" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.85546875" style="1" customWidth="1"/>
+    <col min="4" max="4" width="11.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="18.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="19.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="19.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="10.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="13.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="19.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="10.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="13.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="13.42578125" style="37" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="12.5703125" style="37" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="21.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="20.140625" style="32" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="18.7109375" style="30" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="17.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="20.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="21.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="13.7109375" style="37" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="12.85546875" style="37" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="21.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="20.42578125" style="32" bestFit="1" customWidth="1"/>
     <col min="27" max="27" width="19" style="30" bestFit="1" customWidth="1"/>
     <col min="28" max="28" width="20" style="1" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="24.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="18.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="18.5546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="32" max="35" width="18.5546875" style="1" customWidth="1"/>
-    <col min="36" max="36" width="18.88671875" style="1" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="23.88671875" style="1" bestFit="1" customWidth="1"/>
-    <col min="38" max="38" width="16.88671875" style="1" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="24.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="18.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="18.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="32" max="35" width="18.5703125" style="1" customWidth="1"/>
+    <col min="36" max="36" width="18.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="23.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="38" max="38" width="16.85546875" style="1" bestFit="1" customWidth="1"/>
     <col min="39" max="39" width="13" style="34" bestFit="1" customWidth="1"/>
     <col min="40" max="40" width="17" style="32" bestFit="1" customWidth="1"/>
-    <col min="41" max="41" width="15.6640625" style="30" bestFit="1" customWidth="1"/>
-    <col min="42" max="42" width="26.109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="43" max="43" width="8.6640625" style="39" customWidth="1"/>
-    <col min="44" max="44" width="10.5546875" style="39" bestFit="1" customWidth="1"/>
+    <col min="41" max="41" width="15.7109375" style="30" bestFit="1" customWidth="1"/>
+    <col min="42" max="42" width="26.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="43" max="43" width="8.7109375" style="39" customWidth="1"/>
+    <col min="44" max="44" width="10.5703125" style="39" bestFit="1" customWidth="1"/>
     <col min="45" max="45" width="10" style="32" bestFit="1" customWidth="1"/>
-    <col min="46" max="46" width="8.6640625" style="30" customWidth="1"/>
-    <col min="47" max="16384" width="9.109375" style="1"/>
+    <col min="46" max="46" width="8.7109375" style="30" customWidth="1"/>
+    <col min="47" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:46" s="5" customFormat="1" ht="16.8" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:46" s="5" customFormat="1" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
         <v>70</v>
       </c>
@@ -9068,7 +9075,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="2" spans="1:46" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
+    <row r="2" spans="1:46" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <autoFilter ref="A1:AT1" xr:uid="{00000000-0009-0000-0000-000005000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -9083,49 +9090,49 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:AU2"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.44140625" style="3" customWidth="1"/>
-    <col min="2" max="2" width="13.33203125" style="3" bestFit="1" customWidth="1"/>
-    <col min="3" max="4" width="10.5546875" style="3" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.5546875" style="3" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.5546875" style="3" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13.5546875" style="3" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="13.44140625" style="3" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="12.5546875" style="3" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="21.44140625" style="3" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="20.109375" style="21" bestFit="1" customWidth="1"/>
-    <col min="12" max="13" width="20.109375" style="26" customWidth="1"/>
-    <col min="14" max="14" width="20.109375" style="3" customWidth="1"/>
-    <col min="15" max="15" width="11.44140625" style="3" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="13.5546875" style="3" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="20.109375" style="3" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="18.44140625" style="3" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="23.88671875" style="3" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.42578125" style="3" customWidth="1"/>
+    <col min="2" max="2" width="13.28515625" style="3" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="10.5703125" style="3" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.5703125" style="3" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.5703125" style="3" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.5703125" style="3" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.42578125" style="3" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12.5703125" style="3" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="21.42578125" style="3" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="20.140625" style="21" bestFit="1" customWidth="1"/>
+    <col min="12" max="13" width="20.140625" style="26" customWidth="1"/>
+    <col min="14" max="14" width="20.140625" style="3" customWidth="1"/>
+    <col min="15" max="15" width="11.42578125" style="3" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="13.5703125" style="3" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="20.140625" style="3" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="18.42578125" style="3" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="23.85546875" style="3" bestFit="1" customWidth="1"/>
     <col min="20" max="20" width="19" style="3" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="21.109375" style="3" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="13.6640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="12.88671875" style="3" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="21.6640625" style="3" customWidth="1"/>
-    <col min="25" max="25" width="20.44140625" style="21" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="20.44140625" style="26" customWidth="1"/>
-    <col min="27" max="27" width="20.44140625" style="3" customWidth="1"/>
-    <col min="28" max="28" width="24.6640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="29" max="31" width="24.6640625" style="3" customWidth="1"/>
-    <col min="32" max="35" width="18.5546875" style="1" customWidth="1"/>
-    <col min="36" max="36" width="18.88671875" style="3" bestFit="1" customWidth="1"/>
-    <col min="37" max="40" width="18.88671875" style="3" customWidth="1"/>
-    <col min="41" max="41" width="13.88671875" style="3" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="21.140625" style="3" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="13.7109375" style="3" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="12.85546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="21.7109375" style="3" customWidth="1"/>
+    <col min="25" max="25" width="20.42578125" style="21" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="20.42578125" style="26" customWidth="1"/>
+    <col min="27" max="27" width="20.42578125" style="3" customWidth="1"/>
+    <col min="28" max="28" width="24.7109375" style="3" bestFit="1" customWidth="1"/>
+    <col min="29" max="31" width="24.7109375" style="3" customWidth="1"/>
+    <col min="32" max="35" width="18.5703125" style="1" customWidth="1"/>
+    <col min="36" max="36" width="18.85546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="37" max="40" width="18.85546875" style="3" customWidth="1"/>
+    <col min="41" max="41" width="13.85546875" style="3" bestFit="1" customWidth="1"/>
     <col min="42" max="42" width="13" style="3" bestFit="1" customWidth="1"/>
-    <col min="43" max="43" width="16.88671875" style="3" bestFit="1" customWidth="1"/>
+    <col min="43" max="43" width="16.85546875" style="3" bestFit="1" customWidth="1"/>
     <col min="44" max="44" width="13" style="18" bestFit="1" customWidth="1"/>
     <col min="45" max="45" width="13" style="21" customWidth="1"/>
     <col min="46" max="46" width="17" style="26" bestFit="1" customWidth="1"/>
-    <col min="47" max="47" width="24.88671875" style="3" bestFit="1" customWidth="1"/>
-    <col min="48" max="16384" width="9.109375" style="3"/>
+    <col min="47" max="47" width="24.85546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="48" max="16384" width="9.140625" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:47" s="5" customFormat="1" ht="16.8" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:47" s="5" customFormat="1" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
         <v>70</v>
       </c>
@@ -9268,7 +9275,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="2" spans="1:47" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
+    <row r="2" spans="1:47" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <autoFilter ref="A1:AU1" xr:uid="{00000000-0009-0000-0000-000006000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -9284,22 +9291,22 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1:N2"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="13.8" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="20.6640625" style="7" customWidth="1"/>
-    <col min="2" max="3" width="25.6640625" style="7" customWidth="1"/>
-    <col min="4" max="4" width="20.6640625" style="7" customWidth="1"/>
-    <col min="5" max="5" width="25.6640625" style="7" customWidth="1"/>
-    <col min="6" max="7" width="15.6640625" style="7" customWidth="1"/>
-    <col min="8" max="8" width="13.109375" style="22" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.109375" style="27" bestFit="1" customWidth="1"/>
-    <col min="10" max="11" width="25.6640625" style="7" customWidth="1"/>
-    <col min="12" max="13" width="15.44140625" style="7" customWidth="1"/>
+    <col min="1" max="1" width="20.7109375" style="7" customWidth="1"/>
+    <col min="2" max="3" width="25.7109375" style="7" customWidth="1"/>
+    <col min="4" max="4" width="20.7109375" style="7" customWidth="1"/>
+    <col min="5" max="5" width="25.7109375" style="7" customWidth="1"/>
+    <col min="6" max="7" width="15.7109375" style="7" customWidth="1"/>
+    <col min="8" max="8" width="13.140625" style="22" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13.140625" style="27" bestFit="1" customWidth="1"/>
+    <col min="10" max="11" width="25.7109375" style="7" customWidth="1"/>
+    <col min="12" max="13" width="15.42578125" style="7" customWidth="1"/>
     <col min="14" max="14" width="11" style="7" customWidth="1"/>
-    <col min="15" max="16384" width="9.109375" style="7"/>
+    <col min="15" max="16384" width="9.140625" style="7"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" s="9" customFormat="1" ht="20.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:14" s="9" customFormat="1" ht="20.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="9" t="s">
         <v>27</v>
       </c>
@@ -9343,7 +9350,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="2" spans="1:14" ht="14.4" thickTop="1" x14ac:dyDescent="0.3"/>
+    <row r="2" spans="1:14" ht="13.5" thickTop="1" x14ac:dyDescent="0.2"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -9357,25 +9364,25 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
   <dimension ref="A1:P2"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12" style="16" customWidth="1"/>
     <col min="2" max="2" width="24" style="16" customWidth="1"/>
-    <col min="3" max="3" width="25.5546875" style="16" customWidth="1"/>
-    <col min="4" max="4" width="10.5546875" style="16" customWidth="1"/>
-    <col min="5" max="6" width="10.5546875" style="16" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="10.5546875" style="16" customWidth="1"/>
-    <col min="8" max="8" width="20.44140625" style="16" customWidth="1"/>
-    <col min="9" max="9" width="18.109375" style="16" bestFit="1" customWidth="1"/>
-    <col min="10" max="11" width="18.109375" style="16" customWidth="1"/>
-    <col min="12" max="12" width="18.88671875" style="16" bestFit="1" customWidth="1"/>
-    <col min="13" max="14" width="10.6640625" style="17" customWidth="1"/>
-    <col min="15" max="15" width="20.6640625" style="24" customWidth="1"/>
-    <col min="16" max="16" width="20.6640625" style="29" customWidth="1"/>
-    <col min="17" max="16384" width="9.109375" style="16"/>
+    <col min="3" max="3" width="25.5703125" style="16" customWidth="1"/>
+    <col min="4" max="4" width="10.5703125" style="16" customWidth="1"/>
+    <col min="5" max="6" width="10.5703125" style="16" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.5703125" style="16" customWidth="1"/>
+    <col min="8" max="8" width="20.42578125" style="16" customWidth="1"/>
+    <col min="9" max="9" width="18.140625" style="16" bestFit="1" customWidth="1"/>
+    <col min="10" max="11" width="18.140625" style="16" customWidth="1"/>
+    <col min="12" max="12" width="18.85546875" style="16" bestFit="1" customWidth="1"/>
+    <col min="13" max="14" width="10.7109375" style="17" customWidth="1"/>
+    <col min="15" max="15" width="20.7109375" style="24" customWidth="1"/>
+    <col min="16" max="16" width="20.7109375" style="29" customWidth="1"/>
+    <col min="17" max="16384" width="9.140625" style="16"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" s="2" customFormat="1" ht="16.8" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:16" s="2" customFormat="1" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>2</v>
       </c>
@@ -9425,7 +9432,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="2" spans="1:16" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
+    <row r="2" spans="1:16" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <autoFilter ref="A1:P2" xr:uid="{00000000-0009-0000-0000-000008000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -9541,15 +9548,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance">
   <documentManagement>
     <Unity_Description xmlns="D75E00DB-06CE-4005-B397-8C0860A4229B" xsi:nil="true"/>
@@ -9560,6 +9558,15 @@
     </SipLabel>
   </documentManagement>
 </p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -9582,14 +9589,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2653FDDC-5C81-4B5A-A42F-7A63208AFFF7}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{268822B0-DCAE-4D2C-8340-AB7554C48D72}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
@@ -9604,4 +9603,12 @@
     <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2653FDDC-5C81-4B5A-A42F-7A63208AFFF7}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
PROPH-1754: Add Task URL into 5 different tabs in Workspace Data Report
</commit_message>
<xml_diff>
--- a/GenBOE/GenBOE.Web/Templates/Export/WorkspaceDataMST.xlsx
+++ b/GenBOE/GenBOE.Web/Templates/Export/WorkspaceDataMST.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\gitBoe\GenBOE\GenBOE.Web\Templates\Export\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37A2B01A-8844-4C24-8B34-A14A32448E44}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3925AB23-A7CF-4FBF-8E6E-F7E6E2E001FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5190" yWindow="30" windowWidth="34035" windowHeight="21570" firstSheet="5" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1290" yWindow="0" windowWidth="37755" windowHeight="21600" firstSheet="5" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="BOE3 Pivot" sheetId="19" state="hidden" r:id="rId1"/>
@@ -36,13 +36,13 @@
     <externalReference r:id="rId19"/>
   </externalReferences>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'BOE &amp; Resource Combo'!$A$1:$AT$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">BOEs!$A$1:$AU$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'BOE &amp; Resource Combo'!$A$1:$AU$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">BOEs!$A$1:$AV$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'BOEs (2)'!$B$1:$T$16</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'BOEs (3)'!$A$1:$N$16</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'MOQ by BOE by Task'!$A$1:$F$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'MOQ Table Data'!$A$1:$Q$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Resource Spreads'!$A$1:$P$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'MOQ by BOE by Task'!$A$1:$G$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'MOQ Table Data'!$A$1:$R$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Resource Spreads'!$B$1:$Q$2</definedName>
     <definedName name="Approvers">'[1]Options Lists'!$D$2:$D$4</definedName>
     <definedName name="Authors">'[1]Options Lists'!$C$2:$C$4</definedName>
     <definedName name="CLINs">'[1]Options Lists'!$B$2:$B$5</definedName>
@@ -53,9 +53,9 @@
   </definedNames>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="3" r:id="rId20"/>
-    <pivotCache cacheId="4" r:id="rId21"/>
-    <pivotCache cacheId="5" r:id="rId22"/>
+    <pivotCache cacheId="0" r:id="rId20"/>
+    <pivotCache cacheId="1" r:id="rId21"/>
+    <pivotCache cacheId="2" r:id="rId22"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -76,7 +76,7 @@
     <author>Lindsay Yorks</author>
   </authors>
   <commentList>
-    <comment ref="O1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0600-000001000000}">
+    <comment ref="P1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0600-000001000000}">
       <text>
         <r>
           <rPr>
@@ -320,7 +320,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="888" uniqueCount="146">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="893" uniqueCount="147">
   <si>
     <t>Start Date</t>
   </si>
@@ -758,6 +758,9 @@
   </si>
   <si>
     <t>Rationale</t>
+  </si>
+  <si>
+    <t>Task URL</t>
   </si>
 </sst>
 </file>
@@ -3153,7 +3156,7 @@
 <file path=xl/pivotCache/pivotCacheDefinition2.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="Lindsay Yorks" refreshedDate="40653.729487847224" createdVersion="3" refreshedVersion="3" minRefreshableVersion="3" recordCount="15" xr:uid="{00000000-000A-0000-FFFF-FFFF01000000}">
   <cacheSource type="worksheet">
-    <worksheetSource ref="C1:AT1" sheet="BOEs"/>
+    <worksheetSource ref="C1:AU1" sheet="BOEs"/>
   </cacheSource>
   <cacheFields count="19">
     <cacheField name="Type" numFmtId="49">
@@ -4357,7 +4360,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0000-000000000000}" name="PivotTable7" cacheId="3" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="3" minRefreshableVersion="3" showCalcMbrs="0" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="3" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0000-000000000000}" name="PivotTable7" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="3" minRefreshableVersion="3" showCalcMbrs="0" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="3" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
   <location ref="A3:N33" firstHeaderRow="1" firstDataRow="1" firstDataCol="14"/>
   <pivotFields count="14">
     <pivotField axis="axisRow" compact="0" outline="0" showAll="0" insertBlankRow="1" defaultSubtotal="0">
@@ -4706,7 +4709,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0200-000000000000}" name="PivotTable9" cacheId="4" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="3" minRefreshableVersion="3" showCalcMbrs="0" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="3" indent="0" compact="0" compactData="0" multipleFieldFilters="0" rowHeaderCaption="Type">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0200-000000000000}" name="PivotTable9" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="3" minRefreshableVersion="3" showCalcMbrs="0" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="3" indent="0" compact="0" compactData="0" multipleFieldFilters="0" rowHeaderCaption="Type">
   <location ref="A3:H11" firstHeaderRow="1" firstDataRow="1" firstDataCol="8"/>
   <pivotFields count="19">
     <pivotField axis="axisRow" compact="0" outline="0" showAll="0" defaultSubtotal="0">
@@ -4915,7 +4918,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0300-000000000000}" name="PivotTable4" cacheId="5" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" missingCaption="_" updatedVersion="3" minRefreshableVersion="3" showCalcMbrs="0" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="3" indent="0" compact="0" compactData="0" multipleFieldFilters="0" rowHeaderCaption="BOE ID">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0300-000000000000}" name="PivotTable4" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" missingCaption="_" updatedVersion="3" minRefreshableVersion="3" showCalcMbrs="0" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="3" indent="0" compact="0" compactData="0" multipleFieldFilters="0" rowHeaderCaption="BOE ID">
   <location ref="A3:T33" firstHeaderRow="1" firstDataRow="1" firstDataCol="20"/>
   <pivotFields count="20">
     <pivotField axis="axisRow" compact="0" outline="0" showAll="0" insertBlankRow="1" defaultSubtotal="0">
@@ -6166,18 +6169,19 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3DA6D2FB-3F32-46E9-963C-DCD2D761F967}">
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:H2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.140625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="13.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.42578125" bestFit="1" customWidth="1"/>
-    <col min="4" max="5" width="24" customWidth="1"/>
-    <col min="6" max="6" width="40.85546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="64.140625" customWidth="1"/>
+    <col min="3" max="3" width="13.28515625" customWidth="1"/>
+    <col min="4" max="4" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="24" customWidth="1"/>
+    <col min="7" max="7" width="40.85546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="64.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
         <v>70</v>
       </c>
@@ -6185,24 +6189,27 @@
         <v>115</v>
       </c>
       <c r="C1" s="5" t="s">
+        <v>146</v>
+      </c>
+      <c r="D1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="E1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="5" t="s">
+      <c r="F1" s="5" t="s">
         <v>119</v>
       </c>
-      <c r="F1" s="5" t="s">
+      <c r="G1" s="5" t="s">
         <v>84</v>
       </c>
-      <c r="G1" s="5" t="s">
+      <c r="H1" s="5" t="s">
         <v>145</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
+    <row r="2" spans="1:8" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
   </sheetData>
-  <autoFilter ref="A1:F1" xr:uid="{1E7471F8-87B8-4A9F-A5C2-80CE50F530C1}"/>
+  <autoFilter ref="A1:G1" xr:uid="{1E7471F8-87B8-4A9F-A5C2-80CE50F530C1}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter>
     <oddHeader>&amp;C&amp;"Calibri"&amp;10&amp;K000000 Lockheed Martin Proprietary Information&amp;1#_x000D_</oddHeader>
@@ -6213,30 +6220,31 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EDDB750B-2EAA-4C67-B526-87C6863613C3}">
-  <dimension ref="A1:R2"/>
+  <dimension ref="A1:S2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.140625" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="13.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="24" style="1" customWidth="1"/>
-    <col min="5" max="5" width="42.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="15.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="18.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="28.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="21.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="23" style="1" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="42" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="41.140625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="41.140625" style="32" customWidth="1"/>
-    <col min="14" max="14" width="35.28515625" style="32" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="57.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="61.42578125" style="32" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="28.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="27.28515625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="13.28515625" style="1" customWidth="1"/>
+    <col min="4" max="4" width="11.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="24" style="1" customWidth="1"/>
+    <col min="6" max="6" width="42.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="18.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="28.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="21.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="23" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="42" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="41.140625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="41.140625" style="32" customWidth="1"/>
+    <col min="15" max="15" width="35.28515625" style="32" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="57.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="61.42578125" style="32" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="28.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="27.28515625" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" s="5" customFormat="1" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:19" s="5" customFormat="1" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
         <v>70</v>
       </c>
@@ -6244,57 +6252,60 @@
         <v>115</v>
       </c>
       <c r="C1" s="5" t="s">
+        <v>146</v>
+      </c>
+      <c r="D1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="E1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="5" t="s">
+      <c r="F1" s="5" t="s">
         <v>84</v>
       </c>
-      <c r="F1" s="5" t="s">
+      <c r="G1" s="5" t="s">
         <v>127</v>
       </c>
-      <c r="G1" s="5" t="s">
+      <c r="H1" s="5" t="s">
         <v>128</v>
       </c>
-      <c r="H1" s="5" t="s">
+      <c r="I1" s="5" t="s">
         <v>129</v>
       </c>
-      <c r="I1" s="5" t="s">
+      <c r="J1" s="5" t="s">
         <v>130</v>
       </c>
-      <c r="J1" s="5" t="s">
+      <c r="K1" s="5" t="s">
         <v>131</v>
       </c>
-      <c r="K1" s="5" t="s">
+      <c r="L1" s="5" t="s">
         <v>132</v>
       </c>
-      <c r="L1" s="5" t="s">
+      <c r="M1" s="5" t="s">
         <v>133</v>
       </c>
-      <c r="M1" s="31" t="s">
+      <c r="N1" s="31" t="s">
         <v>138</v>
       </c>
-      <c r="N1" s="31" t="s">
+      <c r="O1" s="31" t="s">
         <v>134</v>
       </c>
-      <c r="O1" s="5" t="s">
+      <c r="P1" s="5" t="s">
         <v>135</v>
       </c>
-      <c r="P1" s="31" t="s">
+      <c r="Q1" s="31" t="s">
         <v>136</v>
       </c>
-      <c r="Q1" s="5" t="s">
+      <c r="R1" s="5" t="s">
         <v>140</v>
       </c>
-      <c r="R1" s="5" t="s">
+      <c r="S1" s="5" t="s">
         <v>137</v>
       </c>
     </row>
-    <row r="2" spans="1:18" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
+    <row r="2" spans="1:19" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
   </sheetData>
-  <autoFilter ref="A1:Q1" xr:uid="{EDDB750B-2EAA-4C67-B526-87C6863613C3}"/>
+  <autoFilter ref="A1:R1" xr:uid="{EDDB750B-2EAA-4C67-B526-87C6863613C3}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
   <headerFooter>
@@ -8886,56 +8897,56 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
-  <dimension ref="A1:AT2"/>
+  <dimension ref="A1:AU2"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.140625" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="13.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.85546875" style="1" customWidth="1"/>
-    <col min="4" max="4" width="11.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="18.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="19.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="19.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="10.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="13.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="19.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="10.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="13.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="13.42578125" style="37" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="12.5703125" style="37" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="21.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="20.140625" style="32" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="18.7109375" style="30" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="20.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="21.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="13.7109375" style="37" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="12.85546875" style="37" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="21.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="20.42578125" style="32" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="19" style="30" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="20" style="1" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="24.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="18.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="18.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="32" max="35" width="18.5703125" style="1" customWidth="1"/>
-    <col min="36" max="36" width="18.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="23.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="38" max="38" width="16.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="39" max="39" width="13" style="34" bestFit="1" customWidth="1"/>
-    <col min="40" max="40" width="17" style="32" bestFit="1" customWidth="1"/>
-    <col min="41" max="41" width="15.7109375" style="30" bestFit="1" customWidth="1"/>
-    <col min="42" max="42" width="26.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="43" max="43" width="8.7109375" style="39" customWidth="1"/>
-    <col min="44" max="44" width="10.5703125" style="39" bestFit="1" customWidth="1"/>
-    <col min="45" max="45" width="10" style="32" bestFit="1" customWidth="1"/>
-    <col min="46" max="46" width="8.7109375" style="30" customWidth="1"/>
-    <col min="47" max="16384" width="9.140625" style="1"/>
+    <col min="3" max="4" width="15.85546875" style="1" customWidth="1"/>
+    <col min="5" max="5" width="11.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="18.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="14.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="19.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="19.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="10.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="13.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="19.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="10.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="13.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="13.42578125" style="37" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="12.5703125" style="37" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="21.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="20.140625" style="32" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="18.7109375" style="30" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="17.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="20.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="21.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="13.7109375" style="37" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="12.85546875" style="37" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="21.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="20.42578125" style="32" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="19" style="30" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="20" style="1" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="24.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="18.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="18.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="33" max="36" width="18.5703125" style="1" customWidth="1"/>
+    <col min="37" max="37" width="18.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="38" max="38" width="23.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="39" max="39" width="16.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="40" max="40" width="13" style="34" bestFit="1" customWidth="1"/>
+    <col min="41" max="41" width="17" style="32" bestFit="1" customWidth="1"/>
+    <col min="42" max="42" width="15.7109375" style="30" bestFit="1" customWidth="1"/>
+    <col min="43" max="43" width="26.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="44" max="44" width="8.7109375" style="39" customWidth="1"/>
+    <col min="45" max="45" width="10.5703125" style="39" bestFit="1" customWidth="1"/>
+    <col min="46" max="46" width="10" style="32" bestFit="1" customWidth="1"/>
+    <col min="47" max="47" width="8.7109375" style="30" customWidth="1"/>
+    <col min="48" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:46" s="5" customFormat="1" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:47" s="5" customFormat="1" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
         <v>70</v>
       </c>
@@ -8945,139 +8956,142 @@
       <c r="C1" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="5" t="s">
+        <v>146</v>
+      </c>
+      <c r="E1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="F1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="5" t="s">
+      <c r="G1" s="5" t="s">
         <v>119</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="H1" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="H1" s="5" t="s">
+      <c r="I1" s="5" t="s">
         <v>118</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="J1" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="J1" s="5" t="s">
+      <c r="K1" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="K1" s="5" t="s">
+      <c r="L1" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="L1" s="5" t="s">
+      <c r="M1" s="5" t="s">
         <v>124</v>
       </c>
-      <c r="M1" s="5" t="s">
+      <c r="N1" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="N1" s="5" t="s">
+      <c r="O1" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="O1" s="36" t="s">
+      <c r="P1" s="36" t="s">
         <v>31</v>
       </c>
-      <c r="P1" s="36" t="s">
+      <c r="Q1" s="36" t="s">
         <v>32</v>
       </c>
-      <c r="Q1" s="5" t="s">
+      <c r="R1" s="5" t="s">
         <v>94</v>
       </c>
-      <c r="R1" s="31" t="s">
+      <c r="S1" s="31" t="s">
         <v>86</v>
       </c>
-      <c r="S1" s="25" t="s">
+      <c r="T1" s="25" t="s">
         <v>100</v>
       </c>
-      <c r="T1" s="5" t="s">
+      <c r="U1" s="5" t="s">
         <v>101</v>
       </c>
-      <c r="U1" s="5" t="s">
+      <c r="V1" s="5" t="s">
         <v>83</v>
       </c>
-      <c r="V1" s="5" t="s">
+      <c r="W1" s="5" t="s">
         <v>92</v>
       </c>
-      <c r="W1" s="36" t="s">
+      <c r="X1" s="36" t="s">
         <v>4</v>
       </c>
-      <c r="X1" s="36" t="s">
+      <c r="Y1" s="36" t="s">
         <v>5</v>
       </c>
-      <c r="Y1" s="5" t="s">
+      <c r="Z1" s="5" t="s">
         <v>95</v>
       </c>
-      <c r="Z1" s="31" t="s">
+      <c r="AA1" s="31" t="s">
         <v>85</v>
       </c>
-      <c r="AA1" s="25" t="s">
+      <c r="AB1" s="25" t="s">
         <v>102</v>
       </c>
-      <c r="AB1" s="5" t="s">
+      <c r="AC1" s="5" t="s">
         <v>103</v>
       </c>
-      <c r="AC1" s="5" t="s">
+      <c r="AD1" s="5" t="s">
         <v>89</v>
       </c>
-      <c r="AD1" s="5" t="s">
+      <c r="AE1" s="5" t="s">
         <v>88</v>
       </c>
-      <c r="AE1" s="5" t="s">
+      <c r="AF1" s="5" t="s">
         <v>105</v>
       </c>
-      <c r="AF1" s="5" t="s">
+      <c r="AG1" s="5" t="s">
         <v>141</v>
       </c>
-      <c r="AG1" s="5" t="s">
+      <c r="AH1" s="5" t="s">
         <v>142</v>
       </c>
-      <c r="AH1" s="5" t="s">
+      <c r="AI1" s="5" t="s">
         <v>143</v>
       </c>
-      <c r="AI1" s="5" t="s">
+      <c r="AJ1" s="5" t="s">
         <v>144</v>
       </c>
-      <c r="AJ1" s="5" t="s">
+      <c r="AK1" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="AK1" s="5" t="s">
+      <c r="AL1" s="5" t="s">
         <v>93</v>
       </c>
-      <c r="AL1" s="5" t="s">
+      <c r="AM1" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="AM1" s="33" t="s">
+      <c r="AN1" s="33" t="s">
         <v>14</v>
       </c>
-      <c r="AN1" s="31" t="s">
+      <c r="AO1" s="31" t="s">
         <v>15</v>
       </c>
-      <c r="AO1" s="25" t="s">
+      <c r="AP1" s="25" t="s">
         <v>109</v>
       </c>
-      <c r="AP1" s="5" t="s">
+      <c r="AQ1" s="5" t="s">
         <v>99</v>
       </c>
-      <c r="AQ1" s="38" t="s">
+      <c r="AR1" s="38" t="s">
         <v>90</v>
       </c>
-      <c r="AR1" s="38" t="s">
+      <c r="AS1" s="38" t="s">
         <v>91</v>
       </c>
-      <c r="AS1" s="35" t="s">
+      <c r="AT1" s="35" t="s">
         <v>110</v>
       </c>
-      <c r="AT1" s="28" t="s">
+      <c r="AU1" s="28" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="2" spans="1:46" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
+    <row r="2" spans="1:47" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
   </sheetData>
-  <autoFilter ref="A1:AT1" xr:uid="{00000000-0009-0000-0000-000005000000}"/>
+  <autoFilter ref="A1:AU1" xr:uid="{00000000-0009-0000-0000-000005000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
   <headerFooter>
@@ -9089,7 +9103,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
-  <dimension ref="A1:AU2"/>
+  <dimension ref="A1:AV2"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.42578125" style="3" customWidth="1"/>
@@ -9103,36 +9117,36 @@
     <col min="10" max="10" width="21.42578125" style="3" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="20.140625" style="21" bestFit="1" customWidth="1"/>
     <col min="12" max="13" width="20.140625" style="26" customWidth="1"/>
-    <col min="14" max="14" width="20.140625" style="3" customWidth="1"/>
-    <col min="15" max="15" width="11.42578125" style="3" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="13.5703125" style="3" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="20.140625" style="3" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="18.42578125" style="3" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="23.85546875" style="3" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="19" style="3" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="21.140625" style="3" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="13.7109375" style="3" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="12.85546875" style="3" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="21.7109375" style="3" customWidth="1"/>
-    <col min="25" max="25" width="20.42578125" style="21" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="20.42578125" style="26" customWidth="1"/>
-    <col min="27" max="27" width="20.42578125" style="3" customWidth="1"/>
-    <col min="28" max="28" width="24.7109375" style="3" bestFit="1" customWidth="1"/>
-    <col min="29" max="31" width="24.7109375" style="3" customWidth="1"/>
-    <col min="32" max="35" width="18.5703125" style="1" customWidth="1"/>
-    <col min="36" max="36" width="18.85546875" style="3" bestFit="1" customWidth="1"/>
-    <col min="37" max="40" width="18.85546875" style="3" customWidth="1"/>
-    <col min="41" max="41" width="13.85546875" style="3" bestFit="1" customWidth="1"/>
-    <col min="42" max="42" width="13" style="3" bestFit="1" customWidth="1"/>
-    <col min="43" max="43" width="16.85546875" style="3" bestFit="1" customWidth="1"/>
-    <col min="44" max="44" width="13" style="18" bestFit="1" customWidth="1"/>
-    <col min="45" max="45" width="13" style="21" customWidth="1"/>
-    <col min="46" max="46" width="17" style="26" bestFit="1" customWidth="1"/>
-    <col min="47" max="47" width="24.85546875" style="3" bestFit="1" customWidth="1"/>
-    <col min="48" max="16384" width="9.140625" style="3"/>
+    <col min="14" max="15" width="20.140625" style="3" customWidth="1"/>
+    <col min="16" max="16" width="11.42578125" style="3" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="13.5703125" style="3" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="20.140625" style="3" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="18.42578125" style="3" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="23.85546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="19" style="3" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="21.140625" style="3" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="13.7109375" style="3" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="12.85546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="21.7109375" style="3" customWidth="1"/>
+    <col min="26" max="26" width="20.42578125" style="21" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="20.42578125" style="26" customWidth="1"/>
+    <col min="28" max="28" width="20.42578125" style="3" customWidth="1"/>
+    <col min="29" max="29" width="24.7109375" style="3" bestFit="1" customWidth="1"/>
+    <col min="30" max="32" width="24.7109375" style="3" customWidth="1"/>
+    <col min="33" max="36" width="18.5703125" style="1" customWidth="1"/>
+    <col min="37" max="37" width="18.85546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="38" max="41" width="18.85546875" style="3" customWidth="1"/>
+    <col min="42" max="42" width="13.85546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="43" max="43" width="13" style="3" bestFit="1" customWidth="1"/>
+    <col min="44" max="44" width="16.85546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="45" max="45" width="13" style="18" bestFit="1" customWidth="1"/>
+    <col min="46" max="46" width="13" style="21" customWidth="1"/>
+    <col min="47" max="47" width="17" style="26" bestFit="1" customWidth="1"/>
+    <col min="48" max="48" width="24.85546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="49" max="16384" width="9.140625" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:47" s="5" customFormat="1" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:48" s="5" customFormat="1" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
         <v>70</v>
       </c>
@@ -9176,108 +9190,111 @@
         <v>101</v>
       </c>
       <c r="O1" s="5" t="s">
+        <v>146</v>
+      </c>
+      <c r="P1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="P1" s="5" t="s">
+      <c r="Q1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="Q1" s="5" t="s">
+      <c r="R1" s="5" t="s">
         <v>83</v>
       </c>
-      <c r="R1" s="5" t="s">
+      <c r="S1" s="5" t="s">
         <v>119</v>
       </c>
-      <c r="S1" s="5" t="s">
+      <c r="T1" s="5" t="s">
         <v>84</v>
       </c>
-      <c r="T1" s="5" t="s">
+      <c r="U1" s="5" t="s">
         <v>118</v>
       </c>
-      <c r="U1" s="5" t="s">
+      <c r="V1" s="5" t="s">
         <v>92</v>
       </c>
-      <c r="V1" s="5" t="s">
+      <c r="W1" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="W1" s="5" t="s">
+      <c r="X1" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="X1" s="5" t="s">
+      <c r="Y1" s="5" t="s">
         <v>95</v>
       </c>
-      <c r="Y1" s="20" t="s">
+      <c r="Z1" s="20" t="s">
         <v>85</v>
       </c>
-      <c r="Z1" s="25" t="s">
+      <c r="AA1" s="25" t="s">
         <v>102</v>
       </c>
-      <c r="AA1" s="5" t="s">
+      <c r="AB1" s="5" t="s">
         <v>103</v>
       </c>
-      <c r="AB1" s="5" t="s">
+      <c r="AC1" s="5" t="s">
         <v>89</v>
       </c>
-      <c r="AC1" s="5" t="s">
+      <c r="AD1" s="5" t="s">
         <v>104</v>
       </c>
-      <c r="AD1" s="5" t="s">
+      <c r="AE1" s="5" t="s">
         <v>88</v>
       </c>
-      <c r="AE1" s="5" t="s">
+      <c r="AF1" s="5" t="s">
         <v>105</v>
       </c>
-      <c r="AF1" s="5" t="s">
+      <c r="AG1" s="5" t="s">
         <v>141</v>
       </c>
-      <c r="AG1" s="5" t="s">
+      <c r="AH1" s="5" t="s">
         <v>142</v>
       </c>
-      <c r="AH1" s="5" t="s">
+      <c r="AI1" s="5" t="s">
         <v>143</v>
       </c>
-      <c r="AI1" s="5" t="s">
+      <c r="AJ1" s="5" t="s">
         <v>144</v>
       </c>
-      <c r="AJ1" s="5" t="s">
+      <c r="AK1" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="AK1" s="5" t="s">
+      <c r="AL1" s="5" t="s">
         <v>93</v>
       </c>
-      <c r="AL1" s="5" t="s">
+      <c r="AM1" s="5" t="s">
         <v>106</v>
       </c>
-      <c r="AM1" s="5" t="s">
+      <c r="AN1" s="5" t="s">
         <v>107</v>
       </c>
-      <c r="AN1" s="5" t="s">
+      <c r="AO1" s="5" t="s">
         <v>108</v>
       </c>
-      <c r="AO1" s="5" t="s">
+      <c r="AP1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="AP1" s="5" t="s">
+      <c r="AQ1" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="AQ1" s="5" t="s">
+      <c r="AR1" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="AR1" s="5" t="s">
+      <c r="AS1" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="AS1" s="20" t="s">
+      <c r="AT1" s="20" t="s">
         <v>15</v>
       </c>
-      <c r="AT1" s="25" t="s">
+      <c r="AU1" s="25" t="s">
         <v>109</v>
       </c>
-      <c r="AU1" s="5" t="s">
+      <c r="AV1" s="5" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="2" spans="1:47" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
+    <row r="2" spans="1:48" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
   </sheetData>
-  <autoFilter ref="A1:AU1" xr:uid="{00000000-0009-0000-0000-000006000000}"/>
+  <autoFilter ref="A1:AV1" xr:uid="{00000000-0009-0000-0000-000006000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
   <headerFooter>
@@ -9363,78 +9380,82 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
-  <dimension ref="A1:P2"/>
+  <dimension ref="A1:Q2"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12" style="16" customWidth="1"/>
-    <col min="2" max="2" width="24" style="16" customWidth="1"/>
-    <col min="3" max="3" width="25.5703125" style="16" customWidth="1"/>
-    <col min="4" max="4" width="10.5703125" style="16" customWidth="1"/>
-    <col min="5" max="6" width="10.5703125" style="16" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="10.5703125" style="16" customWidth="1"/>
-    <col min="8" max="8" width="20.42578125" style="16" customWidth="1"/>
-    <col min="9" max="9" width="18.140625" style="16" bestFit="1" customWidth="1"/>
-    <col min="10" max="11" width="18.140625" style="16" customWidth="1"/>
-    <col min="12" max="12" width="18.85546875" style="16" bestFit="1" customWidth="1"/>
-    <col min="13" max="14" width="10.7109375" style="17" customWidth="1"/>
-    <col min="15" max="15" width="20.7109375" style="24" customWidth="1"/>
-    <col min="16" max="16" width="20.7109375" style="29" customWidth="1"/>
-    <col min="17" max="16384" width="9.140625" style="16"/>
+    <col min="1" max="1" width="21" style="16" customWidth="1"/>
+    <col min="2" max="2" width="12" style="16" customWidth="1"/>
+    <col min="3" max="3" width="24" style="16" customWidth="1"/>
+    <col min="4" max="4" width="25.5703125" style="16" customWidth="1"/>
+    <col min="5" max="5" width="10.5703125" style="16" customWidth="1"/>
+    <col min="6" max="7" width="10.5703125" style="16" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.5703125" style="16" customWidth="1"/>
+    <col min="9" max="9" width="20.42578125" style="16" customWidth="1"/>
+    <col min="10" max="10" width="18.140625" style="16" bestFit="1" customWidth="1"/>
+    <col min="11" max="12" width="18.140625" style="16" customWidth="1"/>
+    <col min="13" max="13" width="18.85546875" style="16" bestFit="1" customWidth="1"/>
+    <col min="14" max="15" width="10.7109375" style="17" customWidth="1"/>
+    <col min="16" max="16" width="20.7109375" style="24" customWidth="1"/>
+    <col min="17" max="17" width="20.7109375" style="29" customWidth="1"/>
+    <col min="18" max="16384" width="9.140625" style="16"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" s="2" customFormat="1" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:17" s="2" customFormat="1" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="B1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="C1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="D1" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="E1" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="F1" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="G1" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="H1" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="I1" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="J1" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="J1" s="5" t="s">
+      <c r="K1" s="5" t="s">
         <v>143</v>
       </c>
-      <c r="K1" s="5" t="s">
+      <c r="L1" s="5" t="s">
         <v>144</v>
       </c>
-      <c r="L1" s="2" t="s">
+      <c r="M1" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="2" t="s">
+      <c r="N1" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="N1" s="2" t="s">
+      <c r="O1" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="O1" s="23" t="s">
+      <c r="P1" s="23" t="s">
         <v>110</v>
       </c>
-      <c r="P1" s="28" t="s">
+      <c r="Q1" s="28" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="2" spans="1:16" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
+    <row r="2" spans="1:17" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
   </sheetData>
-  <autoFilter ref="A1:P2" xr:uid="{00000000-0009-0000-0000-000008000000}"/>
+  <autoFilter ref="B1:Q2" xr:uid="{00000000-0009-0000-0000-000008000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
   <headerFooter>
@@ -9445,6 +9466,28 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance">
+  <documentManagement>
+    <Unity_Description xmlns="D75E00DB-06CE-4005-B397-8C0860A4229B" xsi:nil="true"/>
+    <Unity_Tag xmlns="D75E00DB-06CE-4005-B397-8C0860A4229B" xsi:nil="true"/>
+    <Capabilities xmlns="d75e00db-06ce-4005-b397-8c0860a4229b" xsi:nil="true"/>
+    <SipLabel xmlns="372b77af-8063-48a8-888c-73c0edf01dea">
+      <Value>2</Value>
+    </SipLabel>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Custom Document" ma:contentTypeID="0x010100E6322E8F405D4D9EA89D8C83B7E1048B001BB96E1BE0ACBB41BF00782ED0412411" ma:contentTypeVersion="3" ma:contentTypeDescription="Custom Document" ma:contentTypeScope="" ma:versionID="3c14126572fa3c0d4c677ac1f3ba4426">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="D75E00DB-06CE-4005-B397-8C0860A4229B" xmlns:ns3="372b77af-8063-48a8-888c-73c0edf01dea" xmlns:ns4="d75e00db-06ce-4005-b397-8c0860a4229b" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="9e89026a025b72b85b9543506e7af3e1" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="D75E00DB-06CE-4005-B397-8C0860A4229B"/>
@@ -9547,43 +9590,10 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance">
-  <documentManagement>
-    <Unity_Description xmlns="D75E00DB-06CE-4005-B397-8C0860A4229B" xsi:nil="true"/>
-    <Unity_Tag xmlns="D75E00DB-06CE-4005-B397-8C0860A4229B" xsi:nil="true"/>
-    <Capabilities xmlns="d75e00db-06ce-4005-b397-8c0860a4229b" xsi:nil="true"/>
-    <SipLabel xmlns="372b77af-8063-48a8-888c-73c0edf01dea">
-      <Value>2</Value>
-    </SipLabel>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1DE4120D-B400-435F-B862-B3B8683830A5}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2653FDDC-5C81-4B5A-A42F-7A63208AFFF7}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="D75E00DB-06CE-4005-B397-8C0860A4229B"/>
-    <ds:schemaRef ds:uri="372b77af-8063-48a8-888c-73c0edf01dea"/>
-    <ds:schemaRef ds:uri="d75e00db-06ce-4005-b397-8c0860a4229b"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/internal/2005/internalDocumentation"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -9606,9 +9616,20 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2653FDDC-5C81-4B5A-A42F-7A63208AFFF7}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1DE4120D-B400-435F-B862-B3B8683830A5}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="D75E00DB-06CE-4005-B397-8C0860A4229B"/>
+    <ds:schemaRef ds:uri="372b77af-8063-48a8-888c-73c0edf01dea"/>
+    <ds:schemaRef ds:uri="d75e00db-06ce-4005-b397-8c0860a4229b"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/internal/2005/internalDocumentation"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
1992 - Add Skill Mix to Workspace Data Excel Export
</commit_message>
<xml_diff>
--- a/GenBOE/GenBOE.Web/Templates/Export/WorkspaceDataMST.xlsx
+++ b/GenBOE/GenBOE.Web/Templates/Export/WorkspaceDataMST.xlsx
@@ -5,12 +5,12 @@
   <workbookPr showPivotChartFilter="1" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\gitBoe\GenBOE\GenBOE.Web\Templates\Export\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ranzalon\Source\repos\IES\GenBOE\GenBOE.Web\Templates\Export\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3925AB23-A7CF-4FBF-8E6E-F7E6E2E001FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87DA46AB-DE9F-490D-B1BC-CC263702B68B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1290" yWindow="0" windowWidth="37755" windowHeight="21600" firstSheet="5" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="25440" windowHeight="15390" firstSheet="5" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="BOE3 Pivot" sheetId="19" state="hidden" r:id="rId1"/>
@@ -24,22 +24,26 @@
     <sheet name="Resource Spreads" sheetId="41" r:id="rId9"/>
     <sheet name="MOQ by BOE by Task" sheetId="45" r:id="rId10"/>
     <sheet name="MOQ Table Data" sheetId="46" r:id="rId11"/>
-    <sheet name="WBS" sheetId="24" r:id="rId12"/>
-    <sheet name="CLINs" sheetId="25" r:id="rId13"/>
-    <sheet name="User Permissions" sheetId="39" r:id="rId14"/>
-    <sheet name="Workspace Identification" sheetId="40" r:id="rId15"/>
-    <sheet name="Travel Unit Cost" sheetId="43" r:id="rId16"/>
-    <sheet name="Travel Extended Cost" sheetId="44" r:id="rId17"/>
+    <sheet name="Current Skill Mix" sheetId="48" r:id="rId12"/>
+    <sheet name="Common Disclosure Skill Mix" sheetId="47" r:id="rId13"/>
+    <sheet name="WBS" sheetId="24" r:id="rId14"/>
+    <sheet name="CLINs" sheetId="25" r:id="rId15"/>
+    <sheet name="User Permissions" sheetId="39" r:id="rId16"/>
+    <sheet name="Workspace Identification" sheetId="40" r:id="rId17"/>
+    <sheet name="Travel Unit Cost" sheetId="43" r:id="rId18"/>
+    <sheet name="Travel Extended Cost" sheetId="44" r:id="rId19"/>
   </sheets>
   <externalReferences>
-    <externalReference r:id="rId18"/>
-    <externalReference r:id="rId19"/>
+    <externalReference r:id="rId20"/>
+    <externalReference r:id="rId21"/>
   </externalReferences>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'BOE &amp; Resource Combo'!$A$1:$AU$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">BOEs!$A$1:$AV$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'BOEs (2)'!$B$1:$T$16</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'BOEs (3)'!$A$1:$N$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'Common Disclosure Skill Mix'!$A$1:$N$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Current Skill Mix'!$A$1:$N$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'MOQ by BOE by Task'!$A$1:$G$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'MOQ Table Data'!$A$1:$R$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Resource Spreads'!$B$1:$Q$2</definedName>
@@ -53,9 +57,9 @@
   </definedNames>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="0" r:id="rId20"/>
-    <pivotCache cacheId="1" r:id="rId21"/>
-    <pivotCache cacheId="2" r:id="rId22"/>
+    <pivotCache cacheId="3" r:id="rId22"/>
+    <pivotCache cacheId="4" r:id="rId23"/>
+    <pivotCache cacheId="5" r:id="rId24"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -320,7 +324,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="893" uniqueCount="147">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="921" uniqueCount="156">
   <si>
     <t>Start Date</t>
   </si>
@@ -761,17 +765,45 @@
   </si>
   <si>
     <t>Task URL</t>
+  </si>
+  <si>
+    <t>Historical Hours</t>
+  </si>
+  <si>
+    <t>Labor Skill Mix</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Included </t>
+  </si>
+  <si>
+    <t>BOE Skill Mix</t>
+  </si>
+  <si>
+    <t>Proposed Hours</t>
+  </si>
+  <si>
+    <t>Rationale </t>
+  </si>
+  <si>
+    <t>Included</t>
+  </si>
+  <si>
+    <t>Current Resource</t>
+  </si>
+  <si>
+    <t>Business Resource Code</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="4">
+  <numFmts count="5">
     <numFmt numFmtId="164" formatCode="m/yyyy"/>
     <numFmt numFmtId="165" formatCode="m/d/yyyy;@"/>
     <numFmt numFmtId="166" formatCode="0.000"/>
     <numFmt numFmtId="167" formatCode="&quot;$&quot;#,##0.00"/>
+    <numFmt numFmtId="168" formatCode="0.0"/>
   </numFmts>
   <fonts count="14" x14ac:knownFonts="1">
     <font>
@@ -1009,7 +1041,7 @@
     <xf numFmtId="0" fontId="10" fillId="6" borderId="0"/>
     <xf numFmtId="0" fontId="13" fillId="7" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="60">
+  <cellXfs count="62">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="1" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyAlignment="1">
@@ -1164,6 +1196,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="168" fontId="1" fillId="2" borderId="1" xfId="1" applyNumberFormat="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="8">
     <cellStyle name="genBOE" xfId="1" xr:uid="{00000000-0005-0000-0000-000000000000}"/>
@@ -4360,7 +4396,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0000-000000000000}" name="PivotTable7" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="3" minRefreshableVersion="3" showCalcMbrs="0" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="3" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0000-000000000000}" name="PivotTable7" cacheId="3" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="3" minRefreshableVersion="3" showCalcMbrs="0" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="3" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
   <location ref="A3:N33" firstHeaderRow="1" firstDataRow="1" firstDataCol="14"/>
   <pivotFields count="14">
     <pivotField axis="axisRow" compact="0" outline="0" showAll="0" insertBlankRow="1" defaultSubtotal="0">
@@ -4709,7 +4745,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0200-000000000000}" name="PivotTable9" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="3" minRefreshableVersion="3" showCalcMbrs="0" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="3" indent="0" compact="0" compactData="0" multipleFieldFilters="0" rowHeaderCaption="Type">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0200-000000000000}" name="PivotTable9" cacheId="4" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="3" minRefreshableVersion="3" showCalcMbrs="0" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="3" indent="0" compact="0" compactData="0" multipleFieldFilters="0" rowHeaderCaption="Type">
   <location ref="A3:H11" firstHeaderRow="1" firstDataRow="1" firstDataCol="8"/>
   <pivotFields count="19">
     <pivotField axis="axisRow" compact="0" outline="0" showAll="0" defaultSubtotal="0">
@@ -4918,7 +4954,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0300-000000000000}" name="PivotTable4" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" missingCaption="_" updatedVersion="3" minRefreshableVersion="3" showCalcMbrs="0" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="3" indent="0" compact="0" compactData="0" multipleFieldFilters="0" rowHeaderCaption="BOE ID">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0300-000000000000}" name="PivotTable4" cacheId="5" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" missingCaption="_" updatedVersion="3" minRefreshableVersion="3" showCalcMbrs="0" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="3" indent="0" compact="0" compactData="0" multipleFieldFilters="0" rowHeaderCaption="BOE ID">
   <location ref="A3:T33" firstHeaderRow="1" firstDataRow="1" firstDataCol="20"/>
   <pivotFields count="20">
     <pivotField axis="axisRow" compact="0" outline="0" showAll="0" insertBlankRow="1" defaultSubtotal="0">
@@ -6316,6 +6352,150 @@
 </file>
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0DB870C3-50D3-464E-B6EE-1445D5A297E1}">
+  <dimension ref="A1:N2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="11.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.5703125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.85546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="20.85546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="19.7109375" style="61" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="18.140625" style="34" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="12.42578125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="17" style="34" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="19.28515625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="14" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:14" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>115</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>146</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="G1" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="H1" s="5" t="s">
+        <v>154</v>
+      </c>
+      <c r="I1" s="60" t="s">
+        <v>147</v>
+      </c>
+      <c r="J1" s="33" t="s">
+        <v>148</v>
+      </c>
+      <c r="K1" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="L1" s="33" t="s">
+        <v>150</v>
+      </c>
+      <c r="M1" s="5" t="s">
+        <v>151</v>
+      </c>
+      <c r="N1" s="5" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
+  </sheetData>
+  <autoFilter ref="A1:N1" xr:uid="{0DB870C3-50D3-464E-B6EE-1445D5A297E1}"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E39BBE49-D540-4CED-8CD6-9B452AE05592}">
+  <dimension ref="A1:N2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="11.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.5703125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="20.85546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="27.85546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="19.7109375" style="61" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="18.140625" style="34" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="13" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="17" style="34" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="19.28515625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="14" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:14" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>115</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>146</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="G1" s="5" t="s">
+        <v>154</v>
+      </c>
+      <c r="H1" s="5" t="s">
+        <v>155</v>
+      </c>
+      <c r="I1" s="60" t="s">
+        <v>147</v>
+      </c>
+      <c r="J1" s="33" t="s">
+        <v>148</v>
+      </c>
+      <c r="K1" s="5" t="s">
+        <v>149</v>
+      </c>
+      <c r="L1" s="33" t="s">
+        <v>150</v>
+      </c>
+      <c r="M1" s="5" t="s">
+        <v>151</v>
+      </c>
+      <c r="N1" s="5" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
+  </sheetData>
+  <autoFilter ref="A1:N1" xr:uid="{E39BBE49-D540-4CED-8CD6-9B452AE05592}"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
   <dimension ref="A1:E2"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
@@ -6355,7 +6535,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
   <dimension ref="A1:E2"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
@@ -6396,7 +6576,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0B00-000000000000}">
   <dimension ref="A1:I2"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -6452,7 +6632,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0C00-000000000000}">
   <dimension ref="A1:A16"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -6544,7 +6724,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1E9E49D2-B4A1-426D-8F6A-B85DD2E6A5AA}">
   <dimension ref="A1:AA7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -6769,7 +6949,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00BB237A-2FF2-450F-81EE-9A098F6C7133}">
   <dimension ref="A1:AA6"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -9466,15 +9646,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance">
   <documentManagement>
     <Unity_Description xmlns="D75E00DB-06CE-4005-B397-8C0860A4229B" xsi:nil="true"/>
@@ -9487,7 +9658,7 @@
 </p:properties>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Custom Document" ma:contentTypeID="0x010100E6322E8F405D4D9EA89D8C83B7E1048B001BB96E1BE0ACBB41BF00782ED0412411" ma:contentTypeVersion="3" ma:contentTypeDescription="Custom Document" ma:contentTypeScope="" ma:versionID="3c14126572fa3c0d4c677ac1f3ba4426">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="D75E00DB-06CE-4005-B397-8C0860A4229B" xmlns:ns3="372b77af-8063-48a8-888c-73c0edf01dea" xmlns:ns4="d75e00db-06ce-4005-b397-8c0860a4229b" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="9e89026a025b72b85b9543506e7af3e1" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="D75E00DB-06CE-4005-B397-8C0860A4229B"/>
@@ -9590,15 +9761,16 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2653FDDC-5C81-4B5A-A42F-7A63208AFFF7}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{268822B0-DCAE-4D2C-8340-AB7554C48D72}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
@@ -9615,7 +9787,7 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1DE4120D-B400-435F-B862-B3B8683830A5}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -9632,4 +9804,12 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/internal/2005/internalDocumentation"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2653FDDC-5C81-4B5A-A42F-7A63208AFFF7}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Skill Mix recovered and updated code for Workspace Data Export
</commit_message>
<xml_diff>
--- a/GenBOE/GenBOE.Web/Templates/Export/WorkspaceDataMST.xlsx
+++ b/GenBOE/GenBOE.Web/Templates/Export/WorkspaceDataMST.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26731"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27928"/>
   <workbookPr showPivotChartFilter="1" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ranzalon\Source\repos\IES\GenBOE\GenBOE.Web\Templates\Export\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\twilson3\source\IES\GenBOE\GenBOE.Web\Templates\Export\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87DA46AB-DE9F-490D-B1BC-CC263702B68B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{709B05D6-9678-4BC2-BA45-58A1F0827487}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="25440" windowHeight="15390" firstSheet="5" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="19395" windowHeight="15585" firstSheet="5" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="BOE3 Pivot" sheetId="19" state="hidden" r:id="rId1"/>
@@ -25,7 +25,7 @@
     <sheet name="MOQ by BOE by Task" sheetId="45" r:id="rId10"/>
     <sheet name="MOQ Table Data" sheetId="46" r:id="rId11"/>
     <sheet name="Current Skill Mix" sheetId="48" r:id="rId12"/>
-    <sheet name="Common Disclosure Skill Mix" sheetId="47" r:id="rId13"/>
+    <sheet name="LM Enterprise Skill Mix" sheetId="47" r:id="rId13"/>
     <sheet name="WBS" sheetId="24" r:id="rId14"/>
     <sheet name="CLINs" sheetId="25" r:id="rId15"/>
     <sheet name="User Permissions" sheetId="39" r:id="rId16"/>
@@ -42,8 +42,8 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">BOEs!$A$1:$AV$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'BOEs (2)'!$B$1:$T$16</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'BOEs (3)'!$A$1:$N$16</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'Common Disclosure Skill Mix'!$A$1:$N$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Current Skill Mix'!$A$1:$N$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'LM Enterprise Skill Mix'!$A$1:$N$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'MOQ by BOE by Task'!$A$1:$G$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'MOQ Table Data'!$A$1:$R$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Resource Spreads'!$B$1:$Q$2</definedName>
@@ -57,9 +57,9 @@
   </definedNames>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="3" r:id="rId22"/>
-    <pivotCache cacheId="4" r:id="rId23"/>
-    <pivotCache cacheId="5" r:id="rId24"/>
+    <pivotCache cacheId="0" r:id="rId22"/>
+    <pivotCache cacheId="1" r:id="rId23"/>
+    <pivotCache cacheId="2" r:id="rId24"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -4396,7 +4396,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0000-000000000000}" name="PivotTable7" cacheId="3" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="3" minRefreshableVersion="3" showCalcMbrs="0" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="3" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0000-000000000000}" name="PivotTable7" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="3" minRefreshableVersion="3" showCalcMbrs="0" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="3" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
   <location ref="A3:N33" firstHeaderRow="1" firstDataRow="1" firstDataCol="14"/>
   <pivotFields count="14">
     <pivotField axis="axisRow" compact="0" outline="0" showAll="0" insertBlankRow="1" defaultSubtotal="0">
@@ -4745,7 +4745,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0200-000000000000}" name="PivotTable9" cacheId="4" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="3" minRefreshableVersion="3" showCalcMbrs="0" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="3" indent="0" compact="0" compactData="0" multipleFieldFilters="0" rowHeaderCaption="Type">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0200-000000000000}" name="PivotTable9" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="3" minRefreshableVersion="3" showCalcMbrs="0" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="3" indent="0" compact="0" compactData="0" multipleFieldFilters="0" rowHeaderCaption="Type">
   <location ref="A3:H11" firstHeaderRow="1" firstDataRow="1" firstDataCol="8"/>
   <pivotFields count="19">
     <pivotField axis="axisRow" compact="0" outline="0" showAll="0" defaultSubtotal="0">
@@ -4954,7 +4954,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0300-000000000000}" name="PivotTable4" cacheId="5" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" missingCaption="_" updatedVersion="3" minRefreshableVersion="3" showCalcMbrs="0" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="3" indent="0" compact="0" compactData="0" multipleFieldFilters="0" rowHeaderCaption="BOE ID">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0300-000000000000}" name="PivotTable4" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" missingCaption="_" updatedVersion="3" minRefreshableVersion="3" showCalcMbrs="0" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="3" indent="0" compact="0" compactData="0" multipleFieldFilters="0" rowHeaderCaption="BOE ID">
   <location ref="A3:T33" firstHeaderRow="1" firstDataRow="1" firstDataCol="20"/>
   <pivotFields count="20">
     <pivotField axis="axisRow" compact="0" outline="0" showAll="0" insertBlankRow="1" defaultSubtotal="0">
@@ -9646,19 +9646,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance">
-  <documentManagement>
-    <Unity_Description xmlns="D75E00DB-06CE-4005-B397-8C0860A4229B" xsi:nil="true"/>
-    <Unity_Tag xmlns="D75E00DB-06CE-4005-B397-8C0860A4229B" xsi:nil="true"/>
-    <Capabilities xmlns="d75e00db-06ce-4005-b397-8c0860a4229b" xsi:nil="true"/>
-    <SipLabel xmlns="372b77af-8063-48a8-888c-73c0edf01dea">
-      <Value>2</Value>
-    </SipLabel>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Custom Document" ma:contentTypeID="0x010100E6322E8F405D4D9EA89D8C83B7E1048B001BB96E1BE0ACBB41BF00782ED0412411" ma:contentTypeVersion="3" ma:contentTypeDescription="Custom Document" ma:contentTypeScope="" ma:versionID="3c14126572fa3c0d4c677ac1f3ba4426">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="D75E00DB-06CE-4005-B397-8C0860A4229B" xmlns:ns3="372b77af-8063-48a8-888c-73c0edf01dea" xmlns:ns4="d75e00db-06ce-4005-b397-8c0860a4229b" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="9e89026a025b72b85b9543506e7af3e1" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="D75E00DB-06CE-4005-B397-8C0860A4229B"/>
@@ -9761,6 +9748,19 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance">
+  <documentManagement>
+    <Unity_Description xmlns="D75E00DB-06CE-4005-B397-8C0860A4229B" xsi:nil="true"/>
+    <Unity_Tag xmlns="D75E00DB-06CE-4005-B397-8C0860A4229B" xsi:nil="true"/>
+    <Capabilities xmlns="d75e00db-06ce-4005-b397-8c0860a4229b" xsi:nil="true"/>
+    <SipLabel xmlns="372b77af-8063-48a8-888c-73c0edf01dea">
+      <Value>2</Value>
+    </SipLabel>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -9771,23 +9771,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{268822B0-DCAE-4D2C-8340-AB7554C48D72}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="D75E00DB-06CE-4005-B397-8C0860A4229B"/>
-    <ds:schemaRef ds:uri="372b77af-8063-48a8-888c-73c0edf01dea"/>
-    <ds:schemaRef ds:uri="d75e00db-06ce-4005-b397-8c0860a4229b"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1DE4120D-B400-435F-B862-B3B8683830A5}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -9806,6 +9789,23 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{268822B0-DCAE-4D2C-8340-AB7554C48D72}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="D75E00DB-06CE-4005-B397-8C0860A4229B"/>
+    <ds:schemaRef ds:uri="372b77af-8063-48a8-888c-73c0edf01dea"/>
+    <ds:schemaRef ds:uri="d75e00db-06ce-4005-b397-8c0860a4229b"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2653FDDC-5C81-4B5A-A42F-7A63208AFFF7}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
2244 - Remove HIstorical Metrics from Excel Export
</commit_message>
<xml_diff>
--- a/GenBOE/GenBOE.Web/Templates/Export/WorkspaceDataMST.xlsx
+++ b/GenBOE/GenBOE.Web/Templates/Export/WorkspaceDataMST.xlsx
@@ -5,12 +5,12 @@
   <workbookPr showPivotChartFilter="1" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\twilson3\source\IES\GenBOE\GenBOE.Web\Templates\Export\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ranzalon\Source\repos\IES\GenBOE\GenBOE.Web\Templates\Export\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{709B05D6-9678-4BC2-BA45-58A1F0827487}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AFA9CCD1-A055-466C-9FD1-BAB931D763CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="19395" windowHeight="15585" firstSheet="5" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="5" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="BOE3 Pivot" sheetId="19" state="hidden" r:id="rId1"/>
@@ -38,8 +38,8 @@
     <externalReference r:id="rId21"/>
   </externalReferences>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'BOE &amp; Resource Combo'!$A$1:$AU$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">BOEs!$A$1:$AV$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'BOE &amp; Resource Combo'!$A$1:$AT$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">BOEs!$A$1:$AU$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'BOEs (2)'!$B$1:$T$16</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'BOEs (3)'!$A$1:$N$16</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Current Skill Mix'!$A$1:$N$1</definedName>
@@ -324,7 +324,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="921" uniqueCount="156">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="919" uniqueCount="155">
   <si>
     <t>Start Date</t>
   </si>
@@ -600,9 +600,6 @@
   </si>
   <si>
     <t>Month</t>
-  </si>
-  <si>
-    <t>Historical Metrics</t>
   </si>
   <si>
     <t>Perf Org Description</t>
@@ -3192,7 +3189,7 @@
 <file path=xl/pivotCache/pivotCacheDefinition2.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="Lindsay Yorks" refreshedDate="40653.729487847224" createdVersion="3" refreshedVersion="3" minRefreshableVersion="3" recordCount="15" xr:uid="{00000000-000A-0000-FFFF-FFFF01000000}">
   <cacheSource type="worksheet">
-    <worksheetSource ref="C1:AU1" sheet="BOEs"/>
+    <worksheetSource ref="C1:AT1" sheet="BOEs"/>
   </cacheSource>
   <cacheFields count="19">
     <cacheField name="Type" numFmtId="49">
@@ -6222,10 +6219,10 @@
         <v>70</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="D1" s="5" t="s">
         <v>2</v>
@@ -6234,13 +6231,13 @@
         <v>3</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="G1" s="5" t="s">
         <v>84</v>
       </c>
       <c r="H1" s="5" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
@@ -6285,10 +6282,10 @@
         <v>70</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="D1" s="5" t="s">
         <v>2</v>
@@ -6300,43 +6297,43 @@
         <v>84</v>
       </c>
       <c r="G1" s="5" t="s">
+        <v>126</v>
+      </c>
+      <c r="H1" s="5" t="s">
         <v>127</v>
       </c>
-      <c r="H1" s="5" t="s">
+      <c r="I1" s="5" t="s">
         <v>128</v>
       </c>
-      <c r="I1" s="5" t="s">
+      <c r="J1" s="5" t="s">
         <v>129</v>
       </c>
-      <c r="J1" s="5" t="s">
+      <c r="K1" s="5" t="s">
         <v>130</v>
       </c>
-      <c r="K1" s="5" t="s">
+      <c r="L1" s="5" t="s">
         <v>131</v>
       </c>
-      <c r="L1" s="5" t="s">
+      <c r="M1" s="5" t="s">
         <v>132</v>
       </c>
-      <c r="M1" s="5" t="s">
+      <c r="N1" s="31" t="s">
+        <v>137</v>
+      </c>
+      <c r="O1" s="31" t="s">
         <v>133</v>
       </c>
-      <c r="N1" s="31" t="s">
-        <v>138</v>
-      </c>
-      <c r="O1" s="31" t="s">
+      <c r="P1" s="5" t="s">
         <v>134</v>
       </c>
-      <c r="P1" s="5" t="s">
+      <c r="Q1" s="31" t="s">
         <v>135</v>
       </c>
-      <c r="Q1" s="31" t="s">
+      <c r="R1" s="5" t="s">
+        <v>139</v>
+      </c>
+      <c r="S1" s="5" t="s">
         <v>136</v>
-      </c>
-      <c r="R1" s="5" t="s">
-        <v>140</v>
-      </c>
-      <c r="S1" s="5" t="s">
-        <v>137</v>
       </c>
     </row>
     <row r="2" spans="1:19" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
@@ -6377,10 +6374,10 @@
         <v>70</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="D1" s="5" t="s">
         <v>2</v>
@@ -6395,25 +6392,25 @@
         <v>41</v>
       </c>
       <c r="H1" s="5" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="I1" s="60" t="s">
+        <v>146</v>
+      </c>
+      <c r="J1" s="33" t="s">
         <v>147</v>
       </c>
-      <c r="J1" s="33" t="s">
-        <v>148</v>
-      </c>
       <c r="K1" s="5" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="L1" s="33" t="s">
+        <v>149</v>
+      </c>
+      <c r="M1" s="5" t="s">
         <v>150</v>
       </c>
-      <c r="M1" s="5" t="s">
+      <c r="N1" s="5" t="s">
         <v>151</v>
-      </c>
-      <c r="N1" s="5" t="s">
-        <v>152</v>
       </c>
     </row>
     <row r="2" spans="1:14" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
@@ -6449,10 +6446,10 @@
         <v>70</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="D1" s="5" t="s">
         <v>2</v>
@@ -6464,28 +6461,28 @@
         <v>84</v>
       </c>
       <c r="G1" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="H1" s="5" t="s">
         <v>154</v>
       </c>
-      <c r="H1" s="5" t="s">
-        <v>155</v>
-      </c>
       <c r="I1" s="60" t="s">
+        <v>146</v>
+      </c>
+      <c r="J1" s="33" t="s">
         <v>147</v>
       </c>
-      <c r="J1" s="33" t="s">
+      <c r="K1" s="5" t="s">
         <v>148</v>
       </c>
-      <c r="K1" s="5" t="s">
+      <c r="L1" s="33" t="s">
         <v>149</v>
       </c>
-      <c r="L1" s="33" t="s">
+      <c r="M1" s="5" t="s">
         <v>150</v>
       </c>
-      <c r="M1" s="5" t="s">
+      <c r="N1" s="5" t="s">
         <v>151</v>
-      </c>
-      <c r="N1" s="5" t="s">
-        <v>152</v>
       </c>
     </row>
     <row r="2" spans="1:14" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
@@ -6520,7 +6517,7 @@
         <v>69</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="13.5" thickTop="1" x14ac:dyDescent="0.2"/>
@@ -6549,7 +6546,7 @@
   <sheetData>
     <row r="1" spans="1:5" s="5" customFormat="1" ht="20.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B1" s="5" t="s">
         <v>29</v>
@@ -6609,7 +6606,7 @@
         <v>65</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="G1" s="2" t="s">
         <v>75</v>
@@ -6618,7 +6615,7 @@
         <v>76</v>
       </c>
       <c r="I1" s="2" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="2" spans="1:9" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
@@ -6655,7 +6652,7 @@
     </row>
     <row r="4" spans="1:1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="10" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="5" spans="1:1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
@@ -6675,17 +6672,17 @@
     </row>
     <row r="8" spans="1:1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="11" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="9" spans="1:1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="11" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
     <row r="10" spans="1:1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="12" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="11" spans="1:1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
@@ -6695,17 +6692,17 @@
     </row>
     <row r="12" spans="1:1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="10" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="13" spans="1:1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="19" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="14" spans="1:1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="19" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
     <row r="15" spans="1:1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
@@ -6936,7 +6933,7 @@
       <c r="Q7" s="43"/>
       <c r="R7" s="43"/>
       <c r="S7" s="43" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="T7"/>
     </row>
@@ -9077,7 +9074,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
-  <dimension ref="A1:AU2"/>
+  <dimension ref="A1:AT2"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.140625" style="1" bestFit="1" customWidth="1"/>
@@ -9101,43 +9098,42 @@
     <col min="20" max="20" width="18.7109375" style="30" bestFit="1" customWidth="1"/>
     <col min="21" max="21" width="17.140625" style="1" bestFit="1" customWidth="1"/>
     <col min="22" max="22" width="20.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="21.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="13.7109375" style="37" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="12.85546875" style="37" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="21.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="20.42578125" style="32" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="19" style="30" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="20" style="1" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="24.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="18.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="18.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="33" max="36" width="18.5703125" style="1" customWidth="1"/>
-    <col min="37" max="37" width="18.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="38" max="38" width="23.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="39" max="39" width="16.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="40" max="40" width="13" style="34" bestFit="1" customWidth="1"/>
-    <col min="41" max="41" width="17" style="32" bestFit="1" customWidth="1"/>
-    <col min="42" max="42" width="15.7109375" style="30" bestFit="1" customWidth="1"/>
-    <col min="43" max="43" width="26.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="44" max="44" width="8.7109375" style="39" customWidth="1"/>
-    <col min="45" max="45" width="10.5703125" style="39" bestFit="1" customWidth="1"/>
-    <col min="46" max="46" width="10" style="32" bestFit="1" customWidth="1"/>
-    <col min="47" max="47" width="8.7109375" style="30" customWidth="1"/>
-    <col min="48" max="16384" width="9.140625" style="1"/>
+    <col min="23" max="23" width="13.7109375" style="37" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="12.85546875" style="37" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="21.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="20.42578125" style="32" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="19" style="30" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="20" style="1" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="24.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="18.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="18.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="32" max="35" width="18.5703125" style="1" customWidth="1"/>
+    <col min="36" max="36" width="18.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="23.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="38" max="38" width="16.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="39" max="39" width="13" style="34" bestFit="1" customWidth="1"/>
+    <col min="40" max="40" width="17" style="32" bestFit="1" customWidth="1"/>
+    <col min="41" max="41" width="15.7109375" style="30" bestFit="1" customWidth="1"/>
+    <col min="42" max="42" width="26.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="43" max="43" width="8.7109375" style="39" customWidth="1"/>
+    <col min="44" max="44" width="10.5703125" style="39" bestFit="1" customWidth="1"/>
+    <col min="45" max="45" width="10" style="32" bestFit="1" customWidth="1"/>
+    <col min="46" max="46" width="8.7109375" style="30" customWidth="1"/>
+    <col min="47" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:47" s="5" customFormat="1" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:46" s="5" customFormat="1" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
         <v>70</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C1" s="5" t="s">
         <v>26</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="E1" s="2" t="s">
         <v>2</v>
@@ -9146,13 +9142,13 @@
         <v>3</v>
       </c>
       <c r="G1" s="5" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="H1" s="2" t="s">
         <v>84</v>
       </c>
       <c r="I1" s="5" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="J1" s="2" t="s">
         <v>87</v>
@@ -9164,7 +9160,7 @@
         <v>28</v>
       </c>
       <c r="M1" s="5" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="N1" s="5" t="s">
         <v>29</v>
@@ -9179,49 +9175,49 @@
         <v>32</v>
       </c>
       <c r="R1" s="5" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="S1" s="31" t="s">
         <v>86</v>
       </c>
       <c r="T1" s="25" t="s">
+        <v>99</v>
+      </c>
+      <c r="U1" s="5" t="s">
         <v>100</v>
-      </c>
-      <c r="U1" s="5" t="s">
-        <v>101</v>
       </c>
       <c r="V1" s="5" t="s">
         <v>83</v>
       </c>
-      <c r="W1" s="5" t="s">
-        <v>92</v>
+      <c r="W1" s="36" t="s">
+        <v>4</v>
       </c>
       <c r="X1" s="36" t="s">
-        <v>4</v>
-      </c>
-      <c r="Y1" s="36" t="s">
         <v>5</v>
       </c>
-      <c r="Z1" s="5" t="s">
-        <v>95</v>
-      </c>
-      <c r="AA1" s="31" t="s">
+      <c r="Y1" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="Z1" s="31" t="s">
         <v>85</v>
       </c>
-      <c r="AB1" s="25" t="s">
+      <c r="AA1" s="25" t="s">
+        <v>101</v>
+      </c>
+      <c r="AB1" s="5" t="s">
         <v>102</v>
       </c>
       <c r="AC1" s="5" t="s">
-        <v>103</v>
+        <v>89</v>
       </c>
       <c r="AD1" s="5" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="AE1" s="5" t="s">
-        <v>88</v>
+        <v>104</v>
       </c>
       <c r="AF1" s="5" t="s">
-        <v>105</v>
+        <v>140</v>
       </c>
       <c r="AG1" s="5" t="s">
         <v>141</v>
@@ -9233,45 +9229,42 @@
         <v>143</v>
       </c>
       <c r="AJ1" s="5" t="s">
-        <v>144</v>
+        <v>11</v>
       </c>
       <c r="AK1" s="5" t="s">
-        <v>11</v>
+        <v>92</v>
       </c>
       <c r="AL1" s="5" t="s">
-        <v>93</v>
-      </c>
-      <c r="AM1" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="AN1" s="33" t="s">
+      <c r="AM1" s="33" t="s">
         <v>14</v>
       </c>
-      <c r="AO1" s="31" t="s">
+      <c r="AN1" s="31" t="s">
         <v>15</v>
       </c>
-      <c r="AP1" s="25" t="s">
+      <c r="AO1" s="25" t="s">
+        <v>108</v>
+      </c>
+      <c r="AP1" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="AQ1" s="38" t="s">
+        <v>90</v>
+      </c>
+      <c r="AR1" s="38" t="s">
+        <v>91</v>
+      </c>
+      <c r="AS1" s="35" t="s">
         <v>109</v>
       </c>
-      <c r="AQ1" s="5" t="s">
-        <v>99</v>
-      </c>
-      <c r="AR1" s="38" t="s">
-        <v>90</v>
-      </c>
-      <c r="AS1" s="38" t="s">
-        <v>91</v>
-      </c>
-      <c r="AT1" s="35" t="s">
+      <c r="AT1" s="28" t="s">
         <v>110</v>
       </c>
-      <c r="AU1" s="28" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="2" spans="1:47" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
+    </row>
+    <row r="2" spans="1:46" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
   </sheetData>
-  <autoFilter ref="A1:AU1" xr:uid="{00000000-0009-0000-0000-000005000000}"/>
+  <autoFilter ref="A1:AT1" xr:uid="{00000000-0009-0000-0000-000005000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
   <headerFooter>
@@ -9283,7 +9276,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
-  <dimension ref="A1:AV2"/>
+  <dimension ref="A1:AU2"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.42578125" style="3" customWidth="1"/>
@@ -9304,34 +9297,33 @@
     <col min="19" max="19" width="18.42578125" style="3" bestFit="1" customWidth="1"/>
     <col min="20" max="20" width="23.85546875" style="3" bestFit="1" customWidth="1"/>
     <col min="21" max="21" width="19" style="3" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="21.140625" style="3" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="13.7109375" style="3" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="12.85546875" style="3" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="21.7109375" style="3" customWidth="1"/>
-    <col min="26" max="26" width="20.42578125" style="21" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="20.42578125" style="26" customWidth="1"/>
-    <col min="28" max="28" width="20.42578125" style="3" customWidth="1"/>
-    <col min="29" max="29" width="24.7109375" style="3" bestFit="1" customWidth="1"/>
-    <col min="30" max="32" width="24.7109375" style="3" customWidth="1"/>
-    <col min="33" max="36" width="18.5703125" style="1" customWidth="1"/>
-    <col min="37" max="37" width="18.85546875" style="3" bestFit="1" customWidth="1"/>
-    <col min="38" max="41" width="18.85546875" style="3" customWidth="1"/>
-    <col min="42" max="42" width="13.85546875" style="3" bestFit="1" customWidth="1"/>
-    <col min="43" max="43" width="13" style="3" bestFit="1" customWidth="1"/>
-    <col min="44" max="44" width="16.85546875" style="3" bestFit="1" customWidth="1"/>
-    <col min="45" max="45" width="13" style="18" bestFit="1" customWidth="1"/>
-    <col min="46" max="46" width="13" style="21" customWidth="1"/>
-    <col min="47" max="47" width="17" style="26" bestFit="1" customWidth="1"/>
-    <col min="48" max="48" width="24.85546875" style="3" bestFit="1" customWidth="1"/>
-    <col min="49" max="16384" width="9.140625" style="3"/>
+    <col min="22" max="22" width="13.7109375" style="3" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="12.85546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="21.7109375" style="3" customWidth="1"/>
+    <col min="25" max="25" width="20.42578125" style="21" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="20.42578125" style="26" customWidth="1"/>
+    <col min="27" max="27" width="20.42578125" style="3" customWidth="1"/>
+    <col min="28" max="28" width="24.7109375" style="3" bestFit="1" customWidth="1"/>
+    <col min="29" max="31" width="24.7109375" style="3" customWidth="1"/>
+    <col min="32" max="35" width="18.5703125" style="1" customWidth="1"/>
+    <col min="36" max="36" width="18.85546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="37" max="40" width="18.85546875" style="3" customWidth="1"/>
+    <col min="41" max="41" width="13.85546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="42" max="42" width="13" style="3" bestFit="1" customWidth="1"/>
+    <col min="43" max="43" width="16.85546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="44" max="44" width="13" style="18" bestFit="1" customWidth="1"/>
+    <col min="45" max="45" width="13" style="21" customWidth="1"/>
+    <col min="46" max="46" width="17" style="26" bestFit="1" customWidth="1"/>
+    <col min="47" max="47" width="24.85546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="48" max="16384" width="9.140625" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:48" s="5" customFormat="1" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:47" s="5" customFormat="1" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
         <v>70</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C1" s="5" t="s">
         <v>26</v>
@@ -9355,22 +9347,22 @@
         <v>32</v>
       </c>
       <c r="J1" s="5" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="K1" s="20" t="s">
         <v>86</v>
       </c>
       <c r="L1" s="25" t="s">
+        <v>99</v>
+      </c>
+      <c r="M1" s="25" t="s">
+        <v>123</v>
+      </c>
+      <c r="N1" s="5" t="s">
         <v>100</v>
       </c>
-      <c r="M1" s="25" t="s">
-        <v>124</v>
-      </c>
-      <c r="N1" s="5" t="s">
-        <v>101</v>
-      </c>
       <c r="O1" s="5" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="P1" s="5" t="s">
         <v>2</v>
@@ -9382,46 +9374,46 @@
         <v>83</v>
       </c>
       <c r="S1" s="5" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="T1" s="5" t="s">
         <v>84</v>
       </c>
       <c r="U1" s="5" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="V1" s="5" t="s">
-        <v>92</v>
+        <v>4</v>
       </c>
       <c r="W1" s="5" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="X1" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="Y1" s="5" t="s">
-        <v>95</v>
-      </c>
-      <c r="Z1" s="20" t="s">
+        <v>94</v>
+      </c>
+      <c r="Y1" s="20" t="s">
         <v>85</v>
       </c>
-      <c r="AA1" s="25" t="s">
+      <c r="Z1" s="25" t="s">
+        <v>101</v>
+      </c>
+      <c r="AA1" s="5" t="s">
         <v>102</v>
       </c>
       <c r="AB1" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="AC1" s="5" t="s">
         <v>103</v>
       </c>
-      <c r="AC1" s="5" t="s">
-        <v>89</v>
-      </c>
       <c r="AD1" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="AE1" s="5" t="s">
         <v>104</v>
       </c>
-      <c r="AE1" s="5" t="s">
-        <v>88</v>
-      </c>
       <c r="AF1" s="5" t="s">
-        <v>105</v>
+        <v>140</v>
       </c>
       <c r="AG1" s="5" t="s">
         <v>141</v>
@@ -9433,13 +9425,13 @@
         <v>143</v>
       </c>
       <c r="AJ1" s="5" t="s">
-        <v>144</v>
+        <v>11</v>
       </c>
       <c r="AK1" s="5" t="s">
-        <v>11</v>
+        <v>92</v>
       </c>
       <c r="AL1" s="5" t="s">
-        <v>93</v>
+        <v>105</v>
       </c>
       <c r="AM1" s="5" t="s">
         <v>106</v>
@@ -9448,33 +9440,30 @@
         <v>107</v>
       </c>
       <c r="AO1" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="AP1" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="AQ1" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="AR1" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="AS1" s="20" t="s">
+        <v>15</v>
+      </c>
+      <c r="AT1" s="25" t="s">
         <v>108</v>
       </c>
-      <c r="AP1" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="AQ1" s="5" t="s">
-        <v>1</v>
-      </c>
-      <c r="AR1" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="AS1" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="AT1" s="20" t="s">
-        <v>15</v>
-      </c>
-      <c r="AU1" s="25" t="s">
-        <v>109</v>
-      </c>
-      <c r="AV1" s="5" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="2" spans="1:48" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
+      <c r="AU1" s="5" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="2" spans="1:47" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
   </sheetData>
-  <autoFilter ref="A1:AV1" xr:uid="{00000000-0009-0000-0000-000006000000}"/>
+  <autoFilter ref="A1:AU1" xr:uid="{00000000-0009-0000-0000-000006000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
   <headerFooter>
@@ -9511,7 +9500,7 @@
         <v>28</v>
       </c>
       <c r="C1" s="9" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D1" s="9" t="s">
         <v>29</v>
@@ -9529,10 +9518,10 @@
         <v>6</v>
       </c>
       <c r="I1" s="25" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="J1" s="9" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="K1" s="9" t="s">
         <v>66</v>
@@ -9541,10 +9530,10 @@
         <v>67</v>
       </c>
       <c r="M1" s="9" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="N1" s="9" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="2" spans="1:14" ht="13.5" thickTop="1" x14ac:dyDescent="0.2"/>
@@ -9582,7 +9571,7 @@
   <sheetData>
     <row r="1" spans="1:17" s="2" customFormat="1" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>2</v>
@@ -9612,10 +9601,10 @@
         <v>88</v>
       </c>
       <c r="K1" s="5" t="s">
+        <v>142</v>
+      </c>
+      <c r="L1" s="5" t="s">
         <v>143</v>
-      </c>
-      <c r="L1" s="5" t="s">
-        <v>144</v>
       </c>
       <c r="M1" s="2" t="s">
         <v>11</v>
@@ -9627,10 +9616,10 @@
         <v>91</v>
       </c>
       <c r="P1" s="23" t="s">
+        <v>109</v>
+      </c>
+      <c r="Q1" s="28" t="s">
         <v>110</v>
-      </c>
-      <c r="Q1" s="28" t="s">
-        <v>111</v>
       </c>
     </row>
     <row r="2" spans="1:17" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
@@ -9646,6 +9635,19 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance">
+  <documentManagement>
+    <Unity_Description xmlns="D75E00DB-06CE-4005-B397-8C0860A4229B" xsi:nil="true"/>
+    <Unity_Tag xmlns="D75E00DB-06CE-4005-B397-8C0860A4229B" xsi:nil="true"/>
+    <Capabilities xmlns="d75e00db-06ce-4005-b397-8c0860a4229b" xsi:nil="true"/>
+    <SipLabel xmlns="372b77af-8063-48a8-888c-73c0edf01dea">
+      <Value>2</Value>
+    </SipLabel>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Custom Document" ma:contentTypeID="0x010100E6322E8F405D4D9EA89D8C83B7E1048B001BB96E1BE0ACBB41BF00782ED0412411" ma:contentTypeVersion="3" ma:contentTypeDescription="Custom Document" ma:contentTypeScope="" ma:versionID="3c14126572fa3c0d4c677ac1f3ba4426">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="D75E00DB-06CE-4005-B397-8C0860A4229B" xmlns:ns3="372b77af-8063-48a8-888c-73c0edf01dea" xmlns:ns4="d75e00db-06ce-4005-b397-8c0860a4229b" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="9e89026a025b72b85b9543506e7af3e1" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="D75E00DB-06CE-4005-B397-8C0860A4229B"/>
@@ -9748,19 +9750,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance">
-  <documentManagement>
-    <Unity_Description xmlns="D75E00DB-06CE-4005-B397-8C0860A4229B" xsi:nil="true"/>
-    <Unity_Tag xmlns="D75E00DB-06CE-4005-B397-8C0860A4229B" xsi:nil="true"/>
-    <Capabilities xmlns="d75e00db-06ce-4005-b397-8c0860a4229b" xsi:nil="true"/>
-    <SipLabel xmlns="372b77af-8063-48a8-888c-73c0edf01dea">
-      <Value>2</Value>
-    </SipLabel>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -9771,6 +9760,23 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{268822B0-DCAE-4D2C-8340-AB7554C48D72}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="D75E00DB-06CE-4005-B397-8C0860A4229B"/>
+    <ds:schemaRef ds:uri="372b77af-8063-48a8-888c-73c0edf01dea"/>
+    <ds:schemaRef ds:uri="d75e00db-06ce-4005-b397-8c0860a4229b"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1DE4120D-B400-435F-B862-B3B8683830A5}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -9789,23 +9795,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{268822B0-DCAE-4D2C-8340-AB7554C48D72}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="D75E00DB-06CE-4005-B397-8C0860A4229B"/>
-    <ds:schemaRef ds:uri="372b77af-8063-48a8-888c-73c0edf01dea"/>
-    <ds:schemaRef ds:uri="d75e00db-06ce-4005-b397-8c0860a4229b"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2653FDDC-5C81-4B5A-A42F-7A63208AFFF7}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
Conditionally added Task Author to workspace data report
</commit_message>
<xml_diff>
--- a/GenBOE/GenBOE.Web/Templates/Export/WorkspaceDataMST.xlsx
+++ b/GenBOE/GenBOE.Web/Templates/Export/WorkspaceDataMST.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27928"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
   <workbookPr showPivotChartFilter="1" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ranzalon\Source\repos\IES\GenBOE\GenBOE.Web\Templates\Export\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\IES\IES\GenBOE\GenBOE.Web\Templates\Export\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AFA9CCD1-A055-466C-9FD1-BAB931D763CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC2AB81B-094D-4F94-87D5-7D9A2B62B987}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="5" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="20085" yWindow="-15105" windowWidth="21600" windowHeight="12645" firstSheet="5" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="BOE3 Pivot" sheetId="19" state="hidden" r:id="rId1"/>
@@ -38,7 +38,7 @@
     <externalReference r:id="rId21"/>
   </externalReferences>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'BOE &amp; Resource Combo'!$A$1:$AT$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'BOE &amp; Resource Combo'!$A$1:$AU$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">BOEs!$A$1:$AU$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'BOEs (2)'!$B$1:$T$16</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'BOEs (3)'!$A$1:$N$16</definedName>
@@ -57,9 +57,9 @@
   </definedNames>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="0" r:id="rId22"/>
-    <pivotCache cacheId="1" r:id="rId23"/>
-    <pivotCache cacheId="2" r:id="rId24"/>
+    <pivotCache cacheId="51" r:id="rId22"/>
+    <pivotCache cacheId="52" r:id="rId23"/>
+    <pivotCache cacheId="53" r:id="rId24"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -324,7 +324,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="919" uniqueCount="155">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="920" uniqueCount="156">
   <si>
     <t>Start Date</t>
   </si>
@@ -789,6 +789,9 @@
   </si>
   <si>
     <t>Business Resource Code</t>
+  </si>
+  <si>
+    <t>Task Author</t>
   </si>
 </sst>
 </file>
@@ -4393,7 +4396,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0000-000000000000}" name="PivotTable7" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="3" minRefreshableVersion="3" showCalcMbrs="0" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="3" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0000-000000000000}" name="PivotTable7" cacheId="51" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="3" minRefreshableVersion="3" showCalcMbrs="0" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="3" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
   <location ref="A3:N33" firstHeaderRow="1" firstDataRow="1" firstDataCol="14"/>
   <pivotFields count="14">
     <pivotField axis="axisRow" compact="0" outline="0" showAll="0" insertBlankRow="1" defaultSubtotal="0">
@@ -4742,7 +4745,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0200-000000000000}" name="PivotTable9" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="3" minRefreshableVersion="3" showCalcMbrs="0" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="3" indent="0" compact="0" compactData="0" multipleFieldFilters="0" rowHeaderCaption="Type">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0200-000000000000}" name="PivotTable9" cacheId="52" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="3" minRefreshableVersion="3" showCalcMbrs="0" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="3" indent="0" compact="0" compactData="0" multipleFieldFilters="0" rowHeaderCaption="Type">
   <location ref="A3:H11" firstHeaderRow="1" firstDataRow="1" firstDataCol="8"/>
   <pivotFields count="19">
     <pivotField axis="axisRow" compact="0" outline="0" showAll="0" defaultSubtotal="0">
@@ -4951,7 +4954,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0300-000000000000}" name="PivotTable4" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" missingCaption="_" updatedVersion="3" minRefreshableVersion="3" showCalcMbrs="0" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="3" indent="0" compact="0" compactData="0" multipleFieldFilters="0" rowHeaderCaption="BOE ID">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0300-000000000000}" name="PivotTable4" cacheId="53" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" missingCaption="_" updatedVersion="3" minRefreshableVersion="3" showCalcMbrs="0" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="3" indent="0" compact="0" compactData="0" multipleFieldFilters="0" rowHeaderCaption="BOE ID">
   <location ref="A3:T33" firstHeaderRow="1" firstDataRow="1" firstDataCol="20"/>
   <pivotFields count="20">
     <pivotField axis="axisRow" compact="0" outline="0" showAll="0" insertBlankRow="1" defaultSubtotal="0">
@@ -9074,7 +9077,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
-  <dimension ref="A1:AT2"/>
+  <dimension ref="A1:AU2"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.140625" style="1" bestFit="1" customWidth="1"/>
@@ -9082,47 +9085,48 @@
     <col min="3" max="4" width="15.85546875" style="1" customWidth="1"/>
     <col min="5" max="5" width="11.42578125" style="1" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="13.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="18.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="14.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="19.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="19.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="10.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="13.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="19.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="10.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="13.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="13.42578125" style="37" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="12.5703125" style="37" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="21.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="20.140625" style="32" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="18.7109375" style="30" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="17.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="20.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="13.7109375" style="37" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="12.85546875" style="37" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="21.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="20.42578125" style="32" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="19" style="30" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="20" style="1" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="24.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="18.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="18.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="32" max="35" width="18.5703125" style="1" customWidth="1"/>
-    <col min="36" max="36" width="18.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="23.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="38" max="38" width="16.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="39" max="39" width="13" style="34" bestFit="1" customWidth="1"/>
-    <col min="40" max="40" width="17" style="32" bestFit="1" customWidth="1"/>
-    <col min="41" max="41" width="15.7109375" style="30" bestFit="1" customWidth="1"/>
-    <col min="42" max="42" width="26.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="43" max="43" width="8.7109375" style="39" customWidth="1"/>
-    <col min="44" max="44" width="10.5703125" style="39" bestFit="1" customWidth="1"/>
-    <col min="45" max="45" width="10" style="32" bestFit="1" customWidth="1"/>
-    <col min="46" max="46" width="8.7109375" style="30" customWidth="1"/>
-    <col min="47" max="16384" width="9.140625" style="1"/>
+    <col min="7" max="7" width="13.5703125" style="1" customWidth="1"/>
+    <col min="8" max="8" width="18.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="14.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="19.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="19.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="10.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="13.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="19.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="10.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="13.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="13.42578125" style="37" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="12.5703125" style="37" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="21.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="20.140625" style="32" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="18.7109375" style="30" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="17.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="20.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="13.7109375" style="37" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="12.85546875" style="37" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="21.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="20.42578125" style="32" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="19" style="30" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="20" style="1" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="24.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="18.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="18.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="33" max="36" width="18.5703125" style="1" customWidth="1"/>
+    <col min="37" max="37" width="18.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="38" max="38" width="23.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="39" max="39" width="16.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="40" max="40" width="13" style="34" bestFit="1" customWidth="1"/>
+    <col min="41" max="41" width="17" style="32" bestFit="1" customWidth="1"/>
+    <col min="42" max="42" width="15.7109375" style="30" bestFit="1" customWidth="1"/>
+    <col min="43" max="43" width="26.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="44" max="44" width="8.7109375" style="39" customWidth="1"/>
+    <col min="45" max="45" width="10.5703125" style="39" bestFit="1" customWidth="1"/>
+    <col min="46" max="46" width="10" style="32" bestFit="1" customWidth="1"/>
+    <col min="47" max="47" width="8.7109375" style="30" customWidth="1"/>
+    <col min="48" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:46" s="5" customFormat="1" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:47" s="5" customFormat="1" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
         <v>70</v>
       </c>
@@ -9141,130 +9145,133 @@
       <c r="F1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="G1" s="5" t="s">
+      <c r="G1" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="H1" s="5" t="s">
         <v>118</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="I1" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="I1" s="5" t="s">
+      <c r="J1" s="5" t="s">
         <v>117</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="K1" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="K1" s="5" t="s">
+      <c r="L1" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="L1" s="5" t="s">
+      <c r="M1" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="M1" s="5" t="s">
+      <c r="N1" s="5" t="s">
         <v>123</v>
       </c>
-      <c r="N1" s="5" t="s">
+      <c r="O1" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="O1" s="5" t="s">
+      <c r="P1" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="P1" s="36" t="s">
+      <c r="Q1" s="36" t="s">
         <v>31</v>
       </c>
-      <c r="Q1" s="36" t="s">
+      <c r="R1" s="36" t="s">
         <v>32</v>
       </c>
-      <c r="R1" s="5" t="s">
+      <c r="S1" s="5" t="s">
         <v>93</v>
       </c>
-      <c r="S1" s="31" t="s">
+      <c r="T1" s="31" t="s">
         <v>86</v>
       </c>
-      <c r="T1" s="25" t="s">
+      <c r="U1" s="25" t="s">
         <v>99</v>
       </c>
-      <c r="U1" s="5" t="s">
+      <c r="V1" s="5" t="s">
         <v>100</v>
       </c>
-      <c r="V1" s="5" t="s">
+      <c r="W1" s="5" t="s">
         <v>83</v>
       </c>
-      <c r="W1" s="36" t="s">
+      <c r="X1" s="36" t="s">
         <v>4</v>
       </c>
-      <c r="X1" s="36" t="s">
+      <c r="Y1" s="36" t="s">
         <v>5</v>
       </c>
-      <c r="Y1" s="5" t="s">
+      <c r="Z1" s="5" t="s">
         <v>94</v>
       </c>
-      <c r="Z1" s="31" t="s">
+      <c r="AA1" s="31" t="s">
         <v>85</v>
       </c>
-      <c r="AA1" s="25" t="s">
+      <c r="AB1" s="25" t="s">
         <v>101</v>
       </c>
-      <c r="AB1" s="5" t="s">
+      <c r="AC1" s="5" t="s">
         <v>102</v>
       </c>
-      <c r="AC1" s="5" t="s">
+      <c r="AD1" s="5" t="s">
         <v>89</v>
       </c>
-      <c r="AD1" s="5" t="s">
+      <c r="AE1" s="5" t="s">
         <v>88</v>
       </c>
-      <c r="AE1" s="5" t="s">
+      <c r="AF1" s="5" t="s">
         <v>104</v>
       </c>
-      <c r="AF1" s="5" t="s">
+      <c r="AG1" s="5" t="s">
         <v>140</v>
       </c>
-      <c r="AG1" s="5" t="s">
+      <c r="AH1" s="5" t="s">
         <v>141</v>
       </c>
-      <c r="AH1" s="5" t="s">
+      <c r="AI1" s="5" t="s">
         <v>142</v>
       </c>
-      <c r="AI1" s="5" t="s">
+      <c r="AJ1" s="5" t="s">
         <v>143</v>
       </c>
-      <c r="AJ1" s="5" t="s">
+      <c r="AK1" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="AK1" s="5" t="s">
+      <c r="AL1" s="5" t="s">
         <v>92</v>
       </c>
-      <c r="AL1" s="5" t="s">
+      <c r="AM1" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="AM1" s="33" t="s">
+      <c r="AN1" s="33" t="s">
         <v>14</v>
       </c>
-      <c r="AN1" s="31" t="s">
+      <c r="AO1" s="31" t="s">
         <v>15</v>
       </c>
-      <c r="AO1" s="25" t="s">
+      <c r="AP1" s="25" t="s">
         <v>108</v>
       </c>
-      <c r="AP1" s="5" t="s">
+      <c r="AQ1" s="5" t="s">
         <v>98</v>
       </c>
-      <c r="AQ1" s="38" t="s">
+      <c r="AR1" s="38" t="s">
         <v>90</v>
       </c>
-      <c r="AR1" s="38" t="s">
+      <c r="AS1" s="38" t="s">
         <v>91</v>
       </c>
-      <c r="AS1" s="35" t="s">
+      <c r="AT1" s="35" t="s">
         <v>109</v>
       </c>
-      <c r="AT1" s="28" t="s">
+      <c r="AU1" s="28" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="2" spans="1:46" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
+    <row r="2" spans="1:47" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
   </sheetData>
-  <autoFilter ref="A1:AT1" xr:uid="{00000000-0009-0000-0000-000005000000}"/>
+  <autoFilter ref="A1:AU1" xr:uid="{00000000-0009-0000-0000-000005000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
   <headerFooter>

</xml_diff>

<commit_message>
3369 - Workspace Data Report - Add Task Author to BOEs tab, properly remove Task Author when disabled
</commit_message>
<xml_diff>
--- a/GenBOE/GenBOE.Web/Templates/Export/WorkspaceDataMST.xlsx
+++ b/GenBOE/GenBOE.Web/Templates/Export/WorkspaceDataMST.xlsx
@@ -5,12 +5,12 @@
   <workbookPr showPivotChartFilter="1" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\IES\IES\GenBOE\GenBOE.Web\Templates\Export\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ranzalon\Source\repos\IES\GenBOE\GenBOE.Web\Templates\Export\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC2AB81B-094D-4F94-87D5-7D9A2B62B987}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BAFB3397-7F53-4909-8E41-C9FA967C96DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20085" yWindow="-15105" windowWidth="21600" windowHeight="12645" firstSheet="5" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" firstSheet="5" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="BOE3 Pivot" sheetId="19" state="hidden" r:id="rId1"/>
@@ -39,7 +39,7 @@
   </externalReferences>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'BOE &amp; Resource Combo'!$A$1:$AU$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">BOEs!$A$1:$AU$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">BOEs!$A$1:$AV$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'BOEs (2)'!$B$1:$T$16</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'BOEs (3)'!$A$1:$N$16</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Current Skill Mix'!$A$1:$N$1</definedName>
@@ -57,9 +57,9 @@
   </definedNames>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="51" r:id="rId22"/>
-    <pivotCache cacheId="52" r:id="rId23"/>
-    <pivotCache cacheId="53" r:id="rId24"/>
+    <pivotCache cacheId="9" r:id="rId22"/>
+    <pivotCache cacheId="10" r:id="rId23"/>
+    <pivotCache cacheId="11" r:id="rId24"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -324,7 +324,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="920" uniqueCount="156">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="921" uniqueCount="156">
   <si>
     <t>Start Date</t>
   </si>
@@ -3192,7 +3192,7 @@
 <file path=xl/pivotCache/pivotCacheDefinition2.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="Lindsay Yorks" refreshedDate="40653.729487847224" createdVersion="3" refreshedVersion="3" minRefreshableVersion="3" recordCount="15" xr:uid="{00000000-000A-0000-FFFF-FFFF01000000}">
   <cacheSource type="worksheet">
-    <worksheetSource ref="C1:AT1" sheet="BOEs"/>
+    <worksheetSource ref="C1:AU1" sheet="BOEs"/>
   </cacheSource>
   <cacheFields count="19">
     <cacheField name="Type" numFmtId="49">
@@ -4396,7 +4396,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0000-000000000000}" name="PivotTable7" cacheId="51" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="3" minRefreshableVersion="3" showCalcMbrs="0" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="3" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0000-000000000000}" name="PivotTable7" cacheId="9" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="3" minRefreshableVersion="3" showCalcMbrs="0" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="3" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
   <location ref="A3:N33" firstHeaderRow="1" firstDataRow="1" firstDataCol="14"/>
   <pivotFields count="14">
     <pivotField axis="axisRow" compact="0" outline="0" showAll="0" insertBlankRow="1" defaultSubtotal="0">
@@ -4745,7 +4745,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0200-000000000000}" name="PivotTable9" cacheId="52" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="3" minRefreshableVersion="3" showCalcMbrs="0" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="3" indent="0" compact="0" compactData="0" multipleFieldFilters="0" rowHeaderCaption="Type">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0200-000000000000}" name="PivotTable9" cacheId="10" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="3" minRefreshableVersion="3" showCalcMbrs="0" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="3" indent="0" compact="0" compactData="0" multipleFieldFilters="0" rowHeaderCaption="Type">
   <location ref="A3:H11" firstHeaderRow="1" firstDataRow="1" firstDataCol="8"/>
   <pivotFields count="19">
     <pivotField axis="axisRow" compact="0" outline="0" showAll="0" defaultSubtotal="0">
@@ -4954,7 +4954,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0300-000000000000}" name="PivotTable4" cacheId="53" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" missingCaption="_" updatedVersion="3" minRefreshableVersion="3" showCalcMbrs="0" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="3" indent="0" compact="0" compactData="0" multipleFieldFilters="0" rowHeaderCaption="BOE ID">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0300-000000000000}" name="PivotTable4" cacheId="11" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" missingCaption="_" updatedVersion="3" minRefreshableVersion="3" showCalcMbrs="0" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="3" indent="0" compact="0" compactData="0" multipleFieldFilters="0" rowHeaderCaption="BOE ID">
   <location ref="A3:T33" firstHeaderRow="1" firstDataRow="1" firstDataCol="20"/>
   <pivotFields count="20">
     <pivotField axis="axisRow" compact="0" outline="0" showAll="0" insertBlankRow="1" defaultSubtotal="0">
@@ -9283,7 +9283,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
-  <dimension ref="A1:AU2"/>
+  <dimension ref="A1:AV2"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.42578125" style="3" customWidth="1"/>
@@ -9301,31 +9301,32 @@
     <col min="16" max="16" width="11.42578125" style="3" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="13.5703125" style="3" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="20.140625" style="3" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="18.42578125" style="3" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="23.85546875" style="3" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="19" style="3" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="13.7109375" style="3" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="12.85546875" style="3" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="21.7109375" style="3" customWidth="1"/>
-    <col min="25" max="25" width="20.42578125" style="21" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="20.42578125" style="26" customWidth="1"/>
-    <col min="27" max="27" width="20.42578125" style="3" customWidth="1"/>
-    <col min="28" max="28" width="24.7109375" style="3" bestFit="1" customWidth="1"/>
-    <col min="29" max="31" width="24.7109375" style="3" customWidth="1"/>
-    <col min="32" max="35" width="18.5703125" style="1" customWidth="1"/>
-    <col min="36" max="36" width="18.85546875" style="3" bestFit="1" customWidth="1"/>
-    <col min="37" max="40" width="18.85546875" style="3" customWidth="1"/>
-    <col min="41" max="41" width="13.85546875" style="3" bestFit="1" customWidth="1"/>
-    <col min="42" max="42" width="13" style="3" bestFit="1" customWidth="1"/>
-    <col min="43" max="43" width="16.85546875" style="3" bestFit="1" customWidth="1"/>
-    <col min="44" max="44" width="13" style="18" bestFit="1" customWidth="1"/>
-    <col min="45" max="45" width="13" style="21" customWidth="1"/>
-    <col min="46" max="46" width="17" style="26" bestFit="1" customWidth="1"/>
-    <col min="47" max="47" width="24.85546875" style="3" bestFit="1" customWidth="1"/>
-    <col min="48" max="16384" width="9.140625" style="3"/>
+    <col min="19" max="19" width="13.5703125" style="1" customWidth="1"/>
+    <col min="20" max="20" width="18.42578125" style="3" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="23.85546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="19" style="3" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="13.7109375" style="3" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="12.85546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="21.7109375" style="3" customWidth="1"/>
+    <col min="26" max="26" width="20.42578125" style="21" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="20.42578125" style="26" customWidth="1"/>
+    <col min="28" max="28" width="20.42578125" style="3" customWidth="1"/>
+    <col min="29" max="29" width="24.7109375" style="3" bestFit="1" customWidth="1"/>
+    <col min="30" max="32" width="24.7109375" style="3" customWidth="1"/>
+    <col min="33" max="36" width="18.5703125" style="1" customWidth="1"/>
+    <col min="37" max="37" width="18.85546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="38" max="41" width="18.85546875" style="3" customWidth="1"/>
+    <col min="42" max="42" width="13.85546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="43" max="43" width="13" style="3" bestFit="1" customWidth="1"/>
+    <col min="44" max="44" width="16.85546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="45" max="45" width="13" style="18" bestFit="1" customWidth="1"/>
+    <col min="46" max="46" width="13" style="21" customWidth="1"/>
+    <col min="47" max="47" width="17" style="26" bestFit="1" customWidth="1"/>
+    <col min="48" max="48" width="24.85546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="49" max="16384" width="9.140625" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:47" s="5" customFormat="1" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:48" s="5" customFormat="1" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
         <v>70</v>
       </c>
@@ -9380,97 +9381,100 @@
       <c r="R1" s="5" t="s">
         <v>83</v>
       </c>
-      <c r="S1" s="5" t="s">
+      <c r="S1" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="T1" s="5" t="s">
         <v>118</v>
       </c>
-      <c r="T1" s="5" t="s">
+      <c r="U1" s="5" t="s">
         <v>84</v>
       </c>
-      <c r="U1" s="5" t="s">
+      <c r="V1" s="5" t="s">
         <v>117</v>
       </c>
-      <c r="V1" s="5" t="s">
+      <c r="W1" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="W1" s="5" t="s">
+      <c r="X1" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="X1" s="5" t="s">
+      <c r="Y1" s="5" t="s">
         <v>94</v>
       </c>
-      <c r="Y1" s="20" t="s">
+      <c r="Z1" s="20" t="s">
         <v>85</v>
       </c>
-      <c r="Z1" s="25" t="s">
+      <c r="AA1" s="25" t="s">
         <v>101</v>
       </c>
-      <c r="AA1" s="5" t="s">
+      <c r="AB1" s="5" t="s">
         <v>102</v>
       </c>
-      <c r="AB1" s="5" t="s">
+      <c r="AC1" s="5" t="s">
         <v>89</v>
       </c>
-      <c r="AC1" s="5" t="s">
+      <c r="AD1" s="5" t="s">
         <v>103</v>
       </c>
-      <c r="AD1" s="5" t="s">
+      <c r="AE1" s="5" t="s">
         <v>88</v>
       </c>
-      <c r="AE1" s="5" t="s">
+      <c r="AF1" s="5" t="s">
         <v>104</v>
       </c>
-      <c r="AF1" s="5" t="s">
+      <c r="AG1" s="5" t="s">
         <v>140</v>
       </c>
-      <c r="AG1" s="5" t="s">
+      <c r="AH1" s="5" t="s">
         <v>141</v>
       </c>
-      <c r="AH1" s="5" t="s">
+      <c r="AI1" s="5" t="s">
         <v>142</v>
       </c>
-      <c r="AI1" s="5" t="s">
+      <c r="AJ1" s="5" t="s">
         <v>143</v>
       </c>
-      <c r="AJ1" s="5" t="s">
+      <c r="AK1" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="AK1" s="5" t="s">
+      <c r="AL1" s="5" t="s">
         <v>92</v>
       </c>
-      <c r="AL1" s="5" t="s">
+      <c r="AM1" s="5" t="s">
         <v>105</v>
       </c>
-      <c r="AM1" s="5" t="s">
+      <c r="AN1" s="5" t="s">
         <v>106</v>
       </c>
-      <c r="AN1" s="5" t="s">
+      <c r="AO1" s="5" t="s">
         <v>107</v>
       </c>
-      <c r="AO1" s="5" t="s">
+      <c r="AP1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="AP1" s="5" t="s">
+      <c r="AQ1" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="AQ1" s="5" t="s">
+      <c r="AR1" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="AR1" s="5" t="s">
+      <c r="AS1" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="AS1" s="20" t="s">
+      <c r="AT1" s="20" t="s">
         <v>15</v>
       </c>
-      <c r="AT1" s="25" t="s">
+      <c r="AU1" s="25" t="s">
         <v>108</v>
       </c>
-      <c r="AU1" s="5" t="s">
+      <c r="AV1" s="5" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="2" spans="1:47" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
+    <row r="2" spans="1:48" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
   </sheetData>
-  <autoFilter ref="A1:AU1" xr:uid="{00000000-0009-0000-0000-000006000000}"/>
+  <autoFilter ref="A1:AV1" xr:uid="{00000000-0009-0000-0000-000006000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
   <headerFooter>
@@ -9642,19 +9646,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance">
-  <documentManagement>
-    <Unity_Description xmlns="D75E00DB-06CE-4005-B397-8C0860A4229B" xsi:nil="true"/>
-    <Unity_Tag xmlns="D75E00DB-06CE-4005-B397-8C0860A4229B" xsi:nil="true"/>
-    <Capabilities xmlns="d75e00db-06ce-4005-b397-8c0860a4229b" xsi:nil="true"/>
-    <SipLabel xmlns="372b77af-8063-48a8-888c-73c0edf01dea">
-      <Value>2</Value>
-    </SipLabel>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Custom Document" ma:contentTypeID="0x010100E6322E8F405D4D9EA89D8C83B7E1048B001BB96E1BE0ACBB41BF00782ED0412411" ma:contentTypeVersion="3" ma:contentTypeDescription="Custom Document" ma:contentTypeScope="" ma:versionID="3c14126572fa3c0d4c677ac1f3ba4426">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="D75E00DB-06CE-4005-B397-8C0860A4229B" xmlns:ns3="372b77af-8063-48a8-888c-73c0edf01dea" xmlns:ns4="d75e00db-06ce-4005-b397-8c0860a4229b" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="9e89026a025b72b85b9543506e7af3e1" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="D75E00DB-06CE-4005-B397-8C0860A4229B"/>
@@ -9757,6 +9748,19 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance">
+  <documentManagement>
+    <Unity_Description xmlns="D75E00DB-06CE-4005-B397-8C0860A4229B" xsi:nil="true"/>
+    <Unity_Tag xmlns="D75E00DB-06CE-4005-B397-8C0860A4229B" xsi:nil="true"/>
+    <Capabilities xmlns="d75e00db-06ce-4005-b397-8c0860a4229b" xsi:nil="true"/>
+    <SipLabel xmlns="372b77af-8063-48a8-888c-73c0edf01dea">
+      <Value>2</Value>
+    </SipLabel>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -9767,23 +9771,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{268822B0-DCAE-4D2C-8340-AB7554C48D72}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="D75E00DB-06CE-4005-B397-8C0860A4229B"/>
-    <ds:schemaRef ds:uri="372b77af-8063-48a8-888c-73c0edf01dea"/>
-    <ds:schemaRef ds:uri="d75e00db-06ce-4005-b397-8c0860a4229b"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1DE4120D-B400-435F-B862-B3B8683830A5}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -9802,6 +9789,23 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{268822B0-DCAE-4D2C-8340-AB7554C48D72}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="D75E00DB-06CE-4005-B397-8C0860A4229B"/>
+    <ds:schemaRef ds:uri="372b77af-8063-48a8-888c-73c0edf01dea"/>
+    <ds:schemaRef ds:uri="d75e00db-06ce-4005-b397-8c0860a4229b"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2653FDDC-5C81-4B5A-A42F-7A63208AFFF7}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
Changed current resource to proposed resource in various files and comments
</commit_message>
<xml_diff>
--- a/GenBOE/GenBOE.Web/Templates/Export/WorkspaceDataMST.xlsx
+++ b/GenBOE/GenBOE.Web/Templates/Export/WorkspaceDataMST.xlsx
@@ -5,12 +5,12 @@
   <workbookPr showPivotChartFilter="1" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ranzalon\Source\repos\IES\GenBOE\GenBOE.Web\Templates\Export\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\e426263\source\repos\IES\GenBOE\GenBOE.Web\Templates\Export\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BAFB3397-7F53-4909-8E41-C9FA967C96DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{52C423C7-FD8C-4A48-9716-6198D06808E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" firstSheet="5" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-4290" yWindow="-20820" windowWidth="28800" windowHeight="15345" firstSheet="6" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="BOE3 Pivot" sheetId="19" state="hidden" r:id="rId1"/>
@@ -57,9 +57,9 @@
   </definedNames>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="9" r:id="rId22"/>
-    <pivotCache cacheId="10" r:id="rId23"/>
-    <pivotCache cacheId="11" r:id="rId24"/>
+    <pivotCache cacheId="0" r:id="rId22"/>
+    <pivotCache cacheId="1" r:id="rId23"/>
+    <pivotCache cacheId="2" r:id="rId24"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -324,7 +324,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="921" uniqueCount="156">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="921" uniqueCount="157">
   <si>
     <t>Start Date</t>
   </si>
@@ -792,6 +792,9 @@
   </si>
   <si>
     <t>Task Author</t>
+  </si>
+  <si>
+    <t>Proposed Resource</t>
   </si>
 </sst>
 </file>
@@ -4396,7 +4399,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0000-000000000000}" name="PivotTable7" cacheId="9" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="3" minRefreshableVersion="3" showCalcMbrs="0" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="3" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0000-000000000000}" name="PivotTable7" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="3" minRefreshableVersion="3" showCalcMbrs="0" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="3" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
   <location ref="A3:N33" firstHeaderRow="1" firstDataRow="1" firstDataCol="14"/>
   <pivotFields count="14">
     <pivotField axis="axisRow" compact="0" outline="0" showAll="0" insertBlankRow="1" defaultSubtotal="0">
@@ -4745,7 +4748,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0200-000000000000}" name="PivotTable9" cacheId="10" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="3" minRefreshableVersion="3" showCalcMbrs="0" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="3" indent="0" compact="0" compactData="0" multipleFieldFilters="0" rowHeaderCaption="Type">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0200-000000000000}" name="PivotTable9" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="3" minRefreshableVersion="3" showCalcMbrs="0" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="3" indent="0" compact="0" compactData="0" multipleFieldFilters="0" rowHeaderCaption="Type">
   <location ref="A3:H11" firstHeaderRow="1" firstDataRow="1" firstDataCol="8"/>
   <pivotFields count="19">
     <pivotField axis="axisRow" compact="0" outline="0" showAll="0" defaultSubtotal="0">
@@ -4954,7 +4957,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0300-000000000000}" name="PivotTable4" cacheId="11" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" missingCaption="_" updatedVersion="3" minRefreshableVersion="3" showCalcMbrs="0" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="3" indent="0" compact="0" compactData="0" multipleFieldFilters="0" rowHeaderCaption="BOE ID">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0300-000000000000}" name="PivotTable4" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" missingCaption="_" updatedVersion="3" minRefreshableVersion="3" showCalcMbrs="0" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="3" indent="0" compact="0" compactData="0" multipleFieldFilters="0" rowHeaderCaption="BOE ID">
   <location ref="A3:T33" firstHeaderRow="1" firstDataRow="1" firstDataCol="20"/>
   <pivotFields count="20">
     <pivotField axis="axisRow" compact="0" outline="0" showAll="0" insertBlankRow="1" defaultSubtotal="0">
@@ -6363,7 +6366,7 @@
     <col min="5" max="5" width="13.5703125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="14.5703125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="15.85546875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="20.85546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="22.5703125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="19.7109375" style="61" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="18.140625" style="34" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="12.42578125" bestFit="1" customWidth="1"/>
@@ -6395,7 +6398,7 @@
         <v>41</v>
       </c>
       <c r="H1" s="5" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="I1" s="60" t="s">
         <v>146</v>
@@ -9646,6 +9649,19 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance">
+  <documentManagement>
+    <Unity_Description xmlns="D75E00DB-06CE-4005-B397-8C0860A4229B" xsi:nil="true"/>
+    <Unity_Tag xmlns="D75E00DB-06CE-4005-B397-8C0860A4229B" xsi:nil="true"/>
+    <Capabilities xmlns="d75e00db-06ce-4005-b397-8c0860a4229b" xsi:nil="true"/>
+    <SipLabel xmlns="372b77af-8063-48a8-888c-73c0edf01dea">
+      <Value>2</Value>
+    </SipLabel>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Custom Document" ma:contentTypeID="0x010100E6322E8F405D4D9EA89D8C83B7E1048B001BB96E1BE0ACBB41BF00782ED0412411" ma:contentTypeVersion="3" ma:contentTypeDescription="Custom Document" ma:contentTypeScope="" ma:versionID="3c14126572fa3c0d4c677ac1f3ba4426">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="D75E00DB-06CE-4005-B397-8C0860A4229B" xmlns:ns3="372b77af-8063-48a8-888c-73c0edf01dea" xmlns:ns4="d75e00db-06ce-4005-b397-8c0860a4229b" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="9e89026a025b72b85b9543506e7af3e1" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="D75E00DB-06CE-4005-B397-8C0860A4229B"/>
@@ -9748,19 +9764,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance">
-  <documentManagement>
-    <Unity_Description xmlns="D75E00DB-06CE-4005-B397-8C0860A4229B" xsi:nil="true"/>
-    <Unity_Tag xmlns="D75E00DB-06CE-4005-B397-8C0860A4229B" xsi:nil="true"/>
-    <Capabilities xmlns="d75e00db-06ce-4005-b397-8c0860a4229b" xsi:nil="true"/>
-    <SipLabel xmlns="372b77af-8063-48a8-888c-73c0edf01dea">
-      <Value>2</Value>
-    </SipLabel>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -9771,6 +9774,23 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{268822B0-DCAE-4D2C-8340-AB7554C48D72}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="D75E00DB-06CE-4005-B397-8C0860A4229B"/>
+    <ds:schemaRef ds:uri="372b77af-8063-48a8-888c-73c0edf01dea"/>
+    <ds:schemaRef ds:uri="d75e00db-06ce-4005-b397-8c0860a4229b"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1DE4120D-B400-435F-B862-B3B8683830A5}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -9789,23 +9809,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{268822B0-DCAE-4D2C-8340-AB7554C48D72}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="D75E00DB-06CE-4005-B397-8C0860A4229B"/>
-    <ds:schemaRef ds:uri="372b77af-8063-48a8-888c-73c0edf01dea"/>
-    <ds:schemaRef ds:uri="d75e00db-06ce-4005-b397-8c0860a4229b"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2653FDDC-5C81-4B5A-A42F-7A63208AFFF7}">
   <ds:schemaRefs>

</xml_diff>